<commit_message>
veri: iddaa guncellendi (17.10.2026 12:49)
</commit_message>
<xml_diff>
--- a/iddaa/gunluk/gunlukmaclar.xlsx
+++ b/iddaa/gunluk/gunlukmaclar.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD15"/>
+  <dimension ref="A1:BD14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -457,7 +457,7 @@
     <col width="12" customWidth="1" min="27" max="27"/>
     <col width="8" customWidth="1" min="28" max="28"/>
     <col width="8" customWidth="1" min="29" max="29"/>
-    <col width="6" customWidth="1" min="30" max="30"/>
+    <col width="7" customWidth="1" min="30" max="30"/>
     <col width="6" customWidth="1" min="31" max="31"/>
     <col width="6" customWidth="1" min="32" max="32"/>
     <col width="8" customWidth="1" min="33" max="33"/>
@@ -771,69 +771,69 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Le Mans</t>
+          <t>Amed SK</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Konyaspor</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>16.10.2026</t>
+          <t>17.10.2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>Trendyol Süper Lig</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3211162</t>
+          <t>3219266</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2.83</t>
+          <t>1.89</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>3.36</t>
+          <t>3.28</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2.29</t>
+          <t>3.90</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1.47</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>1.67</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>1.37</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>3.11</t>
+          <t>2.46</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -843,466 +843,458 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2.59</t>
+          <t>4.51</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>12.05</t>
+          <t>8.40</t>
         </is>
       </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>4.15</t>
+          <t>2.93</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2.19</t>
+          <t>1.56</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>1.68</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2.53</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>1.26</t>
-        </is>
-      </c>
+          <t>3.26</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>4.52</t>
+          <t>6.75</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>3.46</t>
+          <t>4.56</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>1.13</t>
+          <t>1.67</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>5.17</t>
+          <t>3.22</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>4.38</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>5.16</t>
         </is>
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>3.99</t>
+          <t>9.27</t>
         </is>
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
-          <t>3.28</t>
+          <t>2.51</t>
         </is>
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>1.37</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="AL2" t="inlineStr">
         <is>
-          <t>1.39</t>
+          <t>1.23</t>
         </is>
       </c>
       <c r="AM2" t="inlineStr">
         <is>
-          <t>2.17</t>
+          <t>2.66</t>
         </is>
       </c>
       <c r="AN2" t="inlineStr">
         <is>
-          <t>4.24</t>
+          <t>2.79</t>
         </is>
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>12.50</t>
+          <t>13.90</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
         <is>
-          <t>24.50</t>
+          <t>34.70</t>
         </is>
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>6.67</t>
+          <t>4.64</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
         <is>
-          <t>5.17</t>
+          <t>4.67</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr">
         <is>
-          <t>5.63</t>
+          <t>8.29</t>
         </is>
       </c>
       <c r="AT2" t="inlineStr">
         <is>
-          <t>28.00</t>
+          <t>26.20</t>
         </is>
       </c>
       <c r="AU2" t="inlineStr">
         <is>
-          <t>12.25</t>
+          <t>15.10</t>
         </is>
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>6.71</t>
         </is>
       </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>1.86</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="AY2" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>3.88</t>
         </is>
       </c>
       <c r="AZ2" t="inlineStr">
         <is>
-          <t>9.14</t>
+          <t>17.50</t>
         </is>
       </c>
       <c r="BA2" t="inlineStr">
         <is>
-          <t>2.05</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="BB2" t="inlineStr">
         <is>
-          <t>4.98</t>
+          <t>4.12</t>
         </is>
       </c>
       <c r="BC2" t="inlineStr">
         <is>
-          <t>1.79</t>
+          <t>3.45</t>
         </is>
       </c>
       <c r="BD2" t="inlineStr">
         <is>
-          <t>3.78</t>
+          <t>9.63</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Gençlerbirliği</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Galatasaray</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>16.10.2026</t>
+          <t>17.10.2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Trendyol Süper Lig</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3211087</t>
+          <t>3219152</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2.09</t>
+          <t>6.42</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>3.37</t>
+          <t>5.08</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2.42</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1.22</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>1.33</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>1.29</t>
-        </is>
-      </c>
+          <t>1.26</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2.72</t>
+          <t>5.85</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2.55</t>
+          <t>2.54</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>3.03</t>
+          <t>1.60</t>
         </is>
       </c>
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>6.07</t>
+          <t>5.41</t>
         </is>
       </c>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2.60</t>
+          <t>2.62</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.70</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>1.99</t>
+          <t>2.12</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>3.24</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>3.02</t>
+          <t>3.53</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>3.62</t>
+          <t>14.75</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>4.20</t>
+          <t>7.28</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>4.70</t>
+          <t>3.73</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>4.62</t>
+          <t>1.92</t>
         </is>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>4.02</t>
+          <t>3.95</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="AL3" t="inlineStr">
         <is>
-          <t>1.59</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="AM3" t="inlineStr">
         <is>
-          <t>1.83</t>
+          <t>1.87</t>
         </is>
       </c>
       <c r="AN3" t="inlineStr">
         <is>
-          <t>3.40</t>
+          <t>11.00</t>
         </is>
       </c>
       <c r="AO3" t="inlineStr">
         <is>
-          <t>12.10</t>
+          <t>20.10</t>
         </is>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
-          <t>24.25</t>
+          <t>19.35</t>
         </is>
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>6.28</t>
+          <t>14.35</t>
         </is>
       </c>
       <c r="AR3" t="inlineStr">
         <is>
-          <t>6.33</t>
+          <t>8.04</t>
         </is>
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>6.99</t>
+          <t>4.24</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr">
         <is>
-          <t>22.10</t>
+          <t>34.70</t>
         </is>
       </c>
       <c r="AU3" t="inlineStr">
         <is>
-          <t>12.30</t>
+          <t>17.90</t>
         </is>
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>4.01</t>
+          <t>1.87</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>6.04</t>
+          <t>5.29</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr">
         <is>
-          <t>2.09</t>
+          <t>1.99</t>
         </is>
       </c>
       <c r="AY3" t="inlineStr">
         <is>
-          <t>2.53</t>
+          <t>2.62</t>
         </is>
       </c>
       <c r="AZ3" t="inlineStr">
         <is>
-          <t>5.43</t>
+          <t>6.25</t>
         </is>
       </c>
       <c r="BA3" t="inlineStr">
         <is>
-          <t>1.76</t>
+          <t>3.29</t>
         </is>
       </c>
       <c r="BB3" t="inlineStr">
         <is>
-          <t>3.00</t>
+          <t>9.72</t>
         </is>
       </c>
       <c r="BC3" t="inlineStr">
         <is>
-          <t>1.88</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="BD3" t="inlineStr">
         <is>
-          <t>3.44</t>
+          <t>2.12</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Çorum FK</t>
+          <t>Erzurumspor FK</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ç. Rizespor</t>
+          <t>Eyüpspor</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>16.10.2026</t>
+          <t>17.10.2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1312,899 +1304,791 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3218413</t>
+          <t>3216437</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2.06</t>
+          <t>1.51</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>3.47</t>
+          <t>3.96</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>3.11</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>1.34</t>
-        </is>
-      </c>
+          <t>6.43</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>1.59</t>
+          <t>1.60</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>1.76</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2.58</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2.36</t>
+          <t>2.29</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>6.68</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>12.65</t>
+          <t>8.76</t>
         </is>
       </c>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>4.42</t>
+          <t>2.93</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2.02</t>
+          <t>1.58</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>3.26</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>6.66</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>5.45</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
           <t>1.46</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>1.55</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>2.49</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>1.07</t>
-        </is>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>4.21</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>3.45</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>1.13</t>
-        </is>
-      </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>3.47</t>
+          <t>2.29</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>3.95</t>
+          <t>3.27</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr"/>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>4.86</t>
+          <t>6.86</t>
         </is>
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>6.20</t>
+          <t>18.15</t>
         </is>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>3.33</t>
+          <t>2.62</t>
         </is>
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.24</t>
         </is>
       </c>
       <c r="AL4" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="AM4" t="inlineStr">
         <is>
-          <t>2.35</t>
+          <t>2.60</t>
         </is>
       </c>
       <c r="AN4" t="inlineStr">
         <is>
-          <t>2.86</t>
+          <t>2.08</t>
         </is>
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>12.65</t>
+          <t>17.80</t>
         </is>
       </c>
       <c r="AP4" t="inlineStr">
         <is>
-          <t>30.00</t>
+          <t>34.70</t>
         </is>
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>5.19</t>
+          <t>3.97</t>
         </is>
       </c>
       <c r="AR4" t="inlineStr">
         <is>
-          <t>5.41</t>
+          <t>5.37</t>
         </is>
       </c>
       <c r="AS4" t="inlineStr">
         <is>
-          <t>7.26</t>
+          <t>12.80</t>
         </is>
       </c>
       <c r="AT4" t="inlineStr">
         <is>
-          <t>22.75</t>
+          <t>26.20</t>
         </is>
       </c>
       <c r="AU4" t="inlineStr">
         <is>
-          <t>13.20</t>
+          <t>20.50</t>
         </is>
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>4.83</t>
+          <t>11.70</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>4.41</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>2.07</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="AY4" t="inlineStr">
         <is>
-          <t>3.16</t>
+          <t>3.88</t>
         </is>
       </c>
       <c r="AZ4" t="inlineStr">
         <is>
-          <t>9.04</t>
+          <t>17.50</t>
         </is>
       </c>
       <c r="BA4" t="inlineStr">
         <is>
-          <t>1.87</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="BB4" t="inlineStr">
         <is>
-          <t>3.56</t>
+          <t>2.92</t>
         </is>
       </c>
       <c r="BC4" t="inlineStr">
         <is>
-          <t>2.20</t>
+          <t>5.14</t>
         </is>
       </c>
       <c r="BD4" t="inlineStr">
         <is>
-          <t>5.31</t>
+          <t>17.00</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Deportivo</t>
+          <t>Sivasspor</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Sarıyer</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>16.10.2026</t>
+          <t>17.10.2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Trendyol 1. Lig</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3216309</t>
+          <t>3216202</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2.04</t>
+          <t>2.06</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>3.26</t>
+          <t>2.91</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>3.34</t>
+          <t>2.55</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1.30</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>1.67</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2.63</t>
+          <t>2.65</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2.20</t>
+          <t>1.90</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>3.96</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>9.36</t>
-        </is>
-      </c>
+          <t>3.16</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>3.44</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>1.36</t>
-        </is>
-      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>1.68</t>
+          <t>1.79</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>1.72</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>1.19</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>2.96</t>
-        </is>
-      </c>
+          <t>1.88</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>5.94</t>
-        </is>
-      </c>
+      <c r="AA5" t="inlineStr"/>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>4.17</t>
+          <t>4.05</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>1.76</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>3.39</t>
+          <t>3.94</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>3.54</t>
+          <t>3.55</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>4.64</t>
-        </is>
-      </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>7.12</t>
-        </is>
-      </c>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>2.86</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>1.45</t>
+          <t>1.95</t>
         </is>
       </c>
       <c r="AL5" t="inlineStr">
         <is>
-          <t>1.28</t>
+          <t>1.23</t>
         </is>
       </c>
       <c r="AM5" t="inlineStr">
         <is>
-          <t>2.53</t>
-        </is>
-      </c>
-      <c r="AN5" t="inlineStr">
-        <is>
-          <t>3.08</t>
-        </is>
-      </c>
-      <c r="AO5" t="inlineStr">
-        <is>
-          <t>13.35</t>
-        </is>
-      </c>
-      <c r="AP5" t="inlineStr">
-        <is>
-          <t>35.20</t>
-        </is>
-      </c>
-      <c r="AQ5" t="inlineStr">
-        <is>
-          <t>5.07</t>
-        </is>
-      </c>
-      <c r="AR5" t="inlineStr">
-        <is>
-          <t>4.87</t>
-        </is>
-      </c>
-      <c r="AS5" t="inlineStr">
-        <is>
-          <t>7.51</t>
-        </is>
-      </c>
-      <c r="AT5" t="inlineStr">
-        <is>
-          <t>26.20</t>
-        </is>
-      </c>
-      <c r="AU5" t="inlineStr">
-        <is>
-          <t>14.15</t>
-        </is>
-      </c>
-      <c r="AV5" t="inlineStr">
-        <is>
-          <t>5.61</t>
-        </is>
-      </c>
-      <c r="AW5" t="inlineStr">
-        <is>
-          <t>3.19</t>
-        </is>
-      </c>
-      <c r="AX5" t="inlineStr">
-        <is>
-          <t>1.79</t>
-        </is>
-      </c>
-      <c r="AY5" t="inlineStr">
-        <is>
-          <t>3.59</t>
-        </is>
-      </c>
-      <c r="AZ5" t="inlineStr">
-        <is>
-          <t>14.50</t>
-        </is>
-      </c>
+          <t>2.46</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="inlineStr"/>
       <c r="BA5" t="inlineStr">
         <is>
-          <t>2.06</t>
-        </is>
-      </c>
-      <c r="BB5" t="inlineStr">
-        <is>
-          <t>4.06</t>
-        </is>
-      </c>
+          <t>2.19</t>
+        </is>
+      </c>
+      <c r="BB5" t="inlineStr"/>
       <c r="BC5" t="inlineStr">
         <is>
-          <t>2.91</t>
-        </is>
-      </c>
-      <c r="BD5" t="inlineStr">
-        <is>
-          <t>7.40</t>
-        </is>
-      </c>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="BD5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>E. Frankfurt</t>
+          <t>Brentford</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Köln</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>16.10.2026</t>
+          <t>17.10.2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bundesliga</t>
+          <t>Premier Lig</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3217571</t>
+          <t>3219826</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1.65</t>
+          <t>2.32</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>3.76</t>
+          <t>3.45</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>3.18</t>
+          <t>2.65</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.39</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.56</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2.04</t>
+          <t>2.58</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2.47</t>
+          <t>2.20</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>3.42</t>
+          <t>2.89</t>
         </is>
       </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>7.00</t>
+          <t>4.96</t>
         </is>
       </c>
       <c r="U6" t="inlineStr"/>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2.94</t>
+          <t>2.20</t>
         </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.43</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>1.62</t>
+          <t>2.05</t>
         </is>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>1.30</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>2.76</t>
+          <t>3.82</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>2.85</t>
+          <t>3.12</t>
         </is>
       </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>2.57</t>
+          <t>3.99</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>3.91</t>
+          <t>4.24</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>5.25</t>
+          <t>4.32</t>
         </is>
       </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>6.09</t>
+          <t>4.60</t>
         </is>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>4.20</t>
-        </is>
-      </c>
-      <c r="AK6" t="inlineStr"/>
+          <t>3.35</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
       <c r="AL6" t="inlineStr">
         <is>
+          <t>1.66</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>2.20</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>3.48</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>12.25</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>25.70</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>6.05</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>5.76</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>6.71</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>23.60</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>12.45</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>4.08</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>4.80</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>1.93</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>2.72</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>7.14</t>
+        </is>
+      </c>
+      <c r="BA6" t="inlineStr">
+        <is>
           <t>1.88</t>
         </is>
       </c>
-      <c r="AM6" t="inlineStr">
-        <is>
-          <t>1.91</t>
-        </is>
-      </c>
-      <c r="AN6" t="inlineStr">
-        <is>
-          <t>2.61</t>
-        </is>
-      </c>
-      <c r="AO6" t="inlineStr">
-        <is>
-          <t>12.70</t>
-        </is>
-      </c>
-      <c r="AP6" t="inlineStr">
-        <is>
-          <t>28.20</t>
-        </is>
-      </c>
-      <c r="AQ6" t="inlineStr">
-        <is>
-          <t>5.41</t>
-        </is>
-      </c>
-      <c r="AR6" t="inlineStr">
-        <is>
-          <t>7.15</t>
-        </is>
-      </c>
-      <c r="AS6" t="inlineStr">
-        <is>
-          <t>8.76</t>
-        </is>
-      </c>
-      <c r="AT6" t="inlineStr">
-        <is>
-          <t>18.55</t>
-        </is>
-      </c>
-      <c r="AU6" t="inlineStr">
-        <is>
-          <t>13.55</t>
-        </is>
-      </c>
-      <c r="AV6" t="inlineStr">
-        <is>
-          <t>5.36</t>
-        </is>
-      </c>
-      <c r="AW6" t="inlineStr">
-        <is>
-          <t>7.32</t>
-        </is>
-      </c>
-      <c r="AX6" t="inlineStr">
-        <is>
-          <t>2.42</t>
-        </is>
-      </c>
-      <c r="AY6" t="inlineStr">
-        <is>
-          <t>2.59</t>
-        </is>
-      </c>
-      <c r="AZ6" t="inlineStr">
-        <is>
-          <t>4.64</t>
-        </is>
-      </c>
-      <c r="BA6" t="inlineStr">
-        <is>
-          <t>1.53</t>
-        </is>
-      </c>
       <c r="BB6" t="inlineStr">
         <is>
-          <t>2.41</t>
+          <t>3.65</t>
         </is>
       </c>
       <c r="BC6" t="inlineStr">
         <is>
-          <t>1.82</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="BD6" t="inlineStr">
         <is>
-          <t>4.14</t>
+          <t>3.97</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Heerenveen</t>
+          <t>Fenerbahçe</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Excelsior</t>
+          <t>Alanyaspor</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>16.10.2026</t>
+          <t>17.10.2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Eredivisie</t>
+          <t>Trendyol Süper Lig</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3210976</t>
+          <t>3219012</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1.40</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>4.10</t>
+          <t>5.57</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>4.36</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>1.06</t>
-        </is>
-      </c>
+          <t>8.53</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.23</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>1.58</t>
+          <t>1.88</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.70</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2.49</t>
+          <t>2.81</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>4.45</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>5.85</t>
+          <t>4.91</t>
         </is>
       </c>
       <c r="U7" t="inlineStr"/>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2.63</t>
+          <t>2.31</t>
         </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.33</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.66</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>2.20</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>2.96</t>
+          <t>3.44</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>3.05</t>
+          <t>4.02</t>
         </is>
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>1.07</t>
         </is>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>2.09</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>3.68</t>
+          <t>3.56</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>6.15</t>
-        </is>
-      </c>
-      <c r="AI7" t="inlineStr">
-        <is>
-          <t>9.41</t>
-        </is>
-      </c>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>3.94</t>
+          <t>3.68</t>
         </is>
       </c>
       <c r="AK7" t="inlineStr">
@@ -2214,888 +2098,880 @@
       </c>
       <c r="AL7" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>1.71</t>
         </is>
       </c>
       <c r="AM7" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>2.11</t>
         </is>
       </c>
       <c r="AN7" t="inlineStr">
         <is>
-          <t>1.99</t>
+          <t>1.52</t>
         </is>
       </c>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>14.25</t>
+          <t>20.45</t>
         </is>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>35.00</t>
+          <t>34.50</t>
         </is>
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>4.58</t>
+          <t>3.87</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>7.16</t>
+          <t>8.17</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>10.85</t>
+          <t>17.95</t>
         </is>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t>18.75</t>
+          <t>20.80</t>
         </is>
       </c>
       <c r="AU7" t="inlineStr">
         <is>
-          <t>15.60</t>
+          <t>23.40</t>
         </is>
       </c>
       <c r="AV7" t="inlineStr">
         <is>
-          <t>7.37</t>
+          <t>14.90</t>
         </is>
       </c>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>6.00</t>
+          <t>4.96</t>
         </is>
       </c>
       <c r="AX7" t="inlineStr">
         <is>
-          <t>2.09</t>
+          <t>1.95</t>
         </is>
       </c>
       <c r="AY7" t="inlineStr">
         <is>
-          <t>2.54</t>
+          <t>2.69</t>
         </is>
       </c>
       <c r="AZ7" t="inlineStr">
         <is>
-          <t>5.46</t>
+          <t>6.82</t>
         </is>
       </c>
       <c r="BA7" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="BB7" t="inlineStr">
         <is>
-          <t>2.10</t>
+          <t>2.03</t>
         </is>
       </c>
       <c r="BC7" t="inlineStr">
         <is>
-          <t>2.40</t>
+          <t>4.49</t>
         </is>
       </c>
       <c r="BD7" t="inlineStr">
         <is>
-          <t>6.12</t>
+          <t>13.85</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Annecy </t>
+          <t>Fulham</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Hull City</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>16.10.2026</t>
+          <t>17.10.2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Ligue 2</t>
+          <t>Premier Lig</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>3210967</t>
+          <t>3216588</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2.65</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2.90</t>
+          <t>3.63</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2.15</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>1.23</t>
-        </is>
-      </c>
+          <t>4.62</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>3.29</t>
+          <t>2.11</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>1.94</t>
+          <t>2.38</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2.78</t>
+          <t>5.10</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>8.73</t>
+          <t>11.30</t>
         </is>
       </c>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>3.07</t>
+          <t>3.70</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>1.17</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>2.05</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>1.79</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>3.15</t>
+          <t>2.53</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>6.48</t>
+          <t>4.81</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>4.28</t>
+          <t>4.03</t>
         </is>
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>1.07</t>
         </is>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>5.70</t>
+          <t>2.29</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>4.17</t>
+          <t>3.33</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>3.75</t>
+          <t>6.07</t>
         </is>
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>4.27</t>
+          <t>11.50</t>
         </is>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>2.56</t>
+          <t>2.98</t>
         </is>
       </c>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="AL8" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="AM8" t="inlineStr">
         <is>
-          <t>2.63</t>
+          <t>2.26</t>
         </is>
       </c>
       <c r="AN8" t="inlineStr">
         <is>
-          <t>4.45</t>
+          <t>2.08</t>
         </is>
       </c>
       <c r="AO8" t="inlineStr">
         <is>
-          <t>13.20</t>
+          <t>14.55</t>
         </is>
       </c>
       <c r="AP8" t="inlineStr">
         <is>
-          <t>28.50</t>
+          <t>34.50</t>
         </is>
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>6.31</t>
+          <t>4.22</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>4.38</t>
+          <t>5.54</t>
         </is>
       </c>
       <c r="AS8" t="inlineStr">
         <is>
-          <t>5.40</t>
+          <t>10.30</t>
         </is>
       </c>
       <c r="AT8" t="inlineStr">
         <is>
-          <t>32.50</t>
+          <t>22.10</t>
         </is>
       </c>
       <c r="AU8" t="inlineStr">
         <is>
-          <t>12.90</t>
+          <t>16.30</t>
         </is>
       </c>
       <c r="AV8" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>8.13</t>
         </is>
       </c>
       <c r="AW8" t="inlineStr">
         <is>
-          <t>3.01</t>
+          <t>3.87</t>
         </is>
       </c>
       <c r="AX8" t="inlineStr">
         <is>
-          <t>1.78</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="AY8" t="inlineStr">
         <is>
-          <t>3.77</t>
+          <t>3.37</t>
         </is>
       </c>
       <c r="AZ8" t="inlineStr">
         <is>
-          <t>16.30</t>
+          <t>11.05</t>
         </is>
       </c>
       <c r="BA8" t="inlineStr">
         <is>
-          <t>2.47</t>
+          <t>1.68</t>
         </is>
       </c>
       <c r="BB8" t="inlineStr">
         <is>
-          <t>6.39</t>
+          <t>2.95</t>
         </is>
       </c>
       <c r="BC8" t="inlineStr">
         <is>
-          <t>2.14</t>
+          <t>3.27</t>
         </is>
       </c>
       <c r="BD8" t="inlineStr">
         <is>
-          <t>5.07</t>
+          <t>9.96</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Burnley</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Wolverhampton</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16.10.2026</t>
+          <t>17.10.2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Championship</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>3211144</t>
+          <t>3219061</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2.77</t>
+          <t>4.29</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>3.67</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>1.97</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.07</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>3.36</t>
+          <t>4.61</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2.05</t>
+          <t>2.38</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2.56</t>
+          <t>2.20</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>10.55</t>
+          <t>11.80</t>
         </is>
       </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>3.58</t>
+          <t>4.11</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>2.12</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.70</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>1.24</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>2.68</t>
+          <t>2.61</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>5.19</t>
+          <t>4.71</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>3.83</t>
+          <t>3.76</t>
         </is>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>5.85</t>
+          <t>9.61</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>4.39</t>
+          <t>5.73</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>3.71</t>
+          <t>3.44</t>
         </is>
       </c>
       <c r="AI9" t="inlineStr">
         <is>
-          <t>3.68</t>
+          <t>2.47</t>
         </is>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>2.82</t>
+          <t>3.24</t>
         </is>
       </c>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>1.22</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="AL9" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="AM9" t="inlineStr">
         <is>
-          <t>2.37</t>
+          <t>2.39</t>
         </is>
       </c>
       <c r="AN9" t="inlineStr">
         <is>
-          <t>4.64</t>
+          <t>7.05</t>
         </is>
       </c>
       <c r="AO9" t="inlineStr">
         <is>
-          <t>13.45</t>
+          <t>14.90</t>
         </is>
       </c>
       <c r="AP9" t="inlineStr">
         <is>
-          <t>24.95</t>
+          <t>22.10</t>
         </is>
       </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>6.73</t>
+          <t>9.41</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>4.94</t>
+          <t>5.46</t>
         </is>
       </c>
       <c r="AS9" t="inlineStr">
         <is>
-          <t>5.21</t>
+          <t>4.46</t>
         </is>
       </c>
       <c r="AT9" t="inlineStr">
         <is>
-          <t>31.00</t>
+          <t>34.50</t>
         </is>
       </c>
       <c r="AU9" t="inlineStr">
         <is>
-          <t>12.95</t>
+          <t>13.55</t>
         </is>
       </c>
       <c r="AV9" t="inlineStr">
         <is>
-          <t>3.12</t>
+          <t>2.23</t>
         </is>
       </c>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>3.53</t>
+          <t>4.09</t>
         </is>
       </c>
       <c r="AX9" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>2.03</t>
         </is>
       </c>
       <c r="AY9" t="inlineStr">
         <is>
-          <t>3.31</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="AZ9" t="inlineStr">
         <is>
-          <t>11.90</t>
+          <t>10.00</t>
         </is>
       </c>
       <c r="BA9" t="inlineStr">
         <is>
-          <t>2.34</t>
+          <t>3.05</t>
         </is>
       </c>
       <c r="BB9" t="inlineStr">
         <is>
-          <t>5.85</t>
+          <t>8.19</t>
         </is>
       </c>
       <c r="BC9" t="inlineStr">
         <is>
-          <t>1.86</t>
+          <t>1.51</t>
         </is>
       </c>
       <c r="BD9" t="inlineStr">
         <is>
-          <t>4.05</t>
+          <t>3.03</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Boulogne</t>
+          <t>Inter</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>16.10.2026</t>
+          <t>17.10.2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Ligue 2</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>3211258</t>
+          <t>3217034</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2.46</t>
+          <t>4.89</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2.74</t>
+          <t>3.80</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2.41</t>
+          <t>1.39</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>1.59</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>1.16</t>
-        </is>
-      </c>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
-          <t>3.24</t>
+          <t>4.96</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>2.31</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>3.19</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>6.82</t>
+          <t>12.85</t>
         </is>
       </c>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2.49</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr">
-        <is>
-          <t>1.30</t>
-        </is>
-      </c>
+          <t>4.30</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr"/>
       <c r="V10" t="inlineStr">
         <is>
-          <t>1.40</t>
+          <t>2.06</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>2.15</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
+          <t>1.35</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>2.22</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
           <t>1.07</t>
         </is>
       </c>
-      <c r="Y10" t="inlineStr">
-        <is>
-          <t>4.14</t>
-        </is>
-      </c>
-      <c r="Z10" t="inlineStr"/>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>9.10</t>
+          <t>4.01</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>5.12</t>
+          <t>3.89</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>5.47</t>
+          <t>11.55</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>3.82</t>
+          <t>6.22</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr"/>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>3.79</t>
+          <t>3.65</t>
         </is>
       </c>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>5.35</t>
+          <t>2.32</t>
         </is>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>2.23</t>
+          <t>3.28</t>
         </is>
       </c>
       <c r="AK10" t="inlineStr">
         <is>
-          <t>1.37</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="AL10" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.62</t>
         </is>
       </c>
       <c r="AM10" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>2.26</t>
         </is>
       </c>
       <c r="AN10" t="inlineStr">
         <is>
-          <t>4.16</t>
+          <t>8.51</t>
         </is>
       </c>
       <c r="AO10" t="inlineStr">
         <is>
-          <t>13.95</t>
+          <t>16.15</t>
         </is>
       </c>
       <c r="AP10" t="inlineStr">
         <is>
-          <t>35.00</t>
+          <t>21.00</t>
         </is>
       </c>
       <c r="AQ10" t="inlineStr">
         <is>
-          <t>5.63</t>
+          <t>11.20</t>
         </is>
       </c>
       <c r="AR10" t="inlineStr">
         <is>
-          <t>3.86</t>
+          <t>6.03</t>
         </is>
       </c>
       <c r="AS10" t="inlineStr">
         <is>
-          <t>5.56</t>
+          <t>4.31</t>
         </is>
       </c>
       <c r="AT10" t="inlineStr">
         <is>
-          <t>35.00</t>
+          <t>34.50</t>
         </is>
       </c>
       <c r="AU10" t="inlineStr">
         <is>
-          <t>13.90</t>
+          <t>14.30</t>
         </is>
       </c>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>4.08</t>
+          <t>1.97</t>
         </is>
       </c>
       <c r="AW10" t="inlineStr">
         <is>
-          <t>2.42</t>
+          <t>4.30</t>
         </is>
       </c>
       <c r="AX10" t="inlineStr">
         <is>
-          <t>1.78</t>
+          <t>1.87</t>
         </is>
       </c>
       <c r="AY10" t="inlineStr">
         <is>
-          <t>4.80</t>
+          <t>2.88</t>
         </is>
       </c>
       <c r="AZ10" t="inlineStr">
         <is>
-          <t>27.50</t>
+          <t>8.35</t>
         </is>
       </c>
       <c r="BA10" t="inlineStr">
         <is>
-          <t>2.70</t>
+          <t>3.06</t>
         </is>
       </c>
       <c r="BB10" t="inlineStr">
         <is>
-          <t>7.30</t>
+          <t>9.05</t>
         </is>
       </c>
       <c r="BC10" t="inlineStr">
         <is>
-          <t>2.67</t>
+          <t>1.58</t>
         </is>
       </c>
       <c r="BD10" t="inlineStr">
         <is>
-          <t>7.18</t>
+          <t>2.61</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Reims</t>
+          <t>Telstar</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dijon</t>
+          <t>Feyenoord</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>16.10.2026</t>
+          <t>17.10.2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -3105,1268 +2981,938 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Ligue 2</t>
+          <t>Eredivisie</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>3211001</t>
+          <t>3218688</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>7.14</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>3.41</t>
+          <t>5.23</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>4.06</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>1.86</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>1.38</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>1.44</t>
-        </is>
-      </c>
+          <t>1.21</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2.04</t>
+          <t>6.49</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2.18</t>
+          <t>2.91</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>4.38</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>11.40</t>
-        </is>
-      </c>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>3.91</t>
-        </is>
-      </c>
-      <c r="U11" t="inlineStr">
-        <is>
-          <t>1.09</t>
-        </is>
-      </c>
+          <t>6.01</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr">
         <is>
-          <t>1.92</t>
+          <t>2.70</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>1.53</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>1.30</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>2.45</t>
-        </is>
-      </c>
-      <c r="Z11" t="inlineStr"/>
+          <t>1.94</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>1.40</t>
+        </is>
+      </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>4.62</t>
+          <t>3.03</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>3.81</t>
+          <t>3.38</t>
         </is>
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>1.09</t>
-        </is>
-      </c>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>2.56</t>
-        </is>
-      </c>
-      <c r="AE11" t="inlineStr">
-        <is>
-          <t>3.49</t>
-        </is>
-      </c>
+          <t>1.12</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr"/>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>5.53</t>
+          <t>3.92</t>
         </is>
       </c>
       <c r="AI11" t="inlineStr">
         <is>
-          <t>9.32</t>
+          <t>1.79</t>
         </is>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>3.05</t>
+          <t>4.32</t>
         </is>
       </c>
       <c r="AK11" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="AL11" t="inlineStr">
         <is>
-          <t>1.37</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="AM11" t="inlineStr">
         <is>
-          <t>2.22</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="AN11" t="inlineStr">
         <is>
-          <t>2.29</t>
+          <t>12.50</t>
         </is>
       </c>
       <c r="AO11" t="inlineStr">
         <is>
-          <t>13.30</t>
+          <t>20.95</t>
         </is>
       </c>
       <c r="AP11" t="inlineStr">
         <is>
-          <t>35.00</t>
+          <t>19.10</t>
         </is>
       </c>
       <c r="AQ11" t="inlineStr">
         <is>
-          <t>4.57</t>
+          <t>16.65</t>
         </is>
       </c>
       <c r="AR11" t="inlineStr">
         <is>
-          <t>5.36</t>
+          <t>8.81</t>
         </is>
       </c>
       <c r="AS11" t="inlineStr">
         <is>
-          <t>9.36</t>
+          <t>4.31</t>
         </is>
       </c>
       <c r="AT11" t="inlineStr">
         <is>
-          <t>22.30</t>
+          <t>34.70</t>
         </is>
       </c>
       <c r="AU11" t="inlineStr">
         <is>
-          <t>14.70</t>
+          <t>18.45</t>
         </is>
       </c>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>6.99</t>
+          <t>1.76</t>
         </is>
       </c>
       <c r="AW11" t="inlineStr">
         <is>
-          <t>3.88</t>
+          <t>6.39</t>
         </is>
       </c>
       <c r="AX11" t="inlineStr">
         <is>
-          <t>1.84</t>
+          <t>2.30</t>
         </is>
       </c>
       <c r="AY11" t="inlineStr">
         <is>
-          <t>3.10</t>
+          <t>2.68</t>
         </is>
       </c>
       <c r="AZ11" t="inlineStr">
         <is>
-          <t>10.10</t>
+          <t>5.37</t>
         </is>
       </c>
       <c r="BA11" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>3.47</t>
         </is>
       </c>
       <c r="BB11" t="inlineStr">
         <is>
-          <t>2.92</t>
+          <t>9.83</t>
         </is>
       </c>
       <c r="BC11" t="inlineStr">
         <is>
-          <t>2.85</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="BD11" t="inlineStr">
         <is>
-          <t>7.98</t>
+          <t>1.93</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Guingamp</t>
+          <t>Padova</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pau</t>
+          <t>Virtus Entella</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16.10.2026</t>
+          <t>17.10.2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Ligue 2</t>
+          <t>Serie B</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>3210717</t>
+          <t>3216305</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1.98</t>
+          <t>2.34</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>3.03</t>
+          <t>2.67</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2.85</t>
+          <t>2.59</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>1.45</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>1.28</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2.54</t>
+          <t>2.97</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>3.43</t>
+          <t>3.23</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>9.98</t>
+          <t>7.27</t>
         </is>
       </c>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>3.47</t>
+          <t>2.71</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>1.76</t>
+          <t>1.47</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>1.65</t>
+          <t>1.98</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.10</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>2.75</t>
+          <t>3.60</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr"/>
       <c r="AA12" t="inlineStr">
         <is>
-          <t>5.42</t>
+          <t>7.78</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>3.92</t>
+          <t>4.65</t>
         </is>
       </c>
       <c r="AC12" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.69</t>
         </is>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
-          <t>3.68</t>
+          <t>4.86</t>
         </is>
       </c>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>3.71</t>
+          <t>3.82</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr"/>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>4.46</t>
+          <t>4.03</t>
         </is>
       </c>
       <c r="AI12" t="inlineStr">
         <is>
-          <t>6.13</t>
+          <t>5.62</t>
         </is>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>2.77</t>
+          <t>2.36</t>
         </is>
       </c>
       <c r="AK12" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.31</t>
         </is>
       </c>
       <c r="AL12" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="AM12" t="inlineStr">
         <is>
-          <t>2.42</t>
+          <t>2.85</t>
         </is>
       </c>
       <c r="AN12" t="inlineStr">
         <is>
-          <t>3.11</t>
+          <t>3.81</t>
         </is>
       </c>
       <c r="AO12" t="inlineStr">
         <is>
-          <t>12.60</t>
+          <t>12.55</t>
         </is>
       </c>
       <c r="AP12" t="inlineStr">
         <is>
-          <t>32.50</t>
+          <t>34.50</t>
         </is>
       </c>
       <c r="AQ12" t="inlineStr">
         <is>
-          <t>5.22</t>
+          <t>5.63</t>
         </is>
       </c>
       <c r="AR12" t="inlineStr">
         <is>
-          <t>4.73</t>
+          <t>3.88</t>
         </is>
       </c>
       <c r="AS12" t="inlineStr">
         <is>
-          <t>6.90</t>
+          <t>6.08</t>
         </is>
       </c>
       <c r="AT12" t="inlineStr">
         <is>
-          <t>26.00</t>
+          <t>32.00</t>
         </is>
       </c>
       <c r="AU12" t="inlineStr">
         <is>
-          <t>13.15</t>
+          <t>12.70</t>
         </is>
       </c>
       <c r="AV12" t="inlineStr">
         <is>
-          <t>4.80</t>
+          <t>4.30</t>
         </is>
       </c>
       <c r="AW12" t="inlineStr">
         <is>
-          <t>3.43</t>
+          <t>2.65</t>
         </is>
       </c>
       <c r="AX12" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="AY12" t="inlineStr">
         <is>
-          <t>3.38</t>
+          <t>4.22</t>
         </is>
       </c>
       <c r="AZ12" t="inlineStr">
         <is>
-          <t>12.60</t>
+          <t>21.10</t>
         </is>
       </c>
       <c r="BA12" t="inlineStr">
         <is>
-          <t>1.88</t>
+          <t>2.39</t>
         </is>
       </c>
       <c r="BB12" t="inlineStr">
         <is>
-          <t>4.12</t>
+          <t>6.10</t>
         </is>
       </c>
       <c r="BC12" t="inlineStr">
         <is>
-          <t>2.42</t>
+          <t>2.59</t>
         </is>
       </c>
       <c r="BD12" t="inlineStr">
         <is>
-          <t>6.19</t>
+          <t>6.87</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Lavallois</t>
+          <t>Sporting Gijon</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Clermont</t>
+          <t>Albacete</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16.10.2026</t>
+          <t>17.10.2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ligue 2</t>
+          <t>LaLiga 2</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3210731</t>
+          <t>3219684</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>1.93</t>
+          <t>1.81</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2.91</t>
+          <t>3.07</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>3.07</t>
+          <t>3.24</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>1.09</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>1.28</t>
+          <t>1.31</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2.53</t>
+          <t>2.35</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>1.95</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>3.71</t>
+          <t>3.78</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>8.55</t>
+          <t>9.59</t>
         </is>
       </c>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>3.04</t>
+          <t>3.32</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>1.70</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>1.81</t>
+          <t>1.67</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>3.19</t>
+          <t>2.84</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr"/>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>6.59</t>
+          <t>5.65</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>4.37</t>
+          <t>4.05</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>1.07</t>
         </is>
       </c>
       <c r="AD13" t="inlineStr">
         <is>
-          <t>3.65</t>
+          <t>3.24</t>
         </is>
       </c>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>3.57</t>
+          <t>3.51</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr"/>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>4.53</t>
+          <t>4.71</t>
         </is>
       </c>
       <c r="AI13" t="inlineStr">
         <is>
-          <t>7.01</t>
+          <t>7.28</t>
         </is>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>2.56</t>
+          <t>2.70</t>
         </is>
       </c>
       <c r="AK13" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.22</t>
         </is>
       </c>
       <c r="AL13" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="AM13" t="inlineStr">
         <is>
-          <t>2.65</t>
+          <t>2.45</t>
         </is>
       </c>
       <c r="AN13" t="inlineStr">
         <is>
-          <t>3.05</t>
+          <t>2.78</t>
         </is>
       </c>
       <c r="AO13" t="inlineStr">
         <is>
-          <t>12.90</t>
+          <t>12.85</t>
         </is>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
-          <t>35.00</t>
+          <t>34.50</t>
         </is>
       </c>
       <c r="AQ13" t="inlineStr">
         <is>
-          <t>4.99</t>
+          <t>4.82</t>
         </is>
       </c>
       <c r="AR13" t="inlineStr">
         <is>
-          <t>4.37</t>
+          <t>4.68</t>
         </is>
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>7.11</t>
+          <t>7.50</t>
         </is>
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>27.00</t>
+          <t>24.70</t>
         </is>
       </c>
       <c r="AU13" t="inlineStr">
         <is>
-          <t>13.60</t>
+          <t>13.65</t>
         </is>
       </c>
       <c r="AV13" t="inlineStr">
         <is>
-          <t>5.29</t>
+          <t>5.53</t>
         </is>
       </c>
       <c r="AW13" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>3.26</t>
         </is>
       </c>
       <c r="AX13" t="inlineStr">
         <is>
-          <t>1.77</t>
+          <t>1.78</t>
         </is>
       </c>
       <c r="AY13" t="inlineStr">
         <is>
-          <t>3.82</t>
+          <t>3.46</t>
         </is>
       </c>
       <c r="AZ13" t="inlineStr">
         <is>
-          <t>16.65</t>
+          <t>13.45</t>
         </is>
       </c>
       <c r="BA13" t="inlineStr">
         <is>
-          <t>1.99</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="BB13" t="inlineStr">
         <is>
-          <t>4.50</t>
+          <t>3.83</t>
         </is>
       </c>
       <c r="BC13" t="inlineStr">
         <is>
-          <t>2.77</t>
+          <t>2.68</t>
         </is>
       </c>
       <c r="BD13" t="inlineStr">
         <is>
-          <t>7.64</t>
+          <t>7.30</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Henan Songshan</t>
+          <t>Middelfart</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tianjin Jinmen</t>
+          <t>Roskilde</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16.10.2026</t>
+          <t>17.10.2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Süper Lig</t>
+          <t>2. Lig</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3211053</t>
+          <t>3218902</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>2.16</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>2.92</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>3.29</t>
+          <t>2.33</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>1.40</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.17</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2.26</t>
+          <t>2.65</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>1.93</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>3.85</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>7.15</t>
-        </is>
-      </c>
+          <t>2.82</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2.90</t>
+          <t>3.44</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>1.14</t>
+          <t>1.06</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>1.58</t>
+          <t>1.78</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>1.70</t>
+          <t>1.49</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.23</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>2.88</t>
+          <t>2.36</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr"/>
-      <c r="AA14" t="inlineStr">
-        <is>
-          <t>5.38</t>
-        </is>
-      </c>
+      <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>3.92</t>
+          <t>3.31</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>1.70</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="AD14" t="inlineStr">
         <is>
-          <t>3.05</t>
+          <t>4.03</t>
         </is>
       </c>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>3.27</t>
+          <t>3.76</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr"/>
       <c r="AG14" t="inlineStr"/>
-      <c r="AH14" t="inlineStr">
-        <is>
-          <t>4.45</t>
-        </is>
-      </c>
-      <c r="AI14" t="inlineStr">
-        <is>
-          <t>7.39</t>
-        </is>
-      </c>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>2.46</t>
+          <t>1.52</t>
         </is>
       </c>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="AL14" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.30</t>
         </is>
       </c>
       <c r="AM14" t="inlineStr">
         <is>
-          <t>2.44</t>
-        </is>
-      </c>
-      <c r="AN14" t="inlineStr">
-        <is>
-          <t>2.70</t>
-        </is>
-      </c>
-      <c r="AO14" t="inlineStr">
-        <is>
-          <t>13.40</t>
-        </is>
-      </c>
-      <c r="AP14" t="inlineStr">
-        <is>
-          <t>35.00</t>
-        </is>
-      </c>
-      <c r="AQ14" t="inlineStr">
-        <is>
-          <t>4.61</t>
-        </is>
-      </c>
-      <c r="AR14" t="inlineStr">
-        <is>
-          <t>4.59</t>
-        </is>
-      </c>
-      <c r="AS14" t="inlineStr">
-        <is>
-          <t>7.66</t>
-        </is>
-      </c>
-      <c r="AT14" t="inlineStr">
-        <is>
-          <t>25.50</t>
-        </is>
-      </c>
-      <c r="AU14" t="inlineStr">
-        <is>
-          <t>14.35</t>
-        </is>
-      </c>
-      <c r="AV14" t="inlineStr">
-        <is>
-          <t>5.91</t>
-        </is>
-      </c>
+          <t>2.15</t>
+        </is>
+      </c>
+      <c r="AN14" t="inlineStr"/>
+      <c r="AO14" t="inlineStr"/>
+      <c r="AP14" t="inlineStr"/>
+      <c r="AQ14" t="inlineStr"/>
+      <c r="AR14" t="inlineStr"/>
+      <c r="AS14" t="inlineStr"/>
+      <c r="AT14" t="inlineStr"/>
+      <c r="AU14" t="inlineStr"/>
+      <c r="AV14" t="inlineStr"/>
       <c r="AW14" t="inlineStr">
         <is>
-          <t>2.97</t>
+          <t>3.62</t>
         </is>
       </c>
       <c r="AX14" t="inlineStr">
         <is>
-          <t>1.74</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="AY14" t="inlineStr">
         <is>
-          <t>3.60</t>
+          <t>3.04</t>
         </is>
       </c>
       <c r="AZ14" t="inlineStr">
         <is>
-          <t>15.10</t>
+          <t>10.10</t>
         </is>
       </c>
       <c r="BA14" t="inlineStr">
         <is>
-          <t>1.77</t>
-        </is>
-      </c>
-      <c r="BB14" t="inlineStr">
-        <is>
-          <t>3.61</t>
-        </is>
-      </c>
+          <t>1.85</t>
+        </is>
+      </c>
+      <c r="BB14" t="inlineStr"/>
       <c r="BC14" t="inlineStr">
         <is>
-          <t>2.77</t>
-        </is>
-      </c>
-      <c r="BD14" t="inlineStr">
-        <is>
-          <t>6.79</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>HB Koge</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Akademisk Bo</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>16.10.2026</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>1. Lig</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>3210788</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>2.07</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>3.18</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>2.29</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>1.16</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>1.31</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>1.20</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>2.56</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>2.14</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>2.77</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>4.18</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr"/>
-      <c r="V15" t="inlineStr">
-        <is>
-          <t>2.08</t>
-        </is>
-      </c>
-      <c r="W15" t="inlineStr">
-        <is>
-          <t>1.35</t>
-        </is>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>1.37</t>
-        </is>
-      </c>
-      <c r="Y15" t="inlineStr">
-        <is>
-          <t>2.01</t>
-        </is>
-      </c>
-      <c r="Z15" t="inlineStr">
-        <is>
-          <t>1.08</t>
-        </is>
-      </c>
-      <c r="AA15" t="inlineStr">
-        <is>
-          <t>3.43</t>
-        </is>
-      </c>
-      <c r="AB15" t="inlineStr">
-        <is>
-          <t>2.97</t>
-        </is>
-      </c>
-      <c r="AC15" t="inlineStr">
-        <is>
-          <t>1.13</t>
-        </is>
-      </c>
-      <c r="AD15" t="inlineStr">
-        <is>
-          <t>3.72</t>
-        </is>
-      </c>
-      <c r="AE15" t="inlineStr">
-        <is>
-          <t>3.84</t>
-        </is>
-      </c>
-      <c r="AF15" t="inlineStr"/>
-      <c r="AG15" t="inlineStr"/>
-      <c r="AH15" t="inlineStr">
-        <is>
-          <t>4.02</t>
-        </is>
-      </c>
-      <c r="AI15" t="inlineStr">
-        <is>
-          <t>4.24</t>
-        </is>
-      </c>
-      <c r="AJ15" t="inlineStr">
-        <is>
-          <t>3.07</t>
-        </is>
-      </c>
-      <c r="AK15" t="inlineStr">
-        <is>
-          <t>1.11</t>
-        </is>
-      </c>
-      <c r="AL15" t="inlineStr">
-        <is>
-          <t>1.41</t>
-        </is>
-      </c>
-      <c r="AM15" t="inlineStr">
-        <is>
           <t>1.94</t>
         </is>
       </c>
-      <c r="AN15" t="inlineStr">
-        <is>
-          <t>3.36</t>
-        </is>
-      </c>
-      <c r="AO15" t="inlineStr">
-        <is>
-          <t>12.45</t>
-        </is>
-      </c>
-      <c r="AP15" t="inlineStr">
-        <is>
-          <t>24.95</t>
-        </is>
-      </c>
-      <c r="AQ15" t="inlineStr">
-        <is>
-          <t>5.82</t>
-        </is>
-      </c>
-      <c r="AR15" t="inlineStr">
-        <is>
-          <t>5.63</t>
-        </is>
-      </c>
-      <c r="AS15" t="inlineStr">
-        <is>
-          <t>6.28</t>
-        </is>
-      </c>
-      <c r="AT15" t="inlineStr">
-        <is>
-          <t>23.65</t>
-        </is>
-      </c>
-      <c r="AU15" t="inlineStr">
-        <is>
-          <t>12.55</t>
-        </is>
-      </c>
-      <c r="AV15" t="inlineStr">
-        <is>
-          <t>3.77</t>
-        </is>
-      </c>
-      <c r="AW15" t="inlineStr">
-        <is>
-          <t>4.54</t>
-        </is>
-      </c>
-      <c r="AX15" t="inlineStr">
-        <is>
-          <t>1.89</t>
-        </is>
-      </c>
-      <c r="AY15" t="inlineStr">
-        <is>
-          <t>2.71</t>
-        </is>
-      </c>
-      <c r="AZ15" t="inlineStr">
-        <is>
-          <t>7.24</t>
-        </is>
-      </c>
-      <c r="BA15" t="inlineStr">
-        <is>
-          <t>1.67</t>
-        </is>
-      </c>
-      <c r="BB15" t="inlineStr">
-        <is>
-          <t>3.33</t>
-        </is>
-      </c>
-      <c r="BC15" t="inlineStr">
-        <is>
-          <t>1.77</t>
-        </is>
-      </c>
-      <c r="BD15" t="inlineStr">
-        <is>
-          <t>3.63</t>
-        </is>
-      </c>
+      <c r="BD14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
veri: iddaa guncellendi (20.10.2026 00:59)
</commit_message>
<xml_diff>
--- a/iddaa/gunluk/gunlukmaclar.xlsx
+++ b/iddaa/gunluk/gunlukmaclar.xlsx
@@ -425,11 +425,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD5"/>
+  <dimension ref="A1:BD2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
@@ -1010,768 +1010,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Bromley</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Leicester City</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>20.10.2026</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>21:45</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1. Lig</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>3224032</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>3.56</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>3.47</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>1.51</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>1.37</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>1.27</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>1.07</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>3.83</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>2.20</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>1.93</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>4.29</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>2.13</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>1.31</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>1.40</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>1.94</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>1.08</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>3.26</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>3.02</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>1.11</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>7.32</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>4.99</t>
-        </is>
-      </c>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>3.44</t>
-        </is>
-      </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>2.36</t>
-        </is>
-      </c>
-      <c r="AJ3" t="inlineStr">
-        <is>
-          <t>3.16</t>
-        </is>
-      </c>
-      <c r="AK3" t="inlineStr">
-        <is>
-          <t>1.09</t>
-        </is>
-      </c>
-      <c r="AL3" t="inlineStr">
-        <is>
-          <t>1.42</t>
-        </is>
-      </c>
-      <c r="AM3" t="inlineStr">
-        <is>
-          <t>1.88</t>
-        </is>
-      </c>
-      <c r="AN3" t="inlineStr">
-        <is>
-          <t>6.23</t>
-        </is>
-      </c>
-      <c r="AO3" t="inlineStr">
-        <is>
-          <t>14.20</t>
-        </is>
-      </c>
-      <c r="AP3" t="inlineStr">
-        <is>
-          <t>19.95</t>
-        </is>
-      </c>
-      <c r="AQ3" t="inlineStr">
-        <is>
-          <t>9.02</t>
-        </is>
-      </c>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>6.03</t>
-        </is>
-      </c>
-      <c r="AS3" t="inlineStr">
-        <is>
-          <t>4.62</t>
-        </is>
-      </c>
-      <c r="AT3" t="inlineStr">
-        <is>
-          <t>34.50</t>
-        </is>
-      </c>
-      <c r="AU3" t="inlineStr">
-        <is>
-          <t>13.10</t>
-        </is>
-      </c>
-      <c r="AV3" t="inlineStr">
-        <is>
-          <t>2.24</t>
-        </is>
-      </c>
-      <c r="AW3" t="inlineStr">
-        <is>
-          <t>4.69</t>
-        </is>
-      </c>
-      <c r="AX3" t="inlineStr">
-        <is>
-          <t>1.89</t>
-        </is>
-      </c>
-      <c r="AY3" t="inlineStr">
-        <is>
-          <t>2.64</t>
-        </is>
-      </c>
-      <c r="AZ3" t="inlineStr">
-        <is>
-          <t>6.78</t>
-        </is>
-      </c>
-      <c r="BA3" t="inlineStr">
-        <is>
-          <t>2.25</t>
-        </is>
-      </c>
-      <c r="BB3" t="inlineStr">
-        <is>
-          <t>5.21</t>
-        </is>
-      </c>
-      <c r="BC3" t="inlineStr">
-        <is>
-          <t>1.37</t>
-        </is>
-      </c>
-      <c r="BD3" t="inlineStr">
-        <is>
-          <t>2.39</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Barnet</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Swindon Town</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>20.10.2026</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>21:45</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2. Lig</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>3224036</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>1.29</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>3.94</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>4.82</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>1.23</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>1.51</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>1.68</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>2.32</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>4.82</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>4.31</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>2.15</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>1.30</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>1.40</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>1.93</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>1.08</t>
-        </is>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>3.22</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>3.20</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>1.08</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>3.35</t>
-        </is>
-      </c>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>5.79</t>
-        </is>
-      </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>10.50</t>
-        </is>
-      </c>
-      <c r="AJ4" t="inlineStr">
-        <is>
-          <t>3.26</t>
-        </is>
-      </c>
-      <c r="AK4" t="inlineStr">
-        <is>
-          <t>1.08</t>
-        </is>
-      </c>
-      <c r="AL4" t="inlineStr">
-        <is>
-          <t>1.44</t>
-        </is>
-      </c>
-      <c r="AM4" t="inlineStr">
-        <is>
-          <t>1.86</t>
-        </is>
-      </c>
-      <c r="AN4" t="inlineStr">
-        <is>
-          <t>1.85</t>
-        </is>
-      </c>
-      <c r="AO4" t="inlineStr">
-        <is>
-          <t>15.10</t>
-        </is>
-      </c>
-      <c r="AP4" t="inlineStr">
-        <is>
-          <t>34.50</t>
-        </is>
-      </c>
-      <c r="AQ4" t="inlineStr">
-        <is>
-          <t>4.21</t>
-        </is>
-      </c>
-      <c r="AR4" t="inlineStr">
-        <is>
-          <t>6.71</t>
-        </is>
-      </c>
-      <c r="AS4" t="inlineStr">
-        <is>
-          <t>11.75</t>
-        </is>
-      </c>
-      <c r="AT4" t="inlineStr">
-        <is>
-          <t>19.50</t>
-        </is>
-      </c>
-      <c r="AU4" t="inlineStr">
-        <is>
-          <t>16.85</t>
-        </is>
-      </c>
-      <c r="AV4" t="inlineStr">
-        <is>
-          <t>8.76</t>
-        </is>
-      </c>
-      <c r="AW4" t="inlineStr">
-        <is>
-          <t>4.74</t>
-        </is>
-      </c>
-      <c r="AX4" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
-      <c r="AY4" t="inlineStr">
-        <is>
-          <t>2.63</t>
-        </is>
-      </c>
-      <c r="AZ4" t="inlineStr">
-        <is>
-          <t>6.69</t>
-        </is>
-      </c>
-      <c r="BA4" t="inlineStr">
-        <is>
-          <t>1.27</t>
-        </is>
-      </c>
-      <c r="BB4" t="inlineStr">
-        <is>
-          <t>2.06</t>
-        </is>
-      </c>
-      <c r="BC4" t="inlineStr">
-        <is>
-          <t>2.76</t>
-        </is>
-      </c>
-      <c r="BD4" t="inlineStr">
-        <is>
-          <t>6.77</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Bristol Rovers</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Salford City</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>20.10.2026</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>21:45</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2. Lig</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>3224019</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2.26</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>2.92</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>2.23</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>1.15</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>1.34</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>1.15</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>2.74</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>2.72</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>8.22</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>3.50</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>1.06</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>1.48</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>1.24</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>2.32</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>4.18</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>3.29</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>1.08</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>4.25</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>3.84</t>
-        </is>
-      </c>
-      <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>3.83</t>
-        </is>
-      </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>4.19</t>
-        </is>
-      </c>
-      <c r="AJ5" t="inlineStr">
-        <is>
-          <t>2.73</t>
-        </is>
-      </c>
-      <c r="AK5" t="inlineStr">
-        <is>
-          <t>1.15</t>
-        </is>
-      </c>
-      <c r="AL5" t="inlineStr">
-        <is>
-          <t>1.31</t>
-        </is>
-      </c>
-      <c r="AM5" t="inlineStr">
-        <is>
-          <t>2.13</t>
-        </is>
-      </c>
-      <c r="AN5" t="inlineStr">
-        <is>
-          <t>3.70</t>
-        </is>
-      </c>
-      <c r="AO5" t="inlineStr">
-        <is>
-          <t>12.20</t>
-        </is>
-      </c>
-      <c r="AP5" t="inlineStr">
-        <is>
-          <t>26.50</t>
-        </is>
-      </c>
-      <c r="AQ5" t="inlineStr">
-        <is>
-          <t>5.96</t>
-        </is>
-      </c>
-      <c r="AR5" t="inlineStr">
-        <is>
-          <t>4.87</t>
-        </is>
-      </c>
-      <c r="AS5" t="inlineStr">
-        <is>
-          <t>5.92</t>
-        </is>
-      </c>
-      <c r="AT5" t="inlineStr">
-        <is>
-          <t>26.50</t>
-        </is>
-      </c>
-      <c r="AU5" t="inlineStr">
-        <is>
-          <t>12.15</t>
-        </is>
-      </c>
-      <c r="AV5" t="inlineStr">
-        <is>
-          <t>3.66</t>
-        </is>
-      </c>
-      <c r="AW5" t="inlineStr">
-        <is>
-          <t>3.68</t>
-        </is>
-      </c>
-      <c r="AX5" t="inlineStr">
-        <is>
-          <t>1.78</t>
-        </is>
-      </c>
-      <c r="AY5" t="inlineStr">
-        <is>
-          <t>3.01</t>
-        </is>
-      </c>
-      <c r="AZ5" t="inlineStr">
-        <is>
-          <t>9.85</t>
-        </is>
-      </c>
-      <c r="BA5" t="inlineStr">
-        <is>
-          <t>1.88</t>
-        </is>
-      </c>
-      <c r="BB5" t="inlineStr">
-        <is>
-          <t>4.03</t>
-        </is>
-      </c>
-      <c r="BC5" t="inlineStr">
-        <is>
-          <t>1.87</t>
-        </is>
-      </c>
-      <c r="BD5" t="inlineStr">
-        <is>
-          <t>3.99</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
veri: iddaa guncellendi (20.10.2026 10:00)
</commit_message>
<xml_diff>
--- a/iddaa/gunluk/gunlukmaclar.xlsx
+++ b/iddaa/gunluk/gunlukmaclar.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD37"/>
+  <dimension ref="A1:BD35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -438,7 +438,7 @@
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="6" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
     <col width="7" customWidth="1" min="12" max="12"/>
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
@@ -771,12 +771,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Liverpool</t>
+          <t>Sabah</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>B. Dortmund</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -786,247 +786,91 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Şampiyonlar Ligi</t>
+          <t>Avrupa Şampiyonlar Ligi</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3223961</t>
+          <t>3224154</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>7.71</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>4.57</t>
+          <t>5.27</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>5.57</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>1.27</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>1.66</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>1.68</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>2.49</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>5.20</t>
-        </is>
-      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>5.29</t>
-        </is>
-      </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>2.43</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>1.29</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>1.52</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>1.89</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>1.15</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>3.19</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>3.35</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>1.13</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>1.87</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>3.57</t>
-        </is>
-      </c>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>6.95</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>12.50</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>3.76</t>
-        </is>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>1.08</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>1.54</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>1.86</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>1.79</t>
-        </is>
-      </c>
-      <c r="AO2" t="inlineStr">
-        <is>
-          <t>15.55</t>
-        </is>
-      </c>
-      <c r="AP2" t="inlineStr">
-        <is>
-          <t>34.50</t>
-        </is>
-      </c>
-      <c r="AQ2" t="inlineStr">
-        <is>
-          <t>4.26</t>
-        </is>
-      </c>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>7.23</t>
-        </is>
-      </c>
-      <c r="AS2" t="inlineStr">
-        <is>
-          <t>12.60</t>
-        </is>
-      </c>
-      <c r="AT2" t="inlineStr">
-        <is>
-          <t>19.15</t>
-        </is>
-      </c>
-      <c r="AU2" t="inlineStr">
-        <is>
-          <t>17.40</t>
-        </is>
-      </c>
-      <c r="AV2" t="inlineStr">
-        <is>
-          <t>9.20</t>
-        </is>
-      </c>
-      <c r="AW2" t="inlineStr">
-        <is>
-          <t>5.59</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr">
-        <is>
-          <t>2.20</t>
-        </is>
-      </c>
-      <c r="AY2" t="inlineStr">
-        <is>
-          <t>2.80</t>
-        </is>
-      </c>
-      <c r="AZ2" t="inlineStr">
-        <is>
-          <t>6.31</t>
-        </is>
-      </c>
-      <c r="BA2" t="inlineStr">
-        <is>
-          <t>1.46</t>
-        </is>
-      </c>
-      <c r="BB2" t="inlineStr">
-        <is>
-          <t>2.22</t>
-        </is>
-      </c>
-      <c r="BC2" t="inlineStr">
-        <is>
-          <t>2.89</t>
-        </is>
-      </c>
-      <c r="BD2" t="inlineStr">
-        <is>
-          <t>8.31</t>
-        </is>
-      </c>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr"/>
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Man. City</t>
+          <t>Fenerbahçe</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AEK</t>
+          <t>Slavia Prag</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1036,7 +880,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1046,20 +890,24 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3224028</t>
+          <t>3224111</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>1.37</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>9.33</t>
+          <t>4.08</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>17.35</t>
+          <t>4.68</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -1111,12 +959,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fenerbahçe</t>
+          <t>Liverpool</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Slavia Prag</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1126,7 +974,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1136,24 +984,24 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3224111</t>
+          <t>3223961</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.37</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>4.08</t>
+          <t>4.37</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>4.68</t>
+          <t>5.37</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -1299,12 +1147,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sabah</t>
+          <t>PSG</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>B. Dortmund</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1314,91 +1162,243 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Avrupa Şampiyonlar Ligi</t>
+          <t>Şampiyonlar Ligi</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3224154</t>
+          <t>3224058</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>7.71</t>
+          <t>2.14</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>5.27</t>
+          <t>3.85</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>1.15</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
+          <t>2.17</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2.66</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>2.85</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2.68</t>
+        </is>
+      </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
-      <c r="AB6" t="inlineStr"/>
-      <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>4.36</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>2.49</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>2.36</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>1.58</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>3.47</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>4.59</t>
+        </is>
+      </c>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>4.61</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>3.51</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>5.33</t>
+        </is>
+      </c>
       <c r="AK6" t="inlineStr"/>
-      <c r="AL6" t="inlineStr"/>
-      <c r="AM6" t="inlineStr"/>
-      <c r="AN6" t="inlineStr"/>
-      <c r="AO6" t="inlineStr"/>
-      <c r="AP6" t="inlineStr"/>
-      <c r="AQ6" t="inlineStr"/>
-      <c r="AR6" t="inlineStr"/>
-      <c r="AS6" t="inlineStr"/>
-      <c r="AT6" t="inlineStr"/>
-      <c r="AU6" t="inlineStr"/>
-      <c r="AV6" t="inlineStr"/>
-      <c r="AW6" t="inlineStr"/>
-      <c r="AX6" t="inlineStr"/>
-      <c r="AY6" t="inlineStr"/>
-      <c r="AZ6" t="inlineStr"/>
-      <c r="BA6" t="inlineStr"/>
-      <c r="BB6" t="inlineStr"/>
-      <c r="BC6" t="inlineStr"/>
-      <c r="BD6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>1.99</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>1.47</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>3.22</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>12.00</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>18.40</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>6.77</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>7.93</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>6.81</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>18.30</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>12.05</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>11.60</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>2.96</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>2.47</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>3.12</t>
+        </is>
+      </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>2.23</t>
+        </is>
+      </c>
+      <c r="BC6" t="inlineStr">
+        <is>
+          <t>1.33</t>
+        </is>
+      </c>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>2.45</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PSG</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>PSV</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1413,238 +1413,86 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Şampiyonlar Ligi</t>
+          <t>Avrupa Şampiyonlar Ligi</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3224058</t>
+          <t>3224197</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2.14</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>3.85</t>
+          <t>4.06</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.17</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>1.48</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>1.43</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>1.48</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>2.66</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>2.85</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>2.68</t>
-        </is>
-      </c>
+          <t>4.83</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>4.36</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>1.26</t>
-        </is>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>2.49</t>
-        </is>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>1.53</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>1.51</t>
-        </is>
-      </c>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>1.90</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>2.36</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>1.58</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>3.47</t>
-        </is>
-      </c>
-      <c r="AE7" t="inlineStr">
-        <is>
-          <t>4.59</t>
-        </is>
-      </c>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>4.61</t>
-        </is>
-      </c>
-      <c r="AI7" t="inlineStr">
-        <is>
-          <t>3.51</t>
-        </is>
-      </c>
-      <c r="AJ7" t="inlineStr">
-        <is>
-          <t>5.33</t>
-        </is>
-      </c>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr">
-        <is>
-          <t>1.99</t>
-        </is>
-      </c>
-      <c r="AM7" t="inlineStr">
-        <is>
-          <t>1.47</t>
-        </is>
-      </c>
-      <c r="AN7" t="inlineStr">
-        <is>
-          <t>3.22</t>
-        </is>
-      </c>
-      <c r="AO7" t="inlineStr">
-        <is>
-          <t>12.00</t>
-        </is>
-      </c>
-      <c r="AP7" t="inlineStr">
-        <is>
-          <t>18.40</t>
-        </is>
-      </c>
-      <c r="AQ7" t="inlineStr">
-        <is>
-          <t>6.77</t>
-        </is>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>7.93</t>
-        </is>
-      </c>
-      <c r="AS7" t="inlineStr">
-        <is>
-          <t>6.81</t>
-        </is>
-      </c>
-      <c r="AT7" t="inlineStr">
-        <is>
-          <t>18.30</t>
-        </is>
-      </c>
-      <c r="AU7" t="inlineStr">
-        <is>
-          <t>12.05</t>
-        </is>
-      </c>
-      <c r="AV7" t="inlineStr">
-        <is>
-          <t>3.25</t>
-        </is>
-      </c>
-      <c r="AW7" t="inlineStr">
-        <is>
-          <t>11.60</t>
-        </is>
-      </c>
-      <c r="AX7" t="inlineStr">
-        <is>
-          <t>2.96</t>
-        </is>
-      </c>
-      <c r="AY7" t="inlineStr">
-        <is>
-          <t>2.47</t>
-        </is>
-      </c>
-      <c r="AZ7" t="inlineStr">
-        <is>
-          <t>3.12</t>
-        </is>
-      </c>
-      <c r="BA7" t="inlineStr">
-        <is>
-          <t>1.32</t>
-        </is>
-      </c>
-      <c r="BB7" t="inlineStr">
-        <is>
-          <t>2.23</t>
-        </is>
-      </c>
-      <c r="BC7" t="inlineStr">
-        <is>
-          <t>1.33</t>
-        </is>
-      </c>
-      <c r="BD7" t="inlineStr">
-        <is>
-          <t>2.45</t>
-        </is>
-      </c>
+      <c r="AL7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr"/>
+      <c r="AZ7" t="inlineStr"/>
+      <c r="BA7" t="inlineStr"/>
+      <c r="BB7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr"/>
+      <c r="BD7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Wolverhampton</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PSV</t>
+          <t>Portsmouth</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1654,34 +1502,34 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Avrupa Şampiyonlar Ligi</t>
+          <t>İngiltere Championship</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>3224197</t>
+          <t>3224120</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>4.06</t>
+          <t>3.74</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>4.83</t>
+          <t>4.75</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -1733,12 +1581,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Roma</t>
+          <t>Stuttgart</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>S. Bratislava</t>
+          <t>Atl. Madrid</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1758,20 +1606,24 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>3224207</t>
+          <t>3224221</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2.88</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>9.28</t>
+          <t>3.42</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>17.35</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -1823,12 +1675,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Stuttgart</t>
+          <t>Blackpool</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Atl. Madrid</t>
+          <t>MK Dons</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1838,34 +1690,34 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Avrupa Şampiyonlar Ligi</t>
+          <t>İngiltere 1. Lig</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>3224221</t>
+          <t>3224127</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2.88</t>
+          <t>2.09</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>3.42</t>
+          <t>3.10</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1.83</t>
+          <t>2.31</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -1917,12 +1769,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Wolverhampton</t>
+          <t>Burton Albion</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Portsmouth</t>
+          <t>Bradford</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1937,29 +1789,29 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>İngiltere Championship</t>
+          <t>İngiltere 1. Lig</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>3224120</t>
+          <t>3223962</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1.41</t>
+          <t>3.07</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>3.74</t>
+          <t>2.89</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>4.75</t>
+          <t>1.78</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -2011,12 +1863,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Blackpool</t>
+          <t>Bromley</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MK Dons</t>
+          <t>Leicester City</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2036,24 +1888,24 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>3224127</t>
+          <t>3224032</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2.09</t>
+          <t>3.53</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>3.10</t>
+          <t>3.50</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2.31</t>
+          <t>1.50</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
@@ -2105,12 +1957,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Bromley</t>
+          <t>Cambridge</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Leicester City</t>
+          <t>Wycombe</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2130,24 +1982,24 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3224032</t>
+          <t>3223963</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3.53</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>3.50</t>
+          <t>3.02</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>2.47</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -2199,12 +2051,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Burton Albion</t>
+          <t>Doncaster</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bradford</t>
+          <t>Stockport</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2224,24 +2076,24 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3223962</t>
+          <t>3224204</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>3.07</t>
+          <t>3.23</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2.89</t>
+          <t>3.21</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1.78</t>
+          <t>1.63</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -2293,12 +2145,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cambridge</t>
+          <t>Huddersfield</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Wycombe</t>
+          <t>Peterborough</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2318,24 +2170,24 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3223963</t>
+          <t>3224195</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>3.02</t>
+          <t>3.88</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2.47</t>
+          <t>4.26</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
@@ -2387,12 +2239,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Doncaster</t>
+          <t>Luton Town</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Stockport</t>
+          <t>Barnsley</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2412,24 +2264,24 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>3224204</t>
+          <t>3224071</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>3.23</t>
+          <t>1.32</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3.21</t>
+          <t>4.03</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1.63</t>
+          <t>4.42</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
@@ -2481,12 +2333,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Luton Town</t>
+          <t>Notts County</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Barnsley</t>
+          <t>S. Wednesday</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2506,24 +2358,24 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>3224071</t>
+          <t>3224101</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>1.32</t>
+          <t>2.73</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>4.03</t>
+          <t>2.98</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>4.42</t>
+          <t>1.87</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
@@ -2575,12 +2427,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Huddersfield</t>
+          <t>Oxford Utd</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Peterborough</t>
+          <t>Wigan Ath</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2600,24 +2452,24 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>3224195</t>
+          <t>3224097</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1.35</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>3.88</t>
+          <t>3.03</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>4.26</t>
+          <t>3.08</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
@@ -2669,12 +2521,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Oxford Utd</t>
+          <t>Stevenage</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Wigan Ath</t>
+          <t>Plymouth</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2694,24 +2546,24 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3224097</t>
+          <t>3223983</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>2.27</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>3.03</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>3.08</t>
+          <t>2.26</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
@@ -2763,12 +2615,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Notts County</t>
+          <t>Norrköping</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>S. Wednesday</t>
+          <t>Orebro SK</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2778,34 +2630,34 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>İngiltere 1. Lig</t>
+          <t>İsveç Superettan</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>3224101</t>
+          <t>3224044</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2.73</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>3.61</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>1.87</t>
+          <t>3.95</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
@@ -2857,12 +2709,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Stevenage</t>
+          <t>Wimbledon</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Plymouth</t>
+          <t>Mansfield</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2882,24 +2734,24 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>3223983</t>
+          <t>3224106</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>2.78</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2.87</t>
+          <t>2.98</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2.26</t>
+          <t>1.86</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
@@ -2951,12 +2803,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Wimbledon</t>
+          <t>Barnet</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Mansfield</t>
+          <t>Swindon Town</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2971,29 +2823,29 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>İngiltere 1. Lig</t>
+          <t>İngiltere 2. Lig</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>3224106</t>
+          <t>3224036</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2.78</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>3.99</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>1.86</t>
+          <t>4.81</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
@@ -3045,12 +2897,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Norrköping</t>
+          <t>Bristol Rovers</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Orebro SK</t>
+          <t>Salford City</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3060,34 +2912,34 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>İsveç Superettan</t>
+          <t>İngiltere 2. Lig</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>3224044</t>
+          <t>3224019</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>2.26</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>3.61</t>
+          <t>2.92</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>3.95</t>
+          <t>2.23</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
@@ -3139,12 +2991,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Bristol Rovers</t>
+          <t>Cheltenham</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Salford City</t>
+          <t>Fleetwood</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3164,24 +3016,24 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>3224019</t>
+          <t>3224009</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2.26</t>
+          <t>2.67</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2.92</t>
+          <t>2.97</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2.23</t>
+          <t>1.92</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>
@@ -3233,12 +3085,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Barnet</t>
+          <t>Chesterfield</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Swindon Town</t>
+          <t>Colchester</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3258,24 +3110,24 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>3224036</t>
+          <t>3224222</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>1.29</t>
+          <t>1.39</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>3.99</t>
+          <t>3.61</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>4.81</t>
+          <t>4.24</t>
         </is>
       </c>
       <c r="L25" t="inlineStr"/>
@@ -3327,12 +3179,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Cheltenham</t>
+          <t>Crawley Town</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Fleetwood</t>
+          <t>Shrewsbury</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3352,24 +3204,24 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>3224009</t>
+          <t>3224193</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2.67</t>
+          <t>2.50</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2.97</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>1.92</t>
+          <t>2.06</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
@@ -3421,12 +3273,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Crawley Town</t>
+          <t>Exeter City</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Shrewsbury</t>
+          <t>Crewe</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3446,24 +3298,24 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>3224193</t>
+          <t>3224141</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2.50</t>
+          <t>2.19</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2.87</t>
+          <t>2.78</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>2.06</t>
+          <t>2.41</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
@@ -3515,12 +3367,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Chesterfield</t>
+          <t>Northampton</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Colchester</t>
+          <t>Tranmere</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3540,24 +3392,24 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>3224222</t>
+          <t>3224229</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>1.39</t>
+          <t>1.99</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>3.61</t>
+          <t>2.82</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>4.24</t>
+          <t>2.65</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
@@ -3609,12 +3461,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Exeter City</t>
+          <t>Rochdale</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Crewe</t>
+          <t>Grimsby</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3634,24 +3486,24 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>3224141</t>
+          <t>3224016</t>
         </is>
       </c>
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2.19</t>
+          <t>2.64</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2.78</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>2.41</t>
+          <t>1.93</t>
         </is>
       </c>
       <c r="L29" t="inlineStr"/>
@@ -3703,12 +3555,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Rochdale</t>
+          <t>Rotherham</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Grimsby</t>
+          <t>Newport</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3728,24 +3580,24 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>3224016</t>
+          <t>3224041</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2.64</t>
+          <t>1.91</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>3.00</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>1.93</t>
+          <t>2.77</t>
         </is>
       </c>
       <c r="L30" t="inlineStr"/>
@@ -3797,12 +3649,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Northampton</t>
+          <t>Gillingham</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Tranmere</t>
+          <t>Port Vale</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3812,7 +3664,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3822,24 +3674,24 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>3224229</t>
+          <t>3224153</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>1.99</t>
+          <t>2.70</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2.82</t>
+          <t>2.77</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>2.65</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="L31" t="inlineStr"/>
@@ -3891,12 +3743,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Rotherham</t>
+          <t>Walsall</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Newport</t>
+          <t>Oldham</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3916,24 +3768,24 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>3224041</t>
+          <t>3224242</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>1.91</t>
+          <t>2.08</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2.87</t>
+          <t>2.97</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>2.77</t>
+          <t>2.41</t>
         </is>
       </c>
       <c r="L32" t="inlineStr"/>
@@ -3985,12 +3837,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Walsall</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Oldham</t>
+          <t>Accrington</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -4010,24 +3862,24 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>3224242</t>
+          <t>3224216</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2.08</t>
+          <t>1.52</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2.97</t>
+          <t>3.33</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>2.41</t>
+          <t>3.66</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
@@ -4079,12 +3931,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Dunfermline</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Accrington</t>
+          <t>P. Thistle</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -4099,29 +3951,29 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>İngiltere 2. Lig</t>
+          <t>İskoçya Championship</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>3224216</t>
+          <t>3245943</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>2.47</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>3.33</t>
+          <t>2.83</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>3.66</t>
+          <t>2.10</t>
         </is>
       </c>
       <c r="L34" t="inlineStr"/>
@@ -4173,12 +4025,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Gillingham</t>
+          <t>ASA T. Mureş</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Port Vale</t>
+          <t>Chindia T.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -4188,34 +4040,34 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>İngiltere 2. Lig</t>
+          <t>Romanya 2. Lig</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>3224153</t>
+          <t>3300931</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2.70</t>
+          <t>2.64</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2.77</t>
+          <t>2.92</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>1.95</t>
         </is>
       </c>
       <c r="L35" t="inlineStr"/>
@@ -4264,194 +4116,6 @@
       <c r="BC35" t="inlineStr"/>
       <c r="BD35" t="inlineStr"/>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Dunfermline</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>P. Thistle</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>20.10.2026</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>21:45</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>İskoçya Championship</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>3245943</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>2.47</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>2.83</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr"/>
-      <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr"/>
-      <c r="W36" t="inlineStr"/>
-      <c r="X36" t="inlineStr"/>
-      <c r="Y36" t="inlineStr"/>
-      <c r="Z36" t="inlineStr"/>
-      <c r="AA36" t="inlineStr"/>
-      <c r="AB36" t="inlineStr"/>
-      <c r="AC36" t="inlineStr"/>
-      <c r="AD36" t="inlineStr"/>
-      <c r="AE36" t="inlineStr"/>
-      <c r="AF36" t="inlineStr"/>
-      <c r="AG36" t="inlineStr"/>
-      <c r="AH36" t="inlineStr"/>
-      <c r="AI36" t="inlineStr"/>
-      <c r="AJ36" t="inlineStr"/>
-      <c r="AK36" t="inlineStr"/>
-      <c r="AL36" t="inlineStr"/>
-      <c r="AM36" t="inlineStr"/>
-      <c r="AN36" t="inlineStr"/>
-      <c r="AO36" t="inlineStr"/>
-      <c r="AP36" t="inlineStr"/>
-      <c r="AQ36" t="inlineStr"/>
-      <c r="AR36" t="inlineStr"/>
-      <c r="AS36" t="inlineStr"/>
-      <c r="AT36" t="inlineStr"/>
-      <c r="AU36" t="inlineStr"/>
-      <c r="AV36" t="inlineStr"/>
-      <c r="AW36" t="inlineStr"/>
-      <c r="AX36" t="inlineStr"/>
-      <c r="AY36" t="inlineStr"/>
-      <c r="AZ36" t="inlineStr"/>
-      <c r="BA36" t="inlineStr"/>
-      <c r="BB36" t="inlineStr"/>
-      <c r="BC36" t="inlineStr"/>
-      <c r="BD36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>ASA T. Mureş</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Chindia T.</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>20.10.2026</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>17:30</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Romanya 2. Lig</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>3300931</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>2.64</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>2.92</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>1.95</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
-      <c r="T37" t="inlineStr"/>
-      <c r="U37" t="inlineStr"/>
-      <c r="V37" t="inlineStr"/>
-      <c r="W37" t="inlineStr"/>
-      <c r="X37" t="inlineStr"/>
-      <c r="Y37" t="inlineStr"/>
-      <c r="Z37" t="inlineStr"/>
-      <c r="AA37" t="inlineStr"/>
-      <c r="AB37" t="inlineStr"/>
-      <c r="AC37" t="inlineStr"/>
-      <c r="AD37" t="inlineStr"/>
-      <c r="AE37" t="inlineStr"/>
-      <c r="AF37" t="inlineStr"/>
-      <c r="AG37" t="inlineStr"/>
-      <c r="AH37" t="inlineStr"/>
-      <c r="AI37" t="inlineStr"/>
-      <c r="AJ37" t="inlineStr"/>
-      <c r="AK37" t="inlineStr"/>
-      <c r="AL37" t="inlineStr"/>
-      <c r="AM37" t="inlineStr"/>
-      <c r="AN37" t="inlineStr"/>
-      <c r="AO37" t="inlineStr"/>
-      <c r="AP37" t="inlineStr"/>
-      <c r="AQ37" t="inlineStr"/>
-      <c r="AR37" t="inlineStr"/>
-      <c r="AS37" t="inlineStr"/>
-      <c r="AT37" t="inlineStr"/>
-      <c r="AU37" t="inlineStr"/>
-      <c r="AV37" t="inlineStr"/>
-      <c r="AW37" t="inlineStr"/>
-      <c r="AX37" t="inlineStr"/>
-      <c r="AY37" t="inlineStr"/>
-      <c r="AZ37" t="inlineStr"/>
-      <c r="BA37" t="inlineStr"/>
-      <c r="BB37" t="inlineStr"/>
-      <c r="BC37" t="inlineStr"/>
-      <c r="BD37" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
veri: iddaa guncellendi (22.10.2026 12:04)
</commit_message>
<xml_diff>
--- a/iddaa/gunluk/gunlukmaclar.xlsx
+++ b/iddaa/gunluk/gunlukmaclar.xlsx
@@ -425,20 +425,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD18"/>
+  <dimension ref="A1:BD37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
     <col width="7" customWidth="1" min="12" max="12"/>
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
@@ -457,7 +457,7 @@
     <col width="12" customWidth="1" min="27" max="27"/>
     <col width="8" customWidth="1" min="28" max="28"/>
     <col width="8" customWidth="1" min="29" max="29"/>
-    <col width="6" customWidth="1" min="30" max="30"/>
+    <col width="7" customWidth="1" min="30" max="30"/>
     <col width="6" customWidth="1" min="31" max="31"/>
     <col width="6" customWidth="1" min="32" max="32"/>
     <col width="8" customWidth="1" min="33" max="33"/>
@@ -771,17 +771,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Ararat-Armenia</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Galatasaray</t>
+          <t>AZ Alkmaar</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -791,287 +791,123 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Şampiyonlar Ligi</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3225985</t>
+          <t>3229849</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1.98</t>
+          <t>6.23</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>3.22</t>
+          <t>4.54</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2.70</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>1.15</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>1.38</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>1.28</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>2.47</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>2.13</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>3.18</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>12.30</t>
-        </is>
-      </c>
+          <t>1.24</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>4.42</t>
-        </is>
-      </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>2.01</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>1.45</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>1.34</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>2.26</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>1.06</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>4.15</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>3.58</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>1.32</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>3.72</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>4.02</t>
-        </is>
-      </c>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>4.44</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>5.38</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>3.11</t>
-        </is>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>1.15</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>1.40</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>2.13</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>3.25</t>
-        </is>
-      </c>
-      <c r="AO2" t="inlineStr">
-        <is>
-          <t>12.50</t>
-        </is>
-      </c>
-      <c r="AP2" t="inlineStr">
-        <is>
-          <t>28.20</t>
-        </is>
-      </c>
-      <c r="AQ2" t="inlineStr">
-        <is>
-          <t>5.60</t>
-        </is>
-      </c>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>5.50</t>
-        </is>
-      </c>
-      <c r="AS2" t="inlineStr">
-        <is>
-          <t>7.02</t>
-        </is>
-      </c>
-      <c r="AT2" t="inlineStr">
-        <is>
-          <t>23.60</t>
-        </is>
-      </c>
-      <c r="AU2" t="inlineStr">
-        <is>
-          <t>12.95</t>
-        </is>
-      </c>
-      <c r="AV2" t="inlineStr">
-        <is>
-          <t>4.59</t>
-        </is>
-      </c>
-      <c r="AW2" t="inlineStr">
-        <is>
-          <t>4.41</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr">
-        <is>
-          <t>2.07</t>
-        </is>
-      </c>
-      <c r="AY2" t="inlineStr">
-        <is>
-          <t>3.11</t>
-        </is>
-      </c>
-      <c r="AZ2" t="inlineStr">
-        <is>
-          <t>8.87</t>
-        </is>
-      </c>
-      <c r="BA2" t="inlineStr">
-        <is>
-          <t>1.91</t>
-        </is>
-      </c>
-      <c r="BB2" t="inlineStr">
-        <is>
-          <t>3.72</t>
-        </is>
-      </c>
-      <c r="BC2" t="inlineStr">
-        <is>
-          <t>2.26</t>
-        </is>
-      </c>
-      <c r="BD2" t="inlineStr">
-        <is>
-          <t>4.84</t>
-        </is>
-      </c>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr"/>
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Aston Villa</t>
+          <t>Ferencvaros</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Viking</t>
+          <t>Torreense</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Avrupa Şampiyonlar Ligi</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3226000</t>
+          <t>3230269</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>1.09</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>6.22</t>
+          <t>5.07</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>9.02</t>
+          <t>8.43</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -1123,17 +959,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Trabzonspor</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Man. United</t>
+          <t>Hearts</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1143,29 +979,29 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Avrupa Şampiyonlar Ligi</t>
+          <t>Avrupa Konferans Ligi</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3225931</t>
+          <t>3230845</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>3.36</t>
+          <t>5.87</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2.52</t>
+          <t>8.63</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -1217,49 +1053,49 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Club Brugge</t>
+          <t>D. Zagreb</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lens</t>
+          <t>NEC Nijmegen</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Avrupa Şampiyonlar Ligi</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3225754</t>
+          <t>3230256</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>1.68</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>3.70</t>
+          <t>4.09</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>3.09</t>
+          <t>4.91</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -1311,17 +1147,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bayern Münih</t>
+          <t>Beşiktaş</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>Crystal Palace</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1331,29 +1167,29 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Avrupa Şampiyonlar Ligi</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3225759</t>
+          <t>3229910</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1.83</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>3.38</t>
+          <t>3.34</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.89</t>
+          <t>2.56</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -1405,49 +1241,49 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Inter</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Shakhtar</t>
+          <t>Sunderland</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Avrupa Şampiyonlar Ligi</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3225840</t>
+          <t>3229916</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>4.09</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>6.74</t>
+          <t>3.44</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>10.30</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
@@ -1499,143 +1335,307 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Real Madrid</t>
+          <t>Sturm Graz</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Leipzig</t>
+          <t>Marsilya</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Avrupa Şampiyonlar Ligi</t>
+          <t>Avrupa Ligi</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>3225752</t>
+          <t>3230851</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1.08</t>
+          <t>3.55</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>6.78</t>
+          <t>3.49</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>9.07</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
+          <t>1.91</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1.36</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>1.38</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>3.97</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>2.33</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>2.40</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>11.85</t>
+        </is>
+      </c>
       <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>3.98</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>1.93</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>1.49</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>1.30</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>2.38</t>
+        </is>
+      </c>
       <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr"/>
-      <c r="AB8" t="inlineStr"/>
-      <c r="AC8" t="inlineStr"/>
-      <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="inlineStr"/>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>4.43</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>3.79</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>1.30</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>7.44</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>5.15</t>
+        </is>
+      </c>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr"/>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
-      <c r="AL8" t="inlineStr"/>
-      <c r="AM8" t="inlineStr"/>
-      <c r="AN8" t="inlineStr"/>
-      <c r="AO8" t="inlineStr"/>
-      <c r="AP8" t="inlineStr"/>
-      <c r="AQ8" t="inlineStr"/>
-      <c r="AR8" t="inlineStr"/>
-      <c r="AS8" t="inlineStr"/>
-      <c r="AT8" t="inlineStr"/>
-      <c r="AU8" t="inlineStr"/>
-      <c r="AV8" t="inlineStr"/>
-      <c r="AW8" t="inlineStr"/>
-      <c r="AX8" t="inlineStr"/>
-      <c r="AY8" t="inlineStr"/>
-      <c r="AZ8" t="inlineStr"/>
-      <c r="BA8" t="inlineStr"/>
-      <c r="BB8" t="inlineStr"/>
-      <c r="BC8" t="inlineStr"/>
-      <c r="BD8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>3.77</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>3.03</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>1.16</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>1.57</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>2.39</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>5.84</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>13.85</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>22.75</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>8.20</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>5.47</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>5.02</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>34.70</t>
+        </is>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>12.95</t>
+        </is>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>2.77</t>
+        </is>
+      </c>
+      <c r="AW8" t="inlineStr">
+        <is>
+          <t>4.16</t>
+        </is>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>2.04</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>3.22</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>9.74</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>2.65</t>
+        </is>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>6.57</t>
+        </is>
+      </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>1.60</t>
+        </is>
+      </c>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>3.35</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ath. Bilbao</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>İspanya LaLiga</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>3243571</t>
+          <t>3230667</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3.14</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2.92</t>
+          <t>4.17</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>1.90</t>
+          <t>5.94</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -1687,49 +1687,49 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Real Betis</t>
+          <t>OFI</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Feyenoord</t>
+          <t>B. Leverkusen</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Avrupa Şampiyonlar Ligi</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>3226015</t>
+          <t>3230543</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>10.85</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>6.68</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>3.97</t>
+          <t>1.06</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -1781,49 +1781,49 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sporting CP</t>
+          <t>Union SG</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>LASK</t>
+          <t>HB Sheva</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Avrupa Şampiyonlar Ligi</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>3226062</t>
+          <t>3230467</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1.08</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>6.25</t>
+          <t>4.97</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>9.72</t>
+          <t>7.05</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -1875,49 +1875,49 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Urawa Red</t>
+          <t>Bournemouth</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>JEF Utd</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Japonya J1 Lig</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>3225660</t>
+          <t>3230902</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1.33</t>
+          <t>1.80</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>3.97</t>
+          <t>3.27</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>5.49</t>
+          <t>3.09</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
@@ -1969,17 +1969,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Reading</t>
+          <t>Celtic</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Leyton Orient</t>
+          <t>Celta Vigo</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1989,29 +1989,29 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>İngiltere 1. Lig</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3225707</t>
+          <t>3230592</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>1.33</t>
+          <t>2.43</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>3.76</t>
+          <t>3.06</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>4.63</t>
+          <t>2.23</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -2063,49 +2063,49 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sogndal IL</t>
+          <t>J. Bialystok</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Raufoss</t>
+          <t>Anderlecht</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Norveç 1. Lig</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3247689</t>
+          <t>3230886</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>2.70</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>4.29</t>
+          <t>3.15</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>4.88</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -2157,49 +2157,49 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Kreuzlingen</t>
+          <t>Hoffenheim</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bulle</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>İsviçre Yükselme 1. Lig</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3288451</t>
+          <t>3230445</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2.19</t>
+          <t>1.86</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>3.31</t>
+          <t>3.50</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2.11</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
@@ -2251,143 +2251,303 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bellinzona</t>
+          <t>NK Celje</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Brühl</t>
+          <t>Salzburg</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>İsviçre Yükselme 1. Lig</t>
+          <t>Avrupa Ligi</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>3288461</t>
+          <t>3230023</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2.72</t>
+          <t>5.24</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3.11</t>
+          <t>4.02</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1.84</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
+          <t>1.34</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>1.79</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
       <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>5.47</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>2.52</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1.96</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>13.00</t>
+        </is>
+      </c>
       <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>4.27</t>
+        </is>
+      </c>
       <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
-      <c r="AA16" t="inlineStr"/>
-      <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="inlineStr"/>
-      <c r="AD16" t="inlineStr"/>
-      <c r="AE16" t="inlineStr"/>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>2.06</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>1.35</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>2.24</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>4.03</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>3.98</t>
+        </is>
+      </c>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>12.80</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>6.64</t>
+        </is>
+      </c>
       <c r="AF16" t="inlineStr"/>
       <c r="AG16" t="inlineStr"/>
-      <c r="AH16" t="inlineStr"/>
-      <c r="AI16" t="inlineStr"/>
-      <c r="AJ16" t="inlineStr"/>
-      <c r="AK16" t="inlineStr"/>
-      <c r="AL16" t="inlineStr"/>
-      <c r="AM16" t="inlineStr"/>
-      <c r="AN16" t="inlineStr"/>
-      <c r="AO16" t="inlineStr"/>
-      <c r="AP16" t="inlineStr"/>
-      <c r="AQ16" t="inlineStr"/>
-      <c r="AR16" t="inlineStr"/>
-      <c r="AS16" t="inlineStr"/>
-      <c r="AT16" t="inlineStr"/>
-      <c r="AU16" t="inlineStr"/>
-      <c r="AV16" t="inlineStr"/>
-      <c r="AW16" t="inlineStr"/>
-      <c r="AX16" t="inlineStr"/>
-      <c r="AY16" t="inlineStr"/>
-      <c r="AZ16" t="inlineStr"/>
-      <c r="BA16" t="inlineStr"/>
-      <c r="BB16" t="inlineStr"/>
-      <c r="BC16" t="inlineStr"/>
-      <c r="BD16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>2.01</t>
+        </is>
+      </c>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>3.48</t>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>1.34</t>
+        </is>
+      </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>2.06</t>
+        </is>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>9.40</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>17.50</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>21.00</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>12.00</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>6.50</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>4.36</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>34.70</t>
+        </is>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>15.55</t>
+        </is>
+      </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>2.08</t>
+        </is>
+      </c>
+      <c r="AW16" t="inlineStr">
+        <is>
+          <t>4.27</t>
+        </is>
+      </c>
+      <c r="AX16" t="inlineStr">
+        <is>
+          <t>1.87</t>
+        </is>
+      </c>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>2.89</t>
+        </is>
+      </c>
+      <c r="AZ16" t="inlineStr">
+        <is>
+          <t>8.47</t>
+        </is>
+      </c>
+      <c r="BA16" t="inlineStr">
+        <is>
+          <t>3.26</t>
+        </is>
+      </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>9.63</t>
+        </is>
+      </c>
+      <c r="BC16" t="inlineStr">
+        <is>
+          <t>1.55</t>
+        </is>
+      </c>
+      <c r="BD16" t="inlineStr">
+        <is>
+          <t>2.33</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PK-35</t>
+          <t>Lilleström</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Jaro</t>
+          <t>R. Sociedad</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Finlandiya Veikkausliiga - Küme Düşme Turu</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>3326010</t>
+          <t>3230017</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2.84</t>
+          <t>5.59</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2.71</t>
+          <t>4.30</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2.14</t>
+          <t>1.29</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
@@ -2439,96 +2599,2526 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Terrassa</t>
+          <t>Olympiakos</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Girona II</t>
+          <t>Sparta Prag</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>21.10.2026</t>
+          <t>22.10.2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>İspanya Segunda Lig RFEF</t>
+          <t>Avrupa Ligi</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>3307347</t>
+          <t>3229901</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1.47</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>3.18</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>4.17</t>
+          <t>5.67</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>1.77</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>1.99</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>2.42</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>5.80</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>11.45</t>
+        </is>
+      </c>
       <c r="S18" t="inlineStr"/>
-      <c r="T18" t="inlineStr"/>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>3.66</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>1.84</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>1.55</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>1.25</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>2.57</t>
+        </is>
+      </c>
       <c r="Z18" t="inlineStr"/>
-      <c r="AA18" t="inlineStr"/>
-      <c r="AB18" t="inlineStr"/>
-      <c r="AC18" t="inlineStr"/>
-      <c r="AD18" t="inlineStr"/>
-      <c r="AE18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>4.88</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>4.25</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>1.68</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>2.06</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>3.26</t>
+        </is>
+      </c>
       <c r="AF18" t="inlineStr"/>
       <c r="AG18" t="inlineStr"/>
-      <c r="AH18" t="inlineStr"/>
-      <c r="AI18" t="inlineStr"/>
-      <c r="AJ18" t="inlineStr"/>
-      <c r="AK18" t="inlineStr"/>
-      <c r="AL18" t="inlineStr"/>
-      <c r="AM18" t="inlineStr"/>
-      <c r="AN18" t="inlineStr"/>
-      <c r="AO18" t="inlineStr"/>
-      <c r="AP18" t="inlineStr"/>
-      <c r="AQ18" t="inlineStr"/>
-      <c r="AR18" t="inlineStr"/>
-      <c r="AS18" t="inlineStr"/>
-      <c r="AT18" t="inlineStr"/>
-      <c r="AU18" t="inlineStr"/>
-      <c r="AV18" t="inlineStr"/>
-      <c r="AW18" t="inlineStr"/>
-      <c r="AX18" t="inlineStr"/>
-      <c r="AY18" t="inlineStr"/>
-      <c r="AZ18" t="inlineStr"/>
-      <c r="BA18" t="inlineStr"/>
-      <c r="BB18" t="inlineStr"/>
-      <c r="BC18" t="inlineStr"/>
-      <c r="BD18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr">
+        <is>
+          <t>6.63</t>
+        </is>
+      </c>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>14.20</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>1.37</t>
+        </is>
+      </c>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>2.46</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>16.35</t>
+        </is>
+      </c>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>34.70</t>
+        </is>
+      </c>
+      <c r="AQ18" t="inlineStr">
+        <is>
+          <t>4.19</t>
+        </is>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>6.06</t>
+        </is>
+      </c>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>12.00</t>
+        </is>
+      </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t>22.30</t>
+        </is>
+      </c>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>18.50</t>
+        </is>
+      </c>
+      <c r="AV18" t="inlineStr">
+        <is>
+          <t>9.96</t>
+        </is>
+      </c>
+      <c r="AW18" t="inlineStr">
+        <is>
+          <t>3.62</t>
+        </is>
+      </c>
+      <c r="AX18" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="AZ18" t="inlineStr">
+        <is>
+          <t>11.10</t>
+        </is>
+      </c>
+      <c r="BA18" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="BB18" t="inlineStr">
+        <is>
+          <t>2.76</t>
+        </is>
+      </c>
+      <c r="BC18" t="inlineStr">
+        <is>
+          <t>4.00</t>
+        </is>
+      </c>
+      <c r="BD18" t="inlineStr">
+        <is>
+          <t>12.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Viktoria Plzen</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Levski Sofya</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Avrupa Avrupa Ligi</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>3230355</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>3.48</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>4.06</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr"/>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="inlineStr"/>
+      <c r="AG19" t="inlineStr"/>
+      <c r="AH19" t="inlineStr"/>
+      <c r="AI19" t="inlineStr"/>
+      <c r="AJ19" t="inlineStr"/>
+      <c r="AK19" t="inlineStr"/>
+      <c r="AL19" t="inlineStr"/>
+      <c r="AM19" t="inlineStr"/>
+      <c r="AN19" t="inlineStr"/>
+      <c r="AO19" t="inlineStr"/>
+      <c r="AP19" t="inlineStr"/>
+      <c r="AQ19" t="inlineStr"/>
+      <c r="AR19" t="inlineStr"/>
+      <c r="AS19" t="inlineStr"/>
+      <c r="AT19" t="inlineStr"/>
+      <c r="AU19" t="inlineStr"/>
+      <c r="AV19" t="inlineStr"/>
+      <c r="AW19" t="inlineStr"/>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr"/>
+      <c r="AZ19" t="inlineStr"/>
+      <c r="BA19" t="inlineStr"/>
+      <c r="BB19" t="inlineStr"/>
+      <c r="BC19" t="inlineStr"/>
+      <c r="BD19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Omonia</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Benfica</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Avrupa Avrupa Ligi</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>3230048</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>7.62</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>5.03</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>1.16</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
+      <c r="AD20" t="inlineStr"/>
+      <c r="AE20" t="inlineStr"/>
+      <c r="AF20" t="inlineStr"/>
+      <c r="AG20" t="inlineStr"/>
+      <c r="AH20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr"/>
+      <c r="AJ20" t="inlineStr"/>
+      <c r="AK20" t="inlineStr"/>
+      <c r="AL20" t="inlineStr"/>
+      <c r="AM20" t="inlineStr"/>
+      <c r="AN20" t="inlineStr"/>
+      <c r="AO20" t="inlineStr"/>
+      <c r="AP20" t="inlineStr"/>
+      <c r="AQ20" t="inlineStr"/>
+      <c r="AR20" t="inlineStr"/>
+      <c r="AS20" t="inlineStr"/>
+      <c r="AT20" t="inlineStr"/>
+      <c r="AU20" t="inlineStr"/>
+      <c r="AV20" t="inlineStr"/>
+      <c r="AW20" t="inlineStr"/>
+      <c r="AX20" t="inlineStr"/>
+      <c r="AY20" t="inlineStr"/>
+      <c r="AZ20" t="inlineStr"/>
+      <c r="BA20" t="inlineStr"/>
+      <c r="BB20" t="inlineStr"/>
+      <c r="BC20" t="inlineStr"/>
+      <c r="BD20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>K. Almaty</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Panathinaikos</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Avrupa Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>3229994</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>4.50</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>3.59</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr"/>
+      <c r="AG21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
+      <c r="AJ21" t="inlineStr"/>
+      <c r="AK21" t="inlineStr"/>
+      <c r="AL21" t="inlineStr"/>
+      <c r="AM21" t="inlineStr"/>
+      <c r="AN21" t="inlineStr"/>
+      <c r="AO21" t="inlineStr"/>
+      <c r="AP21" t="inlineStr"/>
+      <c r="AQ21" t="inlineStr"/>
+      <c r="AR21" t="inlineStr"/>
+      <c r="AS21" t="inlineStr"/>
+      <c r="AT21" t="inlineStr"/>
+      <c r="AU21" t="inlineStr"/>
+      <c r="AV21" t="inlineStr"/>
+      <c r="AW21" t="inlineStr"/>
+      <c r="AX21" t="inlineStr"/>
+      <c r="AY21" t="inlineStr"/>
+      <c r="AZ21" t="inlineStr"/>
+      <c r="BA21" t="inlineStr"/>
+      <c r="BB21" t="inlineStr"/>
+      <c r="BC21" t="inlineStr"/>
+      <c r="BD21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Getafe</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Lugano</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Avrupa Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>3230882</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>1.74</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2.98</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>3.57</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
+      <c r="AD22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr"/>
+      <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
+      <c r="AJ22" t="inlineStr"/>
+      <c r="AK22" t="inlineStr"/>
+      <c r="AL22" t="inlineStr"/>
+      <c r="AM22" t="inlineStr"/>
+      <c r="AN22" t="inlineStr"/>
+      <c r="AO22" t="inlineStr"/>
+      <c r="AP22" t="inlineStr"/>
+      <c r="AQ22" t="inlineStr"/>
+      <c r="AR22" t="inlineStr"/>
+      <c r="AS22" t="inlineStr"/>
+      <c r="AT22" t="inlineStr"/>
+      <c r="AU22" t="inlineStr"/>
+      <c r="AV22" t="inlineStr"/>
+      <c r="AW22" t="inlineStr"/>
+      <c r="AX22" t="inlineStr"/>
+      <c r="AY22" t="inlineStr"/>
+      <c r="AZ22" t="inlineStr"/>
+      <c r="BA22" t="inlineStr"/>
+      <c r="BB22" t="inlineStr"/>
+      <c r="BC22" t="inlineStr"/>
+      <c r="BD22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Iberia</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Mjallby</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Avrupa Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>3230000</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2.59</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>3.04</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2.12</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
+      <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="inlineStr"/>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr"/>
+      <c r="AG23" t="inlineStr"/>
+      <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr"/>
+      <c r="AJ23" t="inlineStr"/>
+      <c r="AK23" t="inlineStr"/>
+      <c r="AL23" t="inlineStr"/>
+      <c r="AM23" t="inlineStr"/>
+      <c r="AN23" t="inlineStr"/>
+      <c r="AO23" t="inlineStr"/>
+      <c r="AP23" t="inlineStr"/>
+      <c r="AQ23" t="inlineStr"/>
+      <c r="AR23" t="inlineStr"/>
+      <c r="AS23" t="inlineStr"/>
+      <c r="AT23" t="inlineStr"/>
+      <c r="AU23" t="inlineStr"/>
+      <c r="AV23" t="inlineStr"/>
+      <c r="AW23" t="inlineStr"/>
+      <c r="AX23" t="inlineStr"/>
+      <c r="AY23" t="inlineStr"/>
+      <c r="AZ23" t="inlineStr"/>
+      <c r="BA23" t="inlineStr"/>
+      <c r="BB23" t="inlineStr"/>
+      <c r="BC23" t="inlineStr"/>
+      <c r="BD23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Inter Escaldes</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Univ. Craiova</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Avrupa Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>3230170</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>5.01</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>3.63</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>1.41</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
+      <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr"/>
+      <c r="AG24" t="inlineStr"/>
+      <c r="AH24" t="inlineStr"/>
+      <c r="AI24" t="inlineStr"/>
+      <c r="AJ24" t="inlineStr"/>
+      <c r="AK24" t="inlineStr"/>
+      <c r="AL24" t="inlineStr"/>
+      <c r="AM24" t="inlineStr"/>
+      <c r="AN24" t="inlineStr"/>
+      <c r="AO24" t="inlineStr"/>
+      <c r="AP24" t="inlineStr"/>
+      <c r="AQ24" t="inlineStr"/>
+      <c r="AR24" t="inlineStr"/>
+      <c r="AS24" t="inlineStr"/>
+      <c r="AT24" t="inlineStr"/>
+      <c r="AU24" t="inlineStr"/>
+      <c r="AV24" t="inlineStr"/>
+      <c r="AW24" t="inlineStr"/>
+      <c r="AX24" t="inlineStr"/>
+      <c r="AY24" t="inlineStr"/>
+      <c r="AZ24" t="inlineStr"/>
+      <c r="BA24" t="inlineStr"/>
+      <c r="BB24" t="inlineStr"/>
+      <c r="BC24" t="inlineStr"/>
+      <c r="BD24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Kauno Zalgiris</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Brann</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Avrupa Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>3229861</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>4.05</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>3.55</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>1.52</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
+      <c r="AD25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr"/>
+      <c r="AF25" t="inlineStr"/>
+      <c r="AG25" t="inlineStr"/>
+      <c r="AH25" t="inlineStr"/>
+      <c r="AI25" t="inlineStr"/>
+      <c r="AJ25" t="inlineStr"/>
+      <c r="AK25" t="inlineStr"/>
+      <c r="AL25" t="inlineStr"/>
+      <c r="AM25" t="inlineStr"/>
+      <c r="AN25" t="inlineStr"/>
+      <c r="AO25" t="inlineStr"/>
+      <c r="AP25" t="inlineStr"/>
+      <c r="AQ25" t="inlineStr"/>
+      <c r="AR25" t="inlineStr"/>
+      <c r="AS25" t="inlineStr"/>
+      <c r="AT25" t="inlineStr"/>
+      <c r="AU25" t="inlineStr"/>
+      <c r="AV25" t="inlineStr"/>
+      <c r="AW25" t="inlineStr"/>
+      <c r="AX25" t="inlineStr"/>
+      <c r="AY25" t="inlineStr"/>
+      <c r="AZ25" t="inlineStr"/>
+      <c r="BA25" t="inlineStr"/>
+      <c r="BB25" t="inlineStr"/>
+      <c r="BC25" t="inlineStr"/>
+      <c r="BD25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Kızılyıldız</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Kopenhag</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Avrupa Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>3230408</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>3.21</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>2.67</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
+      <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr"/>
+      <c r="AG26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr"/>
+      <c r="AI26" t="inlineStr"/>
+      <c r="AJ26" t="inlineStr"/>
+      <c r="AK26" t="inlineStr"/>
+      <c r="AL26" t="inlineStr"/>
+      <c r="AM26" t="inlineStr"/>
+      <c r="AN26" t="inlineStr"/>
+      <c r="AO26" t="inlineStr"/>
+      <c r="AP26" t="inlineStr"/>
+      <c r="AQ26" t="inlineStr"/>
+      <c r="AR26" t="inlineStr"/>
+      <c r="AS26" t="inlineStr"/>
+      <c r="AT26" t="inlineStr"/>
+      <c r="AU26" t="inlineStr"/>
+      <c r="AV26" t="inlineStr"/>
+      <c r="AW26" t="inlineStr"/>
+      <c r="AX26" t="inlineStr"/>
+      <c r="AY26" t="inlineStr"/>
+      <c r="AZ26" t="inlineStr"/>
+      <c r="BA26" t="inlineStr"/>
+      <c r="BB26" t="inlineStr"/>
+      <c r="BC26" t="inlineStr"/>
+      <c r="BD26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Nordsjaelland</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CSKA Sofya</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Avrupa Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>3230599</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>4.44</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>5.90</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
+      <c r="AC27" t="inlineStr"/>
+      <c r="AD27" t="inlineStr"/>
+      <c r="AE27" t="inlineStr"/>
+      <c r="AF27" t="inlineStr"/>
+      <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="inlineStr"/>
+      <c r="AI27" t="inlineStr"/>
+      <c r="AJ27" t="inlineStr"/>
+      <c r="AK27" t="inlineStr"/>
+      <c r="AL27" t="inlineStr"/>
+      <c r="AM27" t="inlineStr"/>
+      <c r="AN27" t="inlineStr"/>
+      <c r="AO27" t="inlineStr"/>
+      <c r="AP27" t="inlineStr"/>
+      <c r="AQ27" t="inlineStr"/>
+      <c r="AR27" t="inlineStr"/>
+      <c r="AS27" t="inlineStr"/>
+      <c r="AT27" t="inlineStr"/>
+      <c r="AU27" t="inlineStr"/>
+      <c r="AV27" t="inlineStr"/>
+      <c r="AW27" t="inlineStr"/>
+      <c r="AX27" t="inlineStr"/>
+      <c r="AY27" t="inlineStr"/>
+      <c r="AZ27" t="inlineStr"/>
+      <c r="BA27" t="inlineStr"/>
+      <c r="BB27" t="inlineStr"/>
+      <c r="BC27" t="inlineStr"/>
+      <c r="BD27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Pafos</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Riga</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>3230826</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>3.70</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>4.63</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>1.36</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>1.49</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>2.38</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>5.13</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>11.45</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>3.90</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>1.29</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>1.85</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr">
+        <is>
+          <t>2.74</t>
+        </is>
+      </c>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>4.81</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>4.04</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>3.31</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr"/>
+      <c r="AG28" t="inlineStr"/>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>6.06</t>
+        </is>
+      </c>
+      <c r="AI28" t="inlineStr">
+        <is>
+          <t>11.50</t>
+        </is>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>2.97</t>
+        </is>
+      </c>
+      <c r="AK28" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="AL28" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="AM28" t="inlineStr">
+        <is>
+          <t>2.46</t>
+        </is>
+      </c>
+      <c r="AN28" t="inlineStr">
+        <is>
+          <t>2.26</t>
+        </is>
+      </c>
+      <c r="AO28" t="inlineStr">
+        <is>
+          <t>15.10</t>
+        </is>
+      </c>
+      <c r="AP28" t="inlineStr">
+        <is>
+          <t>34.70</t>
+        </is>
+      </c>
+      <c r="AQ28" t="inlineStr">
+        <is>
+          <t>4.37</t>
+        </is>
+      </c>
+      <c r="AR28" t="inlineStr">
+        <is>
+          <t>5.83</t>
+        </is>
+      </c>
+      <c r="AS28" t="inlineStr">
+        <is>
+          <t>10.50</t>
+        </is>
+      </c>
+      <c r="AT28" t="inlineStr">
+        <is>
+          <t>22.30</t>
+        </is>
+      </c>
+      <c r="AU28" t="inlineStr">
+        <is>
+          <t>16.80</t>
+        </is>
+      </c>
+      <c r="AV28" t="inlineStr">
+        <is>
+          <t>8.35</t>
+        </is>
+      </c>
+      <c r="AW28" t="inlineStr">
+        <is>
+          <t>3.86</t>
+        </is>
+      </c>
+      <c r="AX28" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="AY28" t="inlineStr">
+        <is>
+          <t>3.38</t>
+        </is>
+      </c>
+      <c r="AZ28" t="inlineStr">
+        <is>
+          <t>11.10</t>
+        </is>
+      </c>
+      <c r="BA28" t="inlineStr">
+        <is>
+          <t>1.68</t>
+        </is>
+      </c>
+      <c r="BB28" t="inlineStr">
+        <is>
+          <t>2.74</t>
+        </is>
+      </c>
+      <c r="BC28" t="inlineStr">
+        <is>
+          <t>3.31</t>
+        </is>
+      </c>
+      <c r="BD28" t="inlineStr">
+        <is>
+          <t>10.05</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Ajax</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>3230404</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>1.84</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>3.39</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>2.86</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>1.35</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>2.28</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>3.23</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>5.45</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>2.38</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr">
+        <is>
+          <t>1.30</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>1.71</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="Z29" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>3.27</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>2.99</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>3.28</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>4.08</t>
+        </is>
+      </c>
+      <c r="AF29" t="inlineStr"/>
+      <c r="AG29" t="inlineStr"/>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>4.77</t>
+        </is>
+      </c>
+      <c r="AI29" t="inlineStr">
+        <is>
+          <t>5.56</t>
+        </is>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>3.77</t>
+        </is>
+      </c>
+      <c r="AK29" t="inlineStr">
+        <is>
+          <t>1.30</t>
+        </is>
+      </c>
+      <c r="AL29" t="inlineStr">
+        <is>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="AM29" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="AN29" t="inlineStr">
+        <is>
+          <t>2.76</t>
+        </is>
+      </c>
+      <c r="AO29" t="inlineStr">
+        <is>
+          <t>12.05</t>
+        </is>
+      </c>
+      <c r="AP29" t="inlineStr">
+        <is>
+          <t>28.00</t>
+        </is>
+      </c>
+      <c r="AQ29" t="inlineStr">
+        <is>
+          <t>5.38</t>
+        </is>
+      </c>
+      <c r="AR29" t="inlineStr">
+        <is>
+          <t>5.91</t>
+        </is>
+      </c>
+      <c r="AS29" t="inlineStr">
+        <is>
+          <t>7.50</t>
+        </is>
+      </c>
+      <c r="AT29" t="inlineStr">
+        <is>
+          <t>21.05</t>
+        </is>
+      </c>
+      <c r="AU29" t="inlineStr">
+        <is>
+          <t>12.60</t>
+        </is>
+      </c>
+      <c r="AV29" t="inlineStr">
+        <is>
+          <t>4.61</t>
+        </is>
+      </c>
+      <c r="AW29" t="inlineStr">
+        <is>
+          <t>5.53</t>
+        </is>
+      </c>
+      <c r="AX29" t="inlineStr">
+        <is>
+          <t>2.20</t>
+        </is>
+      </c>
+      <c r="AY29" t="inlineStr">
+        <is>
+          <t>2.81</t>
+        </is>
+      </c>
+      <c r="AZ29" t="inlineStr">
+        <is>
+          <t>6.41</t>
+        </is>
+      </c>
+      <c r="BA29" t="inlineStr">
+        <is>
+          <t>1.70</t>
+        </is>
+      </c>
+      <c r="BB29" t="inlineStr">
+        <is>
+          <t>3.03</t>
+        </is>
+      </c>
+      <c r="BC29" t="inlineStr">
+        <is>
+          <t>2.12</t>
+        </is>
+      </c>
+      <c r="BD29" t="inlineStr">
+        <is>
+          <t>4.31</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Aarhus</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Egnatia</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Avrupa Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>3229986</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>1.30</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>5.71</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr"/>
+      <c r="AD30" t="inlineStr"/>
+      <c r="AE30" t="inlineStr"/>
+      <c r="AF30" t="inlineStr"/>
+      <c r="AG30" t="inlineStr"/>
+      <c r="AH30" t="inlineStr"/>
+      <c r="AI30" t="inlineStr"/>
+      <c r="AJ30" t="inlineStr"/>
+      <c r="AK30" t="inlineStr"/>
+      <c r="AL30" t="inlineStr"/>
+      <c r="AM30" t="inlineStr"/>
+      <c r="AN30" t="inlineStr"/>
+      <c r="AO30" t="inlineStr"/>
+      <c r="AP30" t="inlineStr"/>
+      <c r="AQ30" t="inlineStr"/>
+      <c r="AR30" t="inlineStr"/>
+      <c r="AS30" t="inlineStr"/>
+      <c r="AT30" t="inlineStr"/>
+      <c r="AU30" t="inlineStr"/>
+      <c r="AV30" t="inlineStr"/>
+      <c r="AW30" t="inlineStr"/>
+      <c r="AX30" t="inlineStr"/>
+      <c r="AY30" t="inlineStr"/>
+      <c r="AZ30" t="inlineStr"/>
+      <c r="BA30" t="inlineStr"/>
+      <c r="BB30" t="inlineStr"/>
+      <c r="BC30" t="inlineStr"/>
+      <c r="BD30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Banja Luka</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Kuopion</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Avrupa Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>3230236</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>1.61</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>3.84</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr"/>
+      <c r="AD31" t="inlineStr"/>
+      <c r="AE31" t="inlineStr"/>
+      <c r="AF31" t="inlineStr"/>
+      <c r="AG31" t="inlineStr"/>
+      <c r="AH31" t="inlineStr"/>
+      <c r="AI31" t="inlineStr"/>
+      <c r="AJ31" t="inlineStr"/>
+      <c r="AK31" t="inlineStr"/>
+      <c r="AL31" t="inlineStr"/>
+      <c r="AM31" t="inlineStr"/>
+      <c r="AN31" t="inlineStr"/>
+      <c r="AO31" t="inlineStr"/>
+      <c r="AP31" t="inlineStr"/>
+      <c r="AQ31" t="inlineStr"/>
+      <c r="AR31" t="inlineStr"/>
+      <c r="AS31" t="inlineStr"/>
+      <c r="AT31" t="inlineStr"/>
+      <c r="AU31" t="inlineStr"/>
+      <c r="AV31" t="inlineStr"/>
+      <c r="AW31" t="inlineStr"/>
+      <c r="AX31" t="inlineStr"/>
+      <c r="AY31" t="inlineStr"/>
+      <c r="AZ31" t="inlineStr"/>
+      <c r="BA31" t="inlineStr"/>
+      <c r="BB31" t="inlineStr"/>
+      <c r="BC31" t="inlineStr"/>
+      <c r="BD31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>KAA Gent</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Avrupa Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>3229972</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>1.68</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>3.13</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>3.65</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr"/>
+      <c r="AD32" t="inlineStr"/>
+      <c r="AE32" t="inlineStr"/>
+      <c r="AF32" t="inlineStr"/>
+      <c r="AG32" t="inlineStr"/>
+      <c r="AH32" t="inlineStr"/>
+      <c r="AI32" t="inlineStr"/>
+      <c r="AJ32" t="inlineStr"/>
+      <c r="AK32" t="inlineStr"/>
+      <c r="AL32" t="inlineStr"/>
+      <c r="AM32" t="inlineStr"/>
+      <c r="AN32" t="inlineStr"/>
+      <c r="AO32" t="inlineStr"/>
+      <c r="AP32" t="inlineStr"/>
+      <c r="AQ32" t="inlineStr"/>
+      <c r="AR32" t="inlineStr"/>
+      <c r="AS32" t="inlineStr"/>
+      <c r="AT32" t="inlineStr"/>
+      <c r="AU32" t="inlineStr"/>
+      <c r="AV32" t="inlineStr"/>
+      <c r="AW32" t="inlineStr"/>
+      <c r="AX32" t="inlineStr"/>
+      <c r="AY32" t="inlineStr"/>
+      <c r="AZ32" t="inlineStr"/>
+      <c r="BA32" t="inlineStr"/>
+      <c r="BB32" t="inlineStr"/>
+      <c r="BC32" t="inlineStr"/>
+      <c r="BD32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Midtjylland</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>St. Truidense</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Avrupa Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>3230890</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>3.64</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>4.20</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr"/>
+      <c r="AD33" t="inlineStr"/>
+      <c r="AE33" t="inlineStr"/>
+      <c r="AF33" t="inlineStr"/>
+      <c r="AG33" t="inlineStr"/>
+      <c r="AH33" t="inlineStr"/>
+      <c r="AI33" t="inlineStr"/>
+      <c r="AJ33" t="inlineStr"/>
+      <c r="AK33" t="inlineStr"/>
+      <c r="AL33" t="inlineStr"/>
+      <c r="AM33" t="inlineStr"/>
+      <c r="AN33" t="inlineStr"/>
+      <c r="AO33" t="inlineStr"/>
+      <c r="AP33" t="inlineStr"/>
+      <c r="AQ33" t="inlineStr"/>
+      <c r="AR33" t="inlineStr"/>
+      <c r="AS33" t="inlineStr"/>
+      <c r="AT33" t="inlineStr"/>
+      <c r="AU33" t="inlineStr"/>
+      <c r="AV33" t="inlineStr"/>
+      <c r="AW33" t="inlineStr"/>
+      <c r="AX33" t="inlineStr"/>
+      <c r="AY33" t="inlineStr"/>
+      <c r="AZ33" t="inlineStr"/>
+      <c r="BA33" t="inlineStr"/>
+      <c r="BB33" t="inlineStr"/>
+      <c r="BC33" t="inlineStr"/>
+      <c r="BD33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Freiburg</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>3230640</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>1.94</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>2.78</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>1.40</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>2.46</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>3.29</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>11.75</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>3.93</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>1.08</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>2.12</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr">
+        <is>
+          <t>1.70</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>1.49</t>
+        </is>
+      </c>
+      <c r="Y34" t="inlineStr">
+        <is>
+          <t>2.60</t>
+        </is>
+      </c>
+      <c r="Z34" t="inlineStr"/>
+      <c r="AA34" t="inlineStr">
+        <is>
+          <t>4.71</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>3.55</t>
+        </is>
+      </c>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr">
+        <is>
+          <t>3.48</t>
+        </is>
+      </c>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>3.73</t>
+        </is>
+      </c>
+      <c r="AF34" t="inlineStr"/>
+      <c r="AG34" t="inlineStr"/>
+      <c r="AH34" t="inlineStr">
+        <is>
+          <t>4.45</t>
+        </is>
+      </c>
+      <c r="AI34" t="inlineStr">
+        <is>
+          <t>5.70</t>
+        </is>
+      </c>
+      <c r="AJ34" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="AK34" t="inlineStr">
+        <is>
+          <t>1.37</t>
+        </is>
+      </c>
+      <c r="AL34" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="AM34" t="inlineStr">
+        <is>
+          <t>2.41</t>
+        </is>
+      </c>
+      <c r="AN34" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="AO34" t="inlineStr">
+        <is>
+          <t>12.80</t>
+        </is>
+      </c>
+      <c r="AP34" t="inlineStr">
+        <is>
+          <t>30.20</t>
+        </is>
+      </c>
+      <c r="AQ34" t="inlineStr">
+        <is>
+          <t>5.43</t>
+        </is>
+      </c>
+      <c r="AR34" t="inlineStr">
+        <is>
+          <t>5.35</t>
+        </is>
+      </c>
+      <c r="AS34" t="inlineStr">
+        <is>
+          <t>7.06</t>
+        </is>
+      </c>
+      <c r="AT34" t="inlineStr">
+        <is>
+          <t>24.05</t>
+        </is>
+      </c>
+      <c r="AU34" t="inlineStr">
+        <is>
+          <t>13.25</t>
+        </is>
+      </c>
+      <c r="AV34" t="inlineStr">
+        <is>
+          <t>4.78</t>
+        </is>
+      </c>
+      <c r="AW34" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+      <c r="AX34" t="inlineStr">
+        <is>
+          <t>2.03</t>
+        </is>
+      </c>
+      <c r="AY34" t="inlineStr">
+        <is>
+          <t>3.24</t>
+        </is>
+      </c>
+      <c r="AZ34" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="BA34" t="inlineStr">
+        <is>
+          <t>1.94</t>
+        </is>
+      </c>
+      <c r="BB34" t="inlineStr">
+        <is>
+          <t>3.84</t>
+        </is>
+      </c>
+      <c r="BC34" t="inlineStr">
+        <is>
+          <t>2.19</t>
+        </is>
+      </c>
+      <c r="BD34" t="inlineStr">
+        <is>
+          <t>5.52</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Thun</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Hajduk Split</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Avrupa Konferans Ligi</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>3230065</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2.56</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>2.06</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr"/>
+      <c r="W35" t="inlineStr"/>
+      <c r="X35" t="inlineStr"/>
+      <c r="Y35" t="inlineStr"/>
+      <c r="Z35" t="inlineStr"/>
+      <c r="AA35" t="inlineStr"/>
+      <c r="AB35" t="inlineStr"/>
+      <c r="AC35" t="inlineStr"/>
+      <c r="AD35" t="inlineStr"/>
+      <c r="AE35" t="inlineStr"/>
+      <c r="AF35" t="inlineStr"/>
+      <c r="AG35" t="inlineStr"/>
+      <c r="AH35" t="inlineStr"/>
+      <c r="AI35" t="inlineStr"/>
+      <c r="AJ35" t="inlineStr"/>
+      <c r="AK35" t="inlineStr"/>
+      <c r="AL35" t="inlineStr"/>
+      <c r="AM35" t="inlineStr"/>
+      <c r="AN35" t="inlineStr"/>
+      <c r="AO35" t="inlineStr"/>
+      <c r="AP35" t="inlineStr"/>
+      <c r="AQ35" t="inlineStr"/>
+      <c r="AR35" t="inlineStr"/>
+      <c r="AS35" t="inlineStr"/>
+      <c r="AT35" t="inlineStr"/>
+      <c r="AU35" t="inlineStr"/>
+      <c r="AV35" t="inlineStr"/>
+      <c r="AW35" t="inlineStr"/>
+      <c r="AX35" t="inlineStr"/>
+      <c r="AY35" t="inlineStr"/>
+      <c r="AZ35" t="inlineStr"/>
+      <c r="BA35" t="inlineStr"/>
+      <c r="BB35" t="inlineStr"/>
+      <c r="BC35" t="inlineStr"/>
+      <c r="BD35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>FC Bihor</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Reşita</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Romanya 2. Lig</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>3235235</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>1.82</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2.99</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>2.85</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr"/>
+      <c r="W36" t="inlineStr"/>
+      <c r="X36" t="inlineStr"/>
+      <c r="Y36" t="inlineStr"/>
+      <c r="Z36" t="inlineStr"/>
+      <c r="AA36" t="inlineStr"/>
+      <c r="AB36" t="inlineStr"/>
+      <c r="AC36" t="inlineStr"/>
+      <c r="AD36" t="inlineStr"/>
+      <c r="AE36" t="inlineStr"/>
+      <c r="AF36" t="inlineStr"/>
+      <c r="AG36" t="inlineStr"/>
+      <c r="AH36" t="inlineStr"/>
+      <c r="AI36" t="inlineStr"/>
+      <c r="AJ36" t="inlineStr"/>
+      <c r="AK36" t="inlineStr"/>
+      <c r="AL36" t="inlineStr"/>
+      <c r="AM36" t="inlineStr"/>
+      <c r="AN36" t="inlineStr"/>
+      <c r="AO36" t="inlineStr"/>
+      <c r="AP36" t="inlineStr"/>
+      <c r="AQ36" t="inlineStr"/>
+      <c r="AR36" t="inlineStr"/>
+      <c r="AS36" t="inlineStr"/>
+      <c r="AT36" t="inlineStr"/>
+      <c r="AU36" t="inlineStr"/>
+      <c r="AV36" t="inlineStr"/>
+      <c r="AW36" t="inlineStr"/>
+      <c r="AX36" t="inlineStr"/>
+      <c r="AY36" t="inlineStr"/>
+      <c r="AZ36" t="inlineStr"/>
+      <c r="BA36" t="inlineStr"/>
+      <c r="BB36" t="inlineStr"/>
+      <c r="BC36" t="inlineStr"/>
+      <c r="BD36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Rovaniemen</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Kapa</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>22.10.2026</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Finlandiya Ykkösliiga Play-out</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>3328665</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2.04</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>3.01</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>2.44</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr"/>
+      <c r="W37" t="inlineStr"/>
+      <c r="X37" t="inlineStr"/>
+      <c r="Y37" t="inlineStr"/>
+      <c r="Z37" t="inlineStr"/>
+      <c r="AA37" t="inlineStr"/>
+      <c r="AB37" t="inlineStr"/>
+      <c r="AC37" t="inlineStr"/>
+      <c r="AD37" t="inlineStr"/>
+      <c r="AE37" t="inlineStr"/>
+      <c r="AF37" t="inlineStr"/>
+      <c r="AG37" t="inlineStr"/>
+      <c r="AH37" t="inlineStr"/>
+      <c r="AI37" t="inlineStr"/>
+      <c r="AJ37" t="inlineStr"/>
+      <c r="AK37" t="inlineStr"/>
+      <c r="AL37" t="inlineStr"/>
+      <c r="AM37" t="inlineStr"/>
+      <c r="AN37" t="inlineStr"/>
+      <c r="AO37" t="inlineStr"/>
+      <c r="AP37" t="inlineStr"/>
+      <c r="AQ37" t="inlineStr"/>
+      <c r="AR37" t="inlineStr"/>
+      <c r="AS37" t="inlineStr"/>
+      <c r="AT37" t="inlineStr"/>
+      <c r="AU37" t="inlineStr"/>
+      <c r="AV37" t="inlineStr"/>
+      <c r="AW37" t="inlineStr"/>
+      <c r="AX37" t="inlineStr"/>
+      <c r="AY37" t="inlineStr"/>
+      <c r="AZ37" t="inlineStr"/>
+      <c r="BA37" t="inlineStr"/>
+      <c r="BB37" t="inlineStr"/>
+      <c r="BC37" t="inlineStr"/>
+      <c r="BD37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
veri: iddaa guncellendi (22.10.2026 12:05)
</commit_message>
<xml_diff>
--- a/iddaa/gunluk/gunlukmaclar.xlsx
+++ b/iddaa/gunluk/gunlukmaclar.xlsx
@@ -791,7 +791,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Avrupa Avrupa Ligi</t>
+          <t>Avrupa Ligi</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -816,61 +816,217 @@
           <t>1.24</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>1.27</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>5.86</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>2.48</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1.63</t>
+        </is>
+      </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>5.06</t>
+        </is>
+      </c>
       <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>2.48</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>1.65</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>2.22</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>1.31</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>3.69</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>3.67</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>15.15</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>7.43</t>
+        </is>
+      </c>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>3.70</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>1.97</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>3.59</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>1.93</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>11.10</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>19.30</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>20.25</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>14.20</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>7.40</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>4.29</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>34.70</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>16.95</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>4.90</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>1.94</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>2.70</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>6.92</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>3.41</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>10.25</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>1.45</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>2.02</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ferencvaros</t>
+          <t>Trabzonspor</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Torreense</t>
+          <t>Hearts</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -885,29 +1041,29 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Avrupa Avrupa Ligi</t>
+          <t>Avrupa Konferans Ligi</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3230269</t>
+          <t>3230845</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>5.07</t>
+          <t>5.87</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>8.43</t>
+          <t>8.63</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -959,12 +1115,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Trabzonspor</t>
+          <t>Beşiktaş</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hearts</t>
+          <t>Crystal Palace</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -974,34 +1130,34 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Avrupa Konferans Ligi</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3230845</t>
+          <t>3229910</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>2.01</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>5.87</t>
+          <t>3.34</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>8.63</t>
+          <t>2.56</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -1053,12 +1209,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>D. Zagreb</t>
+          <t>Ferencvaros</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NEC Nijmegen</t>
+          <t>Torreense</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1078,24 +1234,24 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3230256</t>
+          <t>3230269</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>1.35</t>
+          <t>1.15</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>4.09</t>
+          <t>5.07</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>4.91</t>
+          <t>8.43</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -1147,12 +1303,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Beşiktaş</t>
+          <t>D. Zagreb</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Crystal Palace</t>
+          <t>NEC Nijmegen</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1162,7 +1318,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1172,24 +1328,24 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3229910</t>
+          <t>3230256</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2.01</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>3.34</t>
+          <t>4.09</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.56</t>
+          <t>4.91</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -1241,12 +1397,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lech Poznan</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1266,24 +1422,24 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3229916</t>
+          <t>3230667</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>4.09</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>3.44</t>
+          <t>4.17</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>5.94</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
@@ -1593,12 +1749,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Lech Poznan</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Sunderland</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1618,24 +1774,24 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>3230667</t>
+          <t>3229916</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1.28</t>
+          <t>4.09</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>4.17</t>
+          <t>3.44</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>5.94</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -1895,7 +2051,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Avrupa Avrupa Ligi</t>
+          <t>Avrupa Ligi</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1907,74 +2063,238 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>1.92</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>3.27</t>
+          <t>3.56</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>3.09</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
+          <t>3.46</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>1.29</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>1.60</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>2.24</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>3.76</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>11.70</t>
+        </is>
+      </c>
       <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>3.81</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>1.08</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>1.88</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>1.52</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>2.67</t>
+        </is>
+      </c>
       <c r="Z12" t="inlineStr"/>
-      <c r="AA12" t="inlineStr"/>
-      <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
-      <c r="AD12" t="inlineStr"/>
-      <c r="AE12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>4.65</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>3.70</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>3.15</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>3.71</t>
+        </is>
+      </c>
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr"/>
-      <c r="AH12" t="inlineStr"/>
-      <c r="AI12" t="inlineStr"/>
-      <c r="AJ12" t="inlineStr"/>
-      <c r="AK12" t="inlineStr"/>
-      <c r="AL12" t="inlineStr"/>
-      <c r="AM12" t="inlineStr"/>
-      <c r="AN12" t="inlineStr"/>
-      <c r="AO12" t="inlineStr"/>
-      <c r="AP12" t="inlineStr"/>
-      <c r="AQ12" t="inlineStr"/>
-      <c r="AR12" t="inlineStr"/>
-      <c r="AS12" t="inlineStr"/>
-      <c r="AT12" t="inlineStr"/>
-      <c r="AU12" t="inlineStr"/>
-      <c r="AV12" t="inlineStr"/>
-      <c r="AW12" t="inlineStr"/>
-      <c r="AX12" t="inlineStr"/>
-      <c r="AY12" t="inlineStr"/>
-      <c r="AZ12" t="inlineStr"/>
-      <c r="BA12" t="inlineStr"/>
-      <c r="BB12" t="inlineStr"/>
-      <c r="BC12" t="inlineStr"/>
-      <c r="BD12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>4.83</t>
+        </is>
+      </c>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>7.13</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>2.94</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>2.45</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>2.80</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>13.45</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>34.70</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>4.92</t>
+        </is>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>5.50</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>7.91</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>22.75</t>
+        </is>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>14.35</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>5.73</t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>3.97</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>2.02</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>3.31</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>10.50</t>
+        </is>
+      </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>1.84</t>
+        </is>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>3.48</t>
+        </is>
+      </c>
+      <c r="BC12" t="inlineStr">
+        <is>
+          <t>2.70</t>
+        </is>
+      </c>
+      <c r="BD12" t="inlineStr">
+        <is>
+          <t>6.53</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Celtic</t>
+          <t>NK Celje</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Celta Vigo</t>
+          <t>Salzburg</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1989,86 +2309,246 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Avrupa Avrupa Ligi</t>
+          <t>Avrupa Ligi</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3230592</t>
+          <t>3230023</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2.43</t>
+          <t>5.24</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>3.06</t>
+          <t>4.02</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2.23</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
+          <t>1.34</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1.79</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>5.47</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>2.52</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1.96</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>13.00</t>
+        </is>
+      </c>
       <c r="S13" t="inlineStr"/>
-      <c r="T13" t="inlineStr"/>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>4.27</t>
+        </is>
+      </c>
       <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr"/>
-      <c r="AA13" t="inlineStr"/>
-      <c r="AB13" t="inlineStr"/>
-      <c r="AC13" t="inlineStr"/>
-      <c r="AD13" t="inlineStr"/>
-      <c r="AE13" t="inlineStr"/>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>2.06</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>1.35</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>2.24</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>4.03</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>3.98</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>12.80</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>6.64</t>
+        </is>
+      </c>
       <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr"/>
-      <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr"/>
-      <c r="AJ13" t="inlineStr"/>
-      <c r="AK13" t="inlineStr"/>
-      <c r="AL13" t="inlineStr"/>
-      <c r="AM13" t="inlineStr"/>
-      <c r="AN13" t="inlineStr"/>
-      <c r="AO13" t="inlineStr"/>
-      <c r="AP13" t="inlineStr"/>
-      <c r="AQ13" t="inlineStr"/>
-      <c r="AR13" t="inlineStr"/>
-      <c r="AS13" t="inlineStr"/>
-      <c r="AT13" t="inlineStr"/>
-      <c r="AU13" t="inlineStr"/>
-      <c r="AV13" t="inlineStr"/>
-      <c r="AW13" t="inlineStr"/>
-      <c r="AX13" t="inlineStr"/>
-      <c r="AY13" t="inlineStr"/>
-      <c r="AZ13" t="inlineStr"/>
-      <c r="BA13" t="inlineStr"/>
-      <c r="BB13" t="inlineStr"/>
-      <c r="BC13" t="inlineStr"/>
-      <c r="BD13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>2.01</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>3.48</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>1.34</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>2.06</t>
+        </is>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>9.40</t>
+        </is>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>17.50</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>21.00</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>12.00</t>
+        </is>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>6.50</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>4.36</t>
+        </is>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>34.70</t>
+        </is>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>15.55</t>
+        </is>
+      </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>2.08</t>
+        </is>
+      </c>
+      <c r="AW13" t="inlineStr">
+        <is>
+          <t>4.27</t>
+        </is>
+      </c>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>1.87</t>
+        </is>
+      </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>2.89</t>
+        </is>
+      </c>
+      <c r="AZ13" t="inlineStr">
+        <is>
+          <t>8.47</t>
+        </is>
+      </c>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>3.26</t>
+        </is>
+      </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>9.63</t>
+        </is>
+      </c>
+      <c r="BC13" t="inlineStr">
+        <is>
+          <t>1.55</t>
+        </is>
+      </c>
+      <c r="BD13" t="inlineStr">
+        <is>
+          <t>2.33</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>J. Bialystok</t>
+          <t>Celtic</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Anderlecht</t>
+          <t>Celta Vigo</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2088,24 +2568,24 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3230886</t>
+          <t>3230592</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2.70</t>
+          <t>2.43</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>3.15</t>
+          <t>3.06</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>2.23</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -2251,12 +2731,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>NK Celje</t>
+          <t>J. Bialystok</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Salzburg</t>
+          <t>Anderlecht</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2271,236 +2751,76 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Avrupa Ligi</t>
+          <t>Avrupa Avrupa Ligi</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>3230023</t>
+          <t>3230886</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>5.24</t>
+          <t>2.70</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>4.02</t>
+          <t>3.15</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1.34</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>1.79</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>1.51</t>
-        </is>
-      </c>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>5.47</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>2.52</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>1.96</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>13.00</t>
-        </is>
-      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>4.27</t>
-        </is>
-      </c>
+      <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>2.06</t>
-        </is>
-      </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>1.42</t>
-        </is>
-      </c>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>1.35</t>
-        </is>
-      </c>
-      <c r="Y16" t="inlineStr">
-        <is>
-          <t>2.24</t>
-        </is>
-      </c>
-      <c r="Z16" t="inlineStr">
-        <is>
-          <t>1.07</t>
-        </is>
-      </c>
-      <c r="AA16" t="inlineStr">
-        <is>
-          <t>4.03</t>
-        </is>
-      </c>
-      <c r="AB16" t="inlineStr">
-        <is>
-          <t>3.98</t>
-        </is>
-      </c>
-      <c r="AC16" t="inlineStr">
-        <is>
-          <t>1.28</t>
-        </is>
-      </c>
-      <c r="AD16" t="inlineStr">
-        <is>
-          <t>12.80</t>
-        </is>
-      </c>
-      <c r="AE16" t="inlineStr">
-        <is>
-          <t>6.64</t>
-        </is>
-      </c>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
       <c r="AF16" t="inlineStr"/>
       <c r="AG16" t="inlineStr"/>
-      <c r="AH16" t="inlineStr">
-        <is>
-          <t>3.40</t>
-        </is>
-      </c>
-      <c r="AI16" t="inlineStr">
-        <is>
-          <t>2.01</t>
-        </is>
-      </c>
-      <c r="AJ16" t="inlineStr">
-        <is>
-          <t>3.48</t>
-        </is>
-      </c>
-      <c r="AK16" t="inlineStr">
-        <is>
-          <t>1.34</t>
-        </is>
-      </c>
-      <c r="AL16" t="inlineStr">
-        <is>
-          <t>1.42</t>
-        </is>
-      </c>
-      <c r="AM16" t="inlineStr">
-        <is>
-          <t>2.06</t>
-        </is>
-      </c>
-      <c r="AN16" t="inlineStr">
-        <is>
-          <t>9.40</t>
-        </is>
-      </c>
-      <c r="AO16" t="inlineStr">
-        <is>
-          <t>17.50</t>
-        </is>
-      </c>
-      <c r="AP16" t="inlineStr">
-        <is>
-          <t>21.00</t>
-        </is>
-      </c>
-      <c r="AQ16" t="inlineStr">
-        <is>
-          <t>12.00</t>
-        </is>
-      </c>
-      <c r="AR16" t="inlineStr">
-        <is>
-          <t>6.50</t>
-        </is>
-      </c>
-      <c r="AS16" t="inlineStr">
-        <is>
-          <t>4.36</t>
-        </is>
-      </c>
-      <c r="AT16" t="inlineStr">
-        <is>
-          <t>34.70</t>
-        </is>
-      </c>
-      <c r="AU16" t="inlineStr">
-        <is>
-          <t>15.55</t>
-        </is>
-      </c>
-      <c r="AV16" t="inlineStr">
-        <is>
-          <t>2.08</t>
-        </is>
-      </c>
-      <c r="AW16" t="inlineStr">
-        <is>
-          <t>4.27</t>
-        </is>
-      </c>
-      <c r="AX16" t="inlineStr">
-        <is>
-          <t>1.87</t>
-        </is>
-      </c>
-      <c r="AY16" t="inlineStr">
-        <is>
-          <t>2.89</t>
-        </is>
-      </c>
-      <c r="AZ16" t="inlineStr">
-        <is>
-          <t>8.47</t>
-        </is>
-      </c>
-      <c r="BA16" t="inlineStr">
-        <is>
-          <t>3.26</t>
-        </is>
-      </c>
-      <c r="BB16" t="inlineStr">
-        <is>
-          <t>9.63</t>
-        </is>
-      </c>
-      <c r="BC16" t="inlineStr">
-        <is>
-          <t>1.55</t>
-        </is>
-      </c>
-      <c r="BD16" t="inlineStr">
-        <is>
-          <t>2.33</t>
-        </is>
-      </c>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
+      <c r="AJ16" t="inlineStr"/>
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr"/>
+      <c r="AM16" t="inlineStr"/>
+      <c r="AN16" t="inlineStr"/>
+      <c r="AO16" t="inlineStr"/>
+      <c r="AP16" t="inlineStr"/>
+      <c r="AQ16" t="inlineStr"/>
+      <c r="AR16" t="inlineStr"/>
+      <c r="AS16" t="inlineStr"/>
+      <c r="AT16" t="inlineStr"/>
+      <c r="AU16" t="inlineStr"/>
+      <c r="AV16" t="inlineStr"/>
+      <c r="AW16" t="inlineStr"/>
+      <c r="AX16" t="inlineStr"/>
+      <c r="AY16" t="inlineStr"/>
+      <c r="AZ16" t="inlineStr"/>
+      <c r="BA16" t="inlineStr"/>
+      <c r="BB16" t="inlineStr"/>
+      <c r="BC16" t="inlineStr"/>
+      <c r="BD16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2853,12 +3173,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Viktoria Plzen</t>
+          <t>Omonia</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Levski Sofya</t>
+          <t>Benfica</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2878,24 +3198,24 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3230355</t>
+          <t>3230048</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.53</t>
+          <t>7.62</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>5.03</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>4.06</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
@@ -2947,12 +3267,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Omonia</t>
+          <t>Viktoria Plzen</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Benfica</t>
+          <t>Levski Sofya</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2972,24 +3292,24 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>3230048</t>
+          <t>3230355</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>7.62</t>
+          <t>1.53</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>5.03</t>
+          <t>3.48</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>4.06</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
@@ -3041,12 +3361,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>K. Almaty</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Panathinaikos</t>
+          <t>Lugano</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3056,7 +3376,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -3066,24 +3386,24 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>3229994</t>
+          <t>3230882</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>4.50</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>3.59</t>
+          <t>2.98</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>1.46</t>
+          <t>3.57</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
@@ -3135,12 +3455,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>K. Almaty</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Lugano</t>
+          <t>Panathinaikos</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3150,7 +3470,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -3160,24 +3480,24 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>3230882</t>
+          <t>3229994</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1.74</t>
+          <t>4.50</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>3.59</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>3.57</t>
+          <t>1.46</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
@@ -3437,7 +3757,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Avrupa Konferans Ligi</t>
+          <t>Konferans Ligi</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3462,61 +3782,225 @@
           <t>1.52</t>
         </is>
       </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>1.65</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>4.57</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>2.39</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>2.19</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>12.20</t>
+        </is>
+      </c>
       <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr"/>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>4.03</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>1.96</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>1.47</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>2.55</t>
+        </is>
+      </c>
       <c r="Z25" t="inlineStr"/>
-      <c r="AA25" t="inlineStr"/>
-      <c r="AB25" t="inlineStr"/>
-      <c r="AC25" t="inlineStr"/>
-      <c r="AD25" t="inlineStr"/>
-      <c r="AE25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>4.36</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>3.90</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>1.29</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>9.28</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>5.52</t>
+        </is>
+      </c>
       <c r="AF25" t="inlineStr"/>
       <c r="AG25" t="inlineStr"/>
-      <c r="AH25" t="inlineStr"/>
-      <c r="AI25" t="inlineStr"/>
-      <c r="AJ25" t="inlineStr"/>
-      <c r="AK25" t="inlineStr"/>
-      <c r="AL25" t="inlineStr"/>
-      <c r="AM25" t="inlineStr"/>
-      <c r="AN25" t="inlineStr"/>
-      <c r="AO25" t="inlineStr"/>
-      <c r="AP25" t="inlineStr"/>
-      <c r="AQ25" t="inlineStr"/>
-      <c r="AR25" t="inlineStr"/>
-      <c r="AS25" t="inlineStr"/>
-      <c r="AT25" t="inlineStr"/>
-      <c r="AU25" t="inlineStr"/>
-      <c r="AV25" t="inlineStr"/>
-      <c r="AW25" t="inlineStr"/>
-      <c r="AX25" t="inlineStr"/>
-      <c r="AY25" t="inlineStr"/>
-      <c r="AZ25" t="inlineStr"/>
-      <c r="BA25" t="inlineStr"/>
-      <c r="BB25" t="inlineStr"/>
-      <c r="BC25" t="inlineStr"/>
-      <c r="BD25" t="inlineStr"/>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>3.44</t>
+        </is>
+      </c>
+      <c r="AI25" t="inlineStr">
+        <is>
+          <t>2.45</t>
+        </is>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>3.09</t>
+        </is>
+      </c>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>1.15</t>
+        </is>
+      </c>
+      <c r="AL25" t="inlineStr">
+        <is>
+          <t>1.58</t>
+        </is>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>2.36</t>
+        </is>
+      </c>
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>7.17</t>
+        </is>
+      </c>
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>15.25</t>
+        </is>
+      </c>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>21.75</t>
+        </is>
+      </c>
+      <c r="AQ25" t="inlineStr">
+        <is>
+          <t>9.57</t>
+        </is>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>5.81</t>
+        </is>
+      </c>
+      <c r="AS25" t="inlineStr">
+        <is>
+          <t>4.64</t>
+        </is>
+      </c>
+      <c r="AT25" t="inlineStr">
+        <is>
+          <t>34.70</t>
+        </is>
+      </c>
+      <c r="AU25" t="inlineStr">
+        <is>
+          <t>13.90</t>
+        </is>
+      </c>
+      <c r="AV25" t="inlineStr">
+        <is>
+          <t>2.42</t>
+        </is>
+      </c>
+      <c r="AW25" t="inlineStr">
+        <is>
+          <t>4.20</t>
+        </is>
+      </c>
+      <c r="AX25" t="inlineStr">
+        <is>
+          <t>2.04</t>
+        </is>
+      </c>
+      <c r="AY25" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="AZ25" t="inlineStr">
+        <is>
+          <t>9.57</t>
+        </is>
+      </c>
+      <c r="BA25" t="inlineStr">
+        <is>
+          <t>2.80</t>
+        </is>
+      </c>
+      <c r="BB25" t="inlineStr">
+        <is>
+          <t>7.97</t>
+        </is>
+      </c>
+      <c r="BC25" t="inlineStr">
+        <is>
+          <t>1.69</t>
+        </is>
+      </c>
+      <c r="BD25" t="inlineStr">
+        <is>
+          <t>2.97</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Kızılyıldız</t>
+          <t>Pafos</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Kopenhag</t>
+          <t>Riga</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3531,86 +4015,246 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Avrupa Konferans Ligi</t>
+          <t>Konferans Ligi</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>3230408</t>
+          <t>3230826</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>3.21</t>
+          <t>3.70</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>2.67</t>
+          <t>4.63</t>
         </is>
       </c>
       <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>1.36</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>1.49</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>2.38</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>5.13</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>11.45</t>
+        </is>
+      </c>
       <c r="S26" t="inlineStr"/>
-      <c r="T26" t="inlineStr"/>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr"/>
-      <c r="X26" t="inlineStr"/>
-      <c r="Y26" t="inlineStr"/>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>3.90</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>1.29</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>1.85</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>2.74</t>
+        </is>
+      </c>
       <c r="Z26" t="inlineStr"/>
-      <c r="AA26" t="inlineStr"/>
-      <c r="AB26" t="inlineStr"/>
-      <c r="AC26" t="inlineStr"/>
-      <c r="AD26" t="inlineStr"/>
-      <c r="AE26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>4.81</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>4.04</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>3.31</t>
+        </is>
+      </c>
       <c r="AF26" t="inlineStr"/>
       <c r="AG26" t="inlineStr"/>
-      <c r="AH26" t="inlineStr"/>
-      <c r="AI26" t="inlineStr"/>
-      <c r="AJ26" t="inlineStr"/>
-      <c r="AK26" t="inlineStr"/>
-      <c r="AL26" t="inlineStr"/>
-      <c r="AM26" t="inlineStr"/>
-      <c r="AN26" t="inlineStr"/>
-      <c r="AO26" t="inlineStr"/>
-      <c r="AP26" t="inlineStr"/>
-      <c r="AQ26" t="inlineStr"/>
-      <c r="AR26" t="inlineStr"/>
-      <c r="AS26" t="inlineStr"/>
-      <c r="AT26" t="inlineStr"/>
-      <c r="AU26" t="inlineStr"/>
-      <c r="AV26" t="inlineStr"/>
-      <c r="AW26" t="inlineStr"/>
-      <c r="AX26" t="inlineStr"/>
-      <c r="AY26" t="inlineStr"/>
-      <c r="AZ26" t="inlineStr"/>
-      <c r="BA26" t="inlineStr"/>
-      <c r="BB26" t="inlineStr"/>
-      <c r="BC26" t="inlineStr"/>
-      <c r="BD26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>6.06</t>
+        </is>
+      </c>
+      <c r="AI26" t="inlineStr">
+        <is>
+          <t>11.50</t>
+        </is>
+      </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>2.97</t>
+        </is>
+      </c>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="AL26" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="AM26" t="inlineStr">
+        <is>
+          <t>2.46</t>
+        </is>
+      </c>
+      <c r="AN26" t="inlineStr">
+        <is>
+          <t>2.26</t>
+        </is>
+      </c>
+      <c r="AO26" t="inlineStr">
+        <is>
+          <t>15.10</t>
+        </is>
+      </c>
+      <c r="AP26" t="inlineStr">
+        <is>
+          <t>34.70</t>
+        </is>
+      </c>
+      <c r="AQ26" t="inlineStr">
+        <is>
+          <t>4.37</t>
+        </is>
+      </c>
+      <c r="AR26" t="inlineStr">
+        <is>
+          <t>5.83</t>
+        </is>
+      </c>
+      <c r="AS26" t="inlineStr">
+        <is>
+          <t>10.50</t>
+        </is>
+      </c>
+      <c r="AT26" t="inlineStr">
+        <is>
+          <t>22.30</t>
+        </is>
+      </c>
+      <c r="AU26" t="inlineStr">
+        <is>
+          <t>16.80</t>
+        </is>
+      </c>
+      <c r="AV26" t="inlineStr">
+        <is>
+          <t>8.35</t>
+        </is>
+      </c>
+      <c r="AW26" t="inlineStr">
+        <is>
+          <t>3.86</t>
+        </is>
+      </c>
+      <c r="AX26" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="AY26" t="inlineStr">
+        <is>
+          <t>3.38</t>
+        </is>
+      </c>
+      <c r="AZ26" t="inlineStr">
+        <is>
+          <t>11.10</t>
+        </is>
+      </c>
+      <c r="BA26" t="inlineStr">
+        <is>
+          <t>1.68</t>
+        </is>
+      </c>
+      <c r="BB26" t="inlineStr">
+        <is>
+          <t>2.74</t>
+        </is>
+      </c>
+      <c r="BC26" t="inlineStr">
+        <is>
+          <t>3.31</t>
+        </is>
+      </c>
+      <c r="BD26" t="inlineStr">
+        <is>
+          <t>10.05</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Nordsjaelland</t>
+          <t>Kızılyıldız</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CSKA Sofya</t>
+          <t>Kopenhag</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3630,24 +4274,24 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>3230599</t>
+          <t>3230408</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>4.44</t>
+          <t>3.21</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>5.90</t>
+          <t>2.67</t>
         </is>
       </c>
       <c r="L27" t="inlineStr"/>
@@ -3699,12 +4343,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Pafos</t>
+          <t>Nordsjaelland</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Riga</t>
+          <t>CSKA Sofya</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3719,236 +4363,76 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Konferans Ligi</t>
+          <t>Avrupa Konferans Ligi</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>3230826</t>
+          <t>3230599</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>3.70</t>
+          <t>4.44</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>4.63</t>
+          <t>5.90</t>
         </is>
       </c>
       <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>1.36</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>1.49</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>2.11</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>2.38</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>5.13</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>11.45</t>
-        </is>
-      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>3.90</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>1.29</t>
-        </is>
-      </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>1.85</t>
-        </is>
-      </c>
-      <c r="W28" t="inlineStr">
-        <is>
-          <t>1.54</t>
-        </is>
-      </c>
-      <c r="X28" t="inlineStr">
-        <is>
-          <t>1.46</t>
-        </is>
-      </c>
-      <c r="Y28" t="inlineStr">
-        <is>
-          <t>2.74</t>
-        </is>
-      </c>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr"/>
-      <c r="AA28" t="inlineStr">
-        <is>
-          <t>4.81</t>
-        </is>
-      </c>
-      <c r="AB28" t="inlineStr">
-        <is>
-          <t>4.04</t>
-        </is>
-      </c>
-      <c r="AC28" t="inlineStr">
-        <is>
-          <t>1.07</t>
-        </is>
-      </c>
-      <c r="AD28" t="inlineStr">
-        <is>
-          <t>2.27</t>
-        </is>
-      </c>
-      <c r="AE28" t="inlineStr">
-        <is>
-          <t>3.31</t>
-        </is>
-      </c>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr"/>
+      <c r="AD28" t="inlineStr"/>
+      <c r="AE28" t="inlineStr"/>
       <c r="AF28" t="inlineStr"/>
       <c r="AG28" t="inlineStr"/>
-      <c r="AH28" t="inlineStr">
-        <is>
-          <t>6.06</t>
-        </is>
-      </c>
-      <c r="AI28" t="inlineStr">
-        <is>
-          <t>11.50</t>
-        </is>
-      </c>
-      <c r="AJ28" t="inlineStr">
-        <is>
-          <t>2.97</t>
-        </is>
-      </c>
-      <c r="AK28" t="inlineStr">
-        <is>
-          <t>1.18</t>
-        </is>
-      </c>
-      <c r="AL28" t="inlineStr">
-        <is>
-          <t>1.54</t>
-        </is>
-      </c>
-      <c r="AM28" t="inlineStr">
-        <is>
-          <t>2.46</t>
-        </is>
-      </c>
-      <c r="AN28" t="inlineStr">
-        <is>
-          <t>2.26</t>
-        </is>
-      </c>
-      <c r="AO28" t="inlineStr">
-        <is>
-          <t>15.10</t>
-        </is>
-      </c>
-      <c r="AP28" t="inlineStr">
-        <is>
-          <t>34.70</t>
-        </is>
-      </c>
-      <c r="AQ28" t="inlineStr">
-        <is>
-          <t>4.37</t>
-        </is>
-      </c>
-      <c r="AR28" t="inlineStr">
-        <is>
-          <t>5.83</t>
-        </is>
-      </c>
-      <c r="AS28" t="inlineStr">
-        <is>
-          <t>10.50</t>
-        </is>
-      </c>
-      <c r="AT28" t="inlineStr">
-        <is>
-          <t>22.30</t>
-        </is>
-      </c>
-      <c r="AU28" t="inlineStr">
-        <is>
-          <t>16.80</t>
-        </is>
-      </c>
-      <c r="AV28" t="inlineStr">
-        <is>
-          <t>8.35</t>
-        </is>
-      </c>
-      <c r="AW28" t="inlineStr">
-        <is>
-          <t>3.86</t>
-        </is>
-      </c>
-      <c r="AX28" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
-      </c>
-      <c r="AY28" t="inlineStr">
-        <is>
-          <t>3.38</t>
-        </is>
-      </c>
-      <c r="AZ28" t="inlineStr">
-        <is>
-          <t>11.10</t>
-        </is>
-      </c>
-      <c r="BA28" t="inlineStr">
-        <is>
-          <t>1.68</t>
-        </is>
-      </c>
-      <c r="BB28" t="inlineStr">
-        <is>
-          <t>2.74</t>
-        </is>
-      </c>
-      <c r="BC28" t="inlineStr">
-        <is>
-          <t>3.31</t>
-        </is>
-      </c>
-      <c r="BD28" t="inlineStr">
-        <is>
-          <t>10.05</t>
-        </is>
-      </c>
+      <c r="AH28" t="inlineStr"/>
+      <c r="AI28" t="inlineStr"/>
+      <c r="AJ28" t="inlineStr"/>
+      <c r="AK28" t="inlineStr"/>
+      <c r="AL28" t="inlineStr"/>
+      <c r="AM28" t="inlineStr"/>
+      <c r="AN28" t="inlineStr"/>
+      <c r="AO28" t="inlineStr"/>
+      <c r="AP28" t="inlineStr"/>
+      <c r="AQ28" t="inlineStr"/>
+      <c r="AR28" t="inlineStr"/>
+      <c r="AS28" t="inlineStr"/>
+      <c r="AT28" t="inlineStr"/>
+      <c r="AU28" t="inlineStr"/>
+      <c r="AV28" t="inlineStr"/>
+      <c r="AW28" t="inlineStr"/>
+      <c r="AX28" t="inlineStr"/>
+      <c r="AY28" t="inlineStr"/>
+      <c r="AZ28" t="inlineStr"/>
+      <c r="BA28" t="inlineStr"/>
+      <c r="BB28" t="inlineStr"/>
+      <c r="BC28" t="inlineStr"/>
+      <c r="BD28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4301,12 +4785,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Banja Luka</t>
+          <t>Midtjylland</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Kuopion</t>
+          <t>St. Truidense</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -4321,86 +4805,250 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Avrupa Konferans Ligi</t>
+          <t>Konferans Ligi</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>3230236</t>
+          <t>3230890</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>1.61</t>
+          <t>1.48</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>3.64</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>3.84</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
+          <t>4.20</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>1.68</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>2.12</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>2.47</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>4.61</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>13.45</t>
+        </is>
+      </c>
       <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>4.46</t>
+        </is>
+      </c>
       <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr"/>
-      <c r="W31" t="inlineStr"/>
-      <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr"/>
-      <c r="Z31" t="inlineStr"/>
-      <c r="AA31" t="inlineStr"/>
-      <c r="AB31" t="inlineStr"/>
-      <c r="AC31" t="inlineStr"/>
-      <c r="AD31" t="inlineStr"/>
-      <c r="AE31" t="inlineStr"/>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>2.32</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr">
+        <is>
+          <t>1.60</t>
+        </is>
+      </c>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>1.58</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr">
+        <is>
+          <t>2.35</t>
+        </is>
+      </c>
+      <c r="Z31" t="inlineStr">
+        <is>
+          <t>1.08</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>3.86</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>3.49</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>2.32</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>3.51</t>
+        </is>
+      </c>
       <c r="AF31" t="inlineStr"/>
       <c r="AG31" t="inlineStr"/>
-      <c r="AH31" t="inlineStr"/>
-      <c r="AI31" t="inlineStr"/>
-      <c r="AJ31" t="inlineStr"/>
-      <c r="AK31" t="inlineStr"/>
-      <c r="AL31" t="inlineStr"/>
-      <c r="AM31" t="inlineStr"/>
-      <c r="AN31" t="inlineStr"/>
-      <c r="AO31" t="inlineStr"/>
-      <c r="AP31" t="inlineStr"/>
-      <c r="AQ31" t="inlineStr"/>
-      <c r="AR31" t="inlineStr"/>
-      <c r="AS31" t="inlineStr"/>
-      <c r="AT31" t="inlineStr"/>
-      <c r="AU31" t="inlineStr"/>
-      <c r="AV31" t="inlineStr"/>
-      <c r="AW31" t="inlineStr"/>
-      <c r="AX31" t="inlineStr"/>
-      <c r="AY31" t="inlineStr"/>
-      <c r="AZ31" t="inlineStr"/>
-      <c r="BA31" t="inlineStr"/>
-      <c r="BB31" t="inlineStr"/>
-      <c r="BC31" t="inlineStr"/>
-      <c r="BD31" t="inlineStr"/>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>5.73</t>
+        </is>
+      </c>
+      <c r="AI31" t="inlineStr">
+        <is>
+          <t>9.41</t>
+        </is>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>3.31</t>
+        </is>
+      </c>
+      <c r="AK31" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="AL31" t="inlineStr">
+        <is>
+          <t>1.64</t>
+        </is>
+      </c>
+      <c r="AM31" t="inlineStr">
+        <is>
+          <t>2.24</t>
+        </is>
+      </c>
+      <c r="AN31" t="inlineStr">
+        <is>
+          <t>2.13</t>
+        </is>
+      </c>
+      <c r="AO31" t="inlineStr">
+        <is>
+          <t>13.55</t>
+        </is>
+      </c>
+      <c r="AP31" t="inlineStr">
+        <is>
+          <t>34.50</t>
+        </is>
+      </c>
+      <c r="AQ31" t="inlineStr">
+        <is>
+          <t>4.50</t>
+        </is>
+      </c>
+      <c r="AR31" t="inlineStr">
+        <is>
+          <t>5.93</t>
+        </is>
+      </c>
+      <c r="AS31" t="inlineStr">
+        <is>
+          <t>9.89</t>
+        </is>
+      </c>
+      <c r="AT31" t="inlineStr">
+        <is>
+          <t>20.70</t>
+        </is>
+      </c>
+      <c r="AU31" t="inlineStr">
+        <is>
+          <t>14.95</t>
+        </is>
+      </c>
+      <c r="AV31" t="inlineStr">
+        <is>
+          <t>7.17</t>
+        </is>
+      </c>
+      <c r="AW31" t="inlineStr">
+        <is>
+          <t>4.68</t>
+        </is>
+      </c>
+      <c r="AX31" t="inlineStr">
+        <is>
+          <t>2.09</t>
+        </is>
+      </c>
+      <c r="AY31" t="inlineStr">
+        <is>
+          <t>3.02</t>
+        </is>
+      </c>
+      <c r="AZ31" t="inlineStr">
+        <is>
+          <t>8.09</t>
+        </is>
+      </c>
+      <c r="BA31" t="inlineStr">
+        <is>
+          <t>1.61</t>
+        </is>
+      </c>
+      <c r="BB31" t="inlineStr">
+        <is>
+          <t>2.72</t>
+        </is>
+      </c>
+      <c r="BC31" t="inlineStr">
+        <is>
+          <t>2.67</t>
+        </is>
+      </c>
+      <c r="BD31" t="inlineStr">
+        <is>
+          <t>7.48</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Braga</t>
+          <t>Monaco</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>KAA Gent</t>
+          <t>Freiburg</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -4415,86 +5063,250 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Avrupa Konferans Ligi</t>
+          <t>Konferans Ligi</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>3229972</t>
+          <t>3230640</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>1.68</t>
+          <t>1.94</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>3.20</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>3.65</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
+          <t>2.78</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>1.40</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>2.46</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>2.10</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>3.29</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>11.75</t>
+        </is>
+      </c>
       <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr"/>
-      <c r="W32" t="inlineStr"/>
-      <c r="X32" t="inlineStr"/>
-      <c r="Y32" t="inlineStr"/>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>3.93</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>1.08</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>2.12</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>1.70</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>1.49</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr">
+        <is>
+          <t>2.60</t>
+        </is>
+      </c>
       <c r="Z32" t="inlineStr"/>
-      <c r="AA32" t="inlineStr"/>
-      <c r="AB32" t="inlineStr"/>
-      <c r="AC32" t="inlineStr"/>
-      <c r="AD32" t="inlineStr"/>
-      <c r="AE32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>4.71</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>3.55</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>3.48</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>3.73</t>
+        </is>
+      </c>
       <c r="AF32" t="inlineStr"/>
       <c r="AG32" t="inlineStr"/>
-      <c r="AH32" t="inlineStr"/>
-      <c r="AI32" t="inlineStr"/>
-      <c r="AJ32" t="inlineStr"/>
-      <c r="AK32" t="inlineStr"/>
-      <c r="AL32" t="inlineStr"/>
-      <c r="AM32" t="inlineStr"/>
-      <c r="AN32" t="inlineStr"/>
-      <c r="AO32" t="inlineStr"/>
-      <c r="AP32" t="inlineStr"/>
-      <c r="AQ32" t="inlineStr"/>
-      <c r="AR32" t="inlineStr"/>
-      <c r="AS32" t="inlineStr"/>
-      <c r="AT32" t="inlineStr"/>
-      <c r="AU32" t="inlineStr"/>
-      <c r="AV32" t="inlineStr"/>
-      <c r="AW32" t="inlineStr"/>
-      <c r="AX32" t="inlineStr"/>
-      <c r="AY32" t="inlineStr"/>
-      <c r="AZ32" t="inlineStr"/>
-      <c r="BA32" t="inlineStr"/>
-      <c r="BB32" t="inlineStr"/>
-      <c r="BC32" t="inlineStr"/>
-      <c r="BD32" t="inlineStr"/>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>4.45</t>
+        </is>
+      </c>
+      <c r="AI32" t="inlineStr">
+        <is>
+          <t>5.70</t>
+        </is>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="AK32" t="inlineStr">
+        <is>
+          <t>1.37</t>
+        </is>
+      </c>
+      <c r="AL32" t="inlineStr">
+        <is>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="AM32" t="inlineStr">
+        <is>
+          <t>2.41</t>
+        </is>
+      </c>
+      <c r="AN32" t="inlineStr">
+        <is>
+          <t>3.20</t>
+        </is>
+      </c>
+      <c r="AO32" t="inlineStr">
+        <is>
+          <t>12.80</t>
+        </is>
+      </c>
+      <c r="AP32" t="inlineStr">
+        <is>
+          <t>30.20</t>
+        </is>
+      </c>
+      <c r="AQ32" t="inlineStr">
+        <is>
+          <t>5.43</t>
+        </is>
+      </c>
+      <c r="AR32" t="inlineStr">
+        <is>
+          <t>5.35</t>
+        </is>
+      </c>
+      <c r="AS32" t="inlineStr">
+        <is>
+          <t>7.06</t>
+        </is>
+      </c>
+      <c r="AT32" t="inlineStr">
+        <is>
+          <t>24.05</t>
+        </is>
+      </c>
+      <c r="AU32" t="inlineStr">
+        <is>
+          <t>13.25</t>
+        </is>
+      </c>
+      <c r="AV32" t="inlineStr">
+        <is>
+          <t>4.78</t>
+        </is>
+      </c>
+      <c r="AW32" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+      <c r="AX32" t="inlineStr">
+        <is>
+          <t>2.03</t>
+        </is>
+      </c>
+      <c r="AY32" t="inlineStr">
+        <is>
+          <t>3.24</t>
+        </is>
+      </c>
+      <c r="AZ32" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="BA32" t="inlineStr">
+        <is>
+          <t>1.94</t>
+        </is>
+      </c>
+      <c r="BB32" t="inlineStr">
+        <is>
+          <t>3.84</t>
+        </is>
+      </c>
+      <c r="BC32" t="inlineStr">
+        <is>
+          <t>2.19</t>
+        </is>
+      </c>
+      <c r="BD32" t="inlineStr">
+        <is>
+          <t>5.52</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Midtjylland</t>
+          <t>Banja Luka</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>St. Truidense</t>
+          <t>Kuopion</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -4514,24 +5326,24 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>3230890</t>
+          <t>3230236</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>1.48</t>
+          <t>1.61</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>3.64</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>4.20</t>
+          <t>3.84</t>
         </is>
       </c>
       <c r="L33" t="inlineStr"/>
@@ -4583,12 +5395,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Monaco</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Freiburg</t>
+          <t>KAA Gent</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -4603,240 +5415,76 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Konferans Ligi</t>
+          <t>Avrupa Konferans Ligi</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>3230640</t>
+          <t>3229972</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>1.94</t>
+          <t>1.68</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>3.20</t>
+          <t>3.13</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>2.78</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>1.14</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>1.40</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>1.28</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>2.46</t>
-        </is>
-      </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>2.10</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>3.29</t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>11.75</t>
-        </is>
-      </c>
+          <t>3.65</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr"/>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>3.93</t>
-        </is>
-      </c>
-      <c r="U34" t="inlineStr">
-        <is>
-          <t>1.08</t>
-        </is>
-      </c>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>2.12</t>
-        </is>
-      </c>
-      <c r="W34" t="inlineStr">
-        <is>
-          <t>1.70</t>
-        </is>
-      </c>
-      <c r="X34" t="inlineStr">
-        <is>
-          <t>1.49</t>
-        </is>
-      </c>
-      <c r="Y34" t="inlineStr">
-        <is>
-          <t>2.60</t>
-        </is>
-      </c>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr"/>
+      <c r="W34" t="inlineStr"/>
+      <c r="X34" t="inlineStr"/>
+      <c r="Y34" t="inlineStr"/>
       <c r="Z34" t="inlineStr"/>
-      <c r="AA34" t="inlineStr">
-        <is>
-          <t>4.71</t>
-        </is>
-      </c>
-      <c r="AB34" t="inlineStr">
-        <is>
-          <t>3.55</t>
-        </is>
-      </c>
-      <c r="AC34" t="inlineStr">
-        <is>
-          <t>1.10</t>
-        </is>
-      </c>
-      <c r="AD34" t="inlineStr">
-        <is>
-          <t>3.48</t>
-        </is>
-      </c>
-      <c r="AE34" t="inlineStr">
-        <is>
-          <t>3.73</t>
-        </is>
-      </c>
+      <c r="AA34" t="inlineStr"/>
+      <c r="AB34" t="inlineStr"/>
+      <c r="AC34" t="inlineStr"/>
+      <c r="AD34" t="inlineStr"/>
+      <c r="AE34" t="inlineStr"/>
       <c r="AF34" t="inlineStr"/>
       <c r="AG34" t="inlineStr"/>
-      <c r="AH34" t="inlineStr">
-        <is>
-          <t>4.45</t>
-        </is>
-      </c>
-      <c r="AI34" t="inlineStr">
-        <is>
-          <t>5.70</t>
-        </is>
-      </c>
-      <c r="AJ34" t="inlineStr">
-        <is>
-          <t>3.18</t>
-        </is>
-      </c>
-      <c r="AK34" t="inlineStr">
-        <is>
-          <t>1.37</t>
-        </is>
-      </c>
-      <c r="AL34" t="inlineStr">
-        <is>
-          <t>1.56</t>
-        </is>
-      </c>
-      <c r="AM34" t="inlineStr">
-        <is>
-          <t>2.41</t>
-        </is>
-      </c>
-      <c r="AN34" t="inlineStr">
-        <is>
-          <t>3.20</t>
-        </is>
-      </c>
-      <c r="AO34" t="inlineStr">
-        <is>
-          <t>12.80</t>
-        </is>
-      </c>
-      <c r="AP34" t="inlineStr">
-        <is>
-          <t>30.20</t>
-        </is>
-      </c>
-      <c r="AQ34" t="inlineStr">
-        <is>
-          <t>5.43</t>
-        </is>
-      </c>
-      <c r="AR34" t="inlineStr">
-        <is>
-          <t>5.35</t>
-        </is>
-      </c>
-      <c r="AS34" t="inlineStr">
-        <is>
-          <t>7.06</t>
-        </is>
-      </c>
-      <c r="AT34" t="inlineStr">
-        <is>
-          <t>24.05</t>
-        </is>
-      </c>
-      <c r="AU34" t="inlineStr">
-        <is>
-          <t>13.25</t>
-        </is>
-      </c>
-      <c r="AV34" t="inlineStr">
-        <is>
-          <t>4.78</t>
-        </is>
-      </c>
-      <c r="AW34" t="inlineStr">
-        <is>
-          <t>4.10</t>
-        </is>
-      </c>
-      <c r="AX34" t="inlineStr">
-        <is>
-          <t>2.03</t>
-        </is>
-      </c>
-      <c r="AY34" t="inlineStr">
-        <is>
-          <t>3.24</t>
-        </is>
-      </c>
-      <c r="AZ34" t="inlineStr">
-        <is>
-          <t>10.00</t>
-        </is>
-      </c>
-      <c r="BA34" t="inlineStr">
-        <is>
-          <t>1.94</t>
-        </is>
-      </c>
-      <c r="BB34" t="inlineStr">
-        <is>
-          <t>3.84</t>
-        </is>
-      </c>
-      <c r="BC34" t="inlineStr">
-        <is>
-          <t>2.19</t>
-        </is>
-      </c>
-      <c r="BD34" t="inlineStr">
-        <is>
-          <t>5.52</t>
-        </is>
-      </c>
+      <c r="AH34" t="inlineStr"/>
+      <c r="AI34" t="inlineStr"/>
+      <c r="AJ34" t="inlineStr"/>
+      <c r="AK34" t="inlineStr"/>
+      <c r="AL34" t="inlineStr"/>
+      <c r="AM34" t="inlineStr"/>
+      <c r="AN34" t="inlineStr"/>
+      <c r="AO34" t="inlineStr"/>
+      <c r="AP34" t="inlineStr"/>
+      <c r="AQ34" t="inlineStr"/>
+      <c r="AR34" t="inlineStr"/>
+      <c r="AS34" t="inlineStr"/>
+      <c r="AT34" t="inlineStr"/>
+      <c r="AU34" t="inlineStr"/>
+      <c r="AV34" t="inlineStr"/>
+      <c r="AW34" t="inlineStr"/>
+      <c r="AX34" t="inlineStr"/>
+      <c r="AY34" t="inlineStr"/>
+      <c r="AZ34" t="inlineStr"/>
+      <c r="BA34" t="inlineStr"/>
+      <c r="BB34" t="inlineStr"/>
+      <c r="BC34" t="inlineStr"/>
+      <c r="BD34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4935,12 +5583,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>FC Bihor</t>
+          <t>Rovaniemen</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Reşita</t>
+          <t>Kapa</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -4950,34 +5598,34 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Romanya 2. Lig</t>
+          <t>Finlandiya Ykkösliiga Play-out</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>3235235</t>
+          <t>3328665</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>1.82</t>
+          <t>2.04</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2.99</t>
+          <t>3.01</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2.85</t>
+          <t>2.44</t>
         </is>
       </c>
       <c r="L36" t="inlineStr"/>
@@ -5029,12 +5677,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Rovaniemen</t>
+          <t>FC Bihor</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Kapa</t>
+          <t>Reşita</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5044,34 +5692,34 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Finlandiya Ykkösliiga Play-out</t>
+          <t>Romanya 2. Lig</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>3328665</t>
+          <t>3235235</t>
         </is>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2.04</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>3.01</t>
+          <t>2.99</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2.44</t>
+          <t>2.85</t>
         </is>
       </c>
       <c r="L37" t="inlineStr"/>

</xml_diff>

<commit_message>
veri: ikisi guncellendi (27.10.2026 01:15)
</commit_message>
<xml_diff>
--- a/iddaa/gunluk/gunlukmaclar.xlsx
+++ b/iddaa/gunluk/gunlukmaclar.xlsx
@@ -428,11 +428,11 @@
   <dimension ref="A1:BD24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
@@ -771,163 +771,183 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mardin 1969 Spor</t>
+          <t>Roma</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Manisa FK</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Trendyol 1. Lig</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3237343</t>
+          <t>3243656</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1.62</t>
+          <t>1.37</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>3.57</t>
+          <t>5.05</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4.45</t>
+          <t>7.95</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1.51</t>
+          <t>1.28</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>1.60</t>
+          <t>1.79</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1.87</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2.08</t>
+          <t>2.45</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>4.55</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr"/>
+          <t>7.14</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>13.05</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>3.57</t>
+          <t>4.34</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.26</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>1.76</t>
+          <t>2.23</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>1.64</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.33</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2.61</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
+          <t>2.30</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>4.37</t>
+        </is>
+      </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>3.85</t>
+          <t>4.58</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.60</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>2.46</t>
+          <t>1.67</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>3.40</t>
+          <t>3.37</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>8.09</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>20.65</t>
+        </is>
+      </c>
       <c r="AJ2" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>3.30</t>
         </is>
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>2.26</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="AL2" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>1.41</t>
         </is>
       </c>
       <c r="AM2" t="inlineStr">
         <is>
-          <t>2.35</t>
+          <t>2.08</t>
         </is>
       </c>
       <c r="AN2" t="inlineStr">
         <is>
-          <t>2.12</t>
+          <t>1.60</t>
         </is>
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>14.10</t>
+          <t>19.60</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
@@ -937,17 +957,17 @@
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>4.24</t>
+          <t>3.80</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
         <is>
-          <t>5.37</t>
+          <t>7.13</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr">
         <is>
-          <t>9.93</t>
+          <t>16.25</t>
         </is>
       </c>
       <c r="AT2" t="inlineStr">
@@ -957,183 +977,359 @@
       </c>
       <c r="AU2" t="inlineStr">
         <is>
-          <t>15.75</t>
+          <t>22.55</t>
         </is>
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>7.80</t>
+          <t>14.00</t>
         </is>
       </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>3.72</t>
+          <t>4.13</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>1.97</t>
+          <t>1.86</t>
         </is>
       </c>
       <c r="AY2" t="inlineStr">
         <is>
-          <t>3.30</t>
+          <t>2.94</t>
         </is>
       </c>
       <c r="AZ2" t="inlineStr">
         <is>
-          <t>10.80</t>
+          <t>8.94</t>
         </is>
       </c>
       <c r="BA2" t="inlineStr">
         <is>
-          <t>1.46</t>
-        </is>
-      </c>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
+          <t>1.47</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>4.62</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>15.15</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ç. Rizespor</t>
+          <t>Ascoli</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Trabzonspor</t>
+          <t>Sampdoria</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Türkiye Trendyol Süper Lig</t>
+          <t>Serie B</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3241582</t>
+          <t>3243898</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3.31</t>
+          <t>1.93</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>2.95</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>3.01</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1.45</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>2.48</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>1.99</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>3.55</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>9.28</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>3.29</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
           <t>1.67</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>1.69</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>1.19</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>2.87</t>
+        </is>
+      </c>
       <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>5.76</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>4.04</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>3.57</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>3.63</t>
+        </is>
+      </c>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
-      <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
-      <c r="AX3" t="inlineStr"/>
-      <c r="AY3" t="inlineStr"/>
-      <c r="AZ3" t="inlineStr"/>
-      <c r="BA3" t="inlineStr"/>
-      <c r="BB3" t="inlineStr"/>
-      <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>4.53</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>6.58</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>2.67</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>1.23</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>2.47</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>3.01</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>12.35</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>34.50</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>5.09</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>4.50</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>7.10</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>26.00</t>
+        </is>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>13.00</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>5.07</t>
+        </is>
+      </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>3.23</t>
+        </is>
+      </c>
+      <c r="AX3" t="inlineStr">
+        <is>
+          <t>1.77</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>3.49</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>13.75</t>
+        </is>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>1.88</t>
+        </is>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>4.15</t>
+        </is>
+      </c>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>2.55</t>
+        </is>
+      </c>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>6.77</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>İspanya LaLiga</t>
+          <t>İtalya Serie A</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3238701</t>
+          <t>3243683</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.67</t>
+          <t>2.85</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>3.01</t>
+          <t>3.17</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>3.87</t>
+          <t>1.93</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -1185,133 +1381,297 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Beşiktaş</t>
+          <t>Cesena</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Başakşehir</t>
+          <t>Empoli</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Türkiye Trendyol Süper Lig</t>
+          <t>Serie B</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3241516</t>
+          <t>3243866</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>4.99</t>
+          <t>2.99</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>6.59</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+          <t>2.82</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>1.45</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>2.56</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>3.38</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>9.59</t>
+        </is>
+      </c>
       <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
-      <c r="Y5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>3.36</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>1.71</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>2.80</t>
+        </is>
+      </c>
       <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr"/>
-      <c r="AB5" t="inlineStr"/>
-      <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>5.58</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>3.96</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>3.74</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>3.68</t>
+        </is>
+      </c>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
-      <c r="AL5" t="inlineStr"/>
-      <c r="AM5" t="inlineStr"/>
-      <c r="AN5" t="inlineStr"/>
-      <c r="AO5" t="inlineStr"/>
-      <c r="AP5" t="inlineStr"/>
-      <c r="AQ5" t="inlineStr"/>
-      <c r="AR5" t="inlineStr"/>
-      <c r="AS5" t="inlineStr"/>
-      <c r="AT5" t="inlineStr"/>
-      <c r="AU5" t="inlineStr"/>
-      <c r="AV5" t="inlineStr"/>
-      <c r="AW5" t="inlineStr"/>
-      <c r="AX5" t="inlineStr"/>
-      <c r="AY5" t="inlineStr"/>
-      <c r="AZ5" t="inlineStr"/>
-      <c r="BA5" t="inlineStr"/>
-      <c r="BB5" t="inlineStr"/>
-      <c r="BC5" t="inlineStr"/>
-      <c r="BD5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>4.37</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>6.01</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>2.70</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
+        <is>
+          <t>1.22</t>
+        </is>
+      </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>2.44</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>3.14</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>12.55</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>32.00</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>5.21</t>
+        </is>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>4.62</t>
+        </is>
+      </c>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>6.74</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>26.00</t>
+        </is>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>13.00</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>4.71</t>
+        </is>
+      </c>
+      <c r="AW5" t="inlineStr">
+        <is>
+          <t>3.31</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>1.78</t>
+        </is>
+      </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>3.43</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>13.15</t>
+        </is>
+      </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>1.91</t>
+        </is>
+      </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>4.25</t>
+        </is>
+      </c>
+      <c r="BC5" t="inlineStr">
+        <is>
+          <t>2.41</t>
+        </is>
+      </c>
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>6.21</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Galatasaray</t>
+          <t>Benevento</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Fenerbahçe</t>
+          <t>Catanzaro</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Türkiye Trendyol Süper Lig</t>
+          <t>İtalya Serie B</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3241596</t>
+          <t>3243912</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1.80</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1321,7 +1681,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.87</t>
+          <t>4.00</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -1373,111 +1733,275 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Santa Clara</t>
+          <t>Mantova</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Benfica</t>
+          <t>Cremonese</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Portekiz Premier Lig</t>
+          <t>Serie B</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3234895</t>
+          <t>3243727</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>7.89</t>
+          <t>1.93</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>4.63</t>
+          <t>2.98</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>1.18</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+          <t>2.98</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>1.47</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2.52</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1.95</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>3.58</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>8.85</t>
+        </is>
+      </c>
       <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>1.15</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>1.62</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>1.75</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>1.16</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>3.06</t>
+        </is>
+      </c>
       <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>6.23</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>4.22</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>1.80</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>3.63</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>3.56</t>
+        </is>
+      </c>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr"/>
-      <c r="AM7" t="inlineStr"/>
-      <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr"/>
-      <c r="AP7" t="inlineStr"/>
-      <c r="AQ7" t="inlineStr"/>
-      <c r="AR7" t="inlineStr"/>
-      <c r="AS7" t="inlineStr"/>
-      <c r="AT7" t="inlineStr"/>
-      <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="inlineStr"/>
-      <c r="AW7" t="inlineStr"/>
-      <c r="AX7" t="inlineStr"/>
-      <c r="AY7" t="inlineStr"/>
-      <c r="AZ7" t="inlineStr"/>
-      <c r="BA7" t="inlineStr"/>
-      <c r="BB7" t="inlineStr"/>
-      <c r="BC7" t="inlineStr"/>
-      <c r="BD7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>4.42</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>6.62</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>2.58</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>1.25</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>1.25</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>2.58</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>3.04</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>12.95</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>34.50</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>4.96</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>4.48</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>6.88</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>26.50</t>
+        </is>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>13.60</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>5.05</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
+        <is>
+          <t>3.04</t>
+        </is>
+      </c>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>1.76</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>3.68</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>15.55</t>
+        </is>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>1.95</t>
+        </is>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>4.38</t>
+        </is>
+      </c>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>2.64</t>
+        </is>
+      </c>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>7.12</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Boulogne</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Reims</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1487,29 +2011,29 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Fransa Ligue 2</t>
+          <t>İtalya Serie A</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>3230473</t>
+          <t>3243801</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>3.06</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2.91</t>
+          <t>3.47</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>1.93</t>
+          <t>1.52</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -1561,49 +2085,49 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FC Andorra</t>
+          <t>Padova</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Burgos</t>
+          <t>Südtirol</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>İspanya LaLiga 2</t>
+          <t>İtalya Serie B</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>3238748</t>
+          <t>3243718</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1.91</t>
+          <t>2.14</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2.97</t>
+          <t>2.85</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>3.07</t>
+          <t>2.71</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -1655,49 +2179,49 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sepsi OSK</t>
+          <t>Coritiba</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Univ. Craiova</t>
+          <t>Gremio P.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>01:30</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Romanya 1. Lig</t>
+          <t>Brezilya Serie A</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>3234720</t>
+          <t>3239148</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>5.18</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>3.62</t>
+          <t>3.02</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>2.81</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -1749,49 +2273,49 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Torreense</t>
+          <t>Virtus Entella</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Amarante</t>
+          <t>Avellino</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>23:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Portekiz 2. Lig</t>
+          <t>İtalya Serie B</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>3235186</t>
+          <t>3243640</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1.56</t>
+          <t>1.87</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>3.87</t>
+          <t>3.30</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -1843,49 +2367,49 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Orebro SK</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Falkenbergs</t>
+          <t>Modena</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>21:05</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>İsveç Superettan</t>
+          <t>İtalya Serie B</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>3241645</t>
+          <t>3243709</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2.46</t>
+          <t>3.05</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>3.01</t>
+          <t>3.16</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>2.02</t>
+          <t>1.84</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
@@ -1937,49 +2461,49 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Istra</t>
+          <t>AIK Solna</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hajduk Split</t>
+          <t>IF Elfsborg</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Hırvatistan 1. HNL</t>
+          <t>İsveç Allsvenskan</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3235935</t>
+          <t>3243623</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>3.59</t>
+          <t>2.66</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>3.40</t>
+          <t>3.22</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>1.51</t>
+          <t>2.00</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -2031,49 +2555,49 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Walsall</t>
+          <t>Flamengo</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Salford City</t>
+          <t>Atl. Mineiro</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>İngiltere 2. Lig</t>
+          <t>Brezilya Serie A</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3241651</t>
+          <t>3239128</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2.72</t>
+          <t>1.12</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>3.04</t>
+          <t>5.24</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1.87</t>
+          <t>9.72</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -2125,49 +2649,49 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Warta Poznan</t>
+          <t>Leicester City</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>LKS Lodz</t>
+          <t>Wigan Ath</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Polonya 1. Lig</t>
+          <t>İngiltere 1. Lig</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3236360</t>
+          <t>3248006</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2.23</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2.97</t>
+          <t>4.37</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>2.23</t>
+          <t>5.94</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
@@ -2219,49 +2743,49 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Shinnik</t>
+          <t>Luton Town</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Spartak Ks</t>
+          <t>Doncaster</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Rusya FNL</t>
+          <t>İngiltere 1. Lig</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>3230414</t>
+          <t>3297737</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>1.33</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2.68</t>
+          <t>3.86</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>2.45</t>
+          <t>4.57</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
@@ -2313,49 +2837,49 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Metaloglobus B.</t>
+          <t>MK Dons</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ramnicu Valcea</t>
+          <t>Bromley</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Romanya 2. Lig</t>
+          <t>İngiltere 1. Lig</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>3234753</t>
+          <t>3328891</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>1.96</t>
+          <t>1.40</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2.96</t>
+          <t>3.62</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2.59</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
@@ -2407,49 +2931,49 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Blackburn U21</t>
+          <t>Oxford Utd</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>WBA U21</t>
+          <t>Stockport</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>İngiltere Premier Lig 2</t>
+          <t>İngiltere 1. Lig</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>3241711</t>
+          <t>3243887</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2.41</t>
+          <t>2.85</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>3.43</t>
+          <t>3.16</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.90</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
@@ -2501,49 +3025,49 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Derby U21</t>
+          <t>S. Wednesday</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Norwich U21</t>
+          <t>Cambridge</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>İngiltere Premier Lig 2</t>
+          <t>İngiltere 1. Lig</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3241530</t>
+          <t>3270647</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2.16</t>
+          <t>1.74</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>3.48</t>
+          <t>3.14</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.07</t>
+          <t>2.97</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
@@ -2595,49 +3119,49 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Bournemouth U21</t>
+          <t>Landskrona</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Brentford U21</t>
+          <t>Varbergs</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>İngiltere Premier Lig 2</t>
+          <t>İsveç Superettan</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>3241705</t>
+          <t>3243769</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1.98</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>3.61</t>
+          <t>3.15</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>2.89</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
@@ -2689,49 +3213,49 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>C. Palace U21</t>
+          <t>Barnet</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Southampton U21</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>İngiltere Premier Lig 2</t>
+          <t>İngiltere 2. Lig</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>3241578</t>
+          <t>3270642</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2.39</t>
+          <t>1.78</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>3.31</t>
+          <t>3.24</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>1.94</t>
+          <t>2.76</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
@@ -2783,49 +3307,49 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Newcastle U21</t>
+          <t>D. Zagreb</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Sunderland U21</t>
+          <t>Rijeka</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>İngiltere Premier Lig 2</t>
+          <t>Hırvatistan 1. HNL</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>3241648</t>
+          <t>3236281</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2.44</t>
+          <t>1.47</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>3.50</t>
+          <t>3.27</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>1.87</t>
+          <t>4.04</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
@@ -2877,49 +3401,49 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PSG</t>
+          <t>Stenhousemuir</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Dunfermline</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Fransa Ligue 1</t>
+          <t>İskoçya Championship</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>3238586</t>
+          <t>3245963</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>3.29</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>5.23</t>
+          <t>2.87</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>6.75</t>
+          <t>1.72</t>
         </is>
       </c>
       <c r="L23" t="inlineStr"/>
@@ -2971,17 +3495,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Montpellier</t>
+          <t>Ross County</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Red Star</t>
+          <t>Hamilton</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>26.10.2026</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2991,29 +3515,29 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Fransa Ligue 2</t>
+          <t>İskoçya 1. Lig</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>3337432</t>
+          <t>3335588</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2.05</t>
+          <t>1.38</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>3.04</t>
+          <t>3.59</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>2.70</t>
+          <t>4.35</t>
         </is>
       </c>
       <c r="L24" t="inlineStr"/>

</xml_diff>

<commit_message>
veri: ikisi guncellendi (27.10.2026 12:03)
</commit_message>
<xml_diff>
--- a/iddaa/gunluk/gunlukmaclar.xlsx
+++ b/iddaa/gunluk/gunlukmaclar.xlsx
@@ -425,11 +425,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD24"/>
+  <dimension ref="A1:BD22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -442,9 +442,9 @@
     <col width="7" customWidth="1" min="12" max="12"/>
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
-    <col width="6" customWidth="1" min="15" max="15"/>
-    <col width="6" customWidth="1" min="16" max="16"/>
-    <col width="6" customWidth="1" min="17" max="17"/>
+    <col width="5" customWidth="1" min="15" max="15"/>
+    <col width="5" customWidth="1" min="16" max="16"/>
+    <col width="5" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
@@ -771,12 +771,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Roma</t>
+          <t>Ascoli</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Sampdoria</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -786,255 +786,91 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>İtalya Serie B</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3243656</t>
+          <t>3243898</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1.37</t>
+          <t>1.93</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>5.05</t>
+          <t>2.96</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>7.95</t>
+          <t>3.02</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>1.28</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>1.79</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>1.57</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>2.45</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>7.14</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>13.05</t>
-        </is>
-      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>4.34</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>1.26</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>2.23</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>1.64</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>1.33</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>2.30</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>1.26</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>4.37</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>4.58</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>1.60</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>1.67</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>3.37</t>
-        </is>
-      </c>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>8.09</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>20.65</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>3.30</t>
-        </is>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>1.13</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>1.41</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>2.08</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>1.60</t>
-        </is>
-      </c>
-      <c r="AO2" t="inlineStr">
-        <is>
-          <t>19.60</t>
-        </is>
-      </c>
-      <c r="AP2" t="inlineStr">
-        <is>
-          <t>34.50</t>
-        </is>
-      </c>
-      <c r="AQ2" t="inlineStr">
-        <is>
-          <t>3.80</t>
-        </is>
-      </c>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>7.13</t>
-        </is>
-      </c>
-      <c r="AS2" t="inlineStr">
-        <is>
-          <t>16.25</t>
-        </is>
-      </c>
-      <c r="AT2" t="inlineStr">
-        <is>
-          <t>22.10</t>
-        </is>
-      </c>
-      <c r="AU2" t="inlineStr">
-        <is>
-          <t>22.55</t>
-        </is>
-      </c>
-      <c r="AV2" t="inlineStr">
-        <is>
-          <t>14.00</t>
-        </is>
-      </c>
-      <c r="AW2" t="inlineStr">
-        <is>
-          <t>4.13</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr">
-        <is>
-          <t>1.86</t>
-        </is>
-      </c>
-      <c r="AY2" t="inlineStr">
-        <is>
-          <t>2.94</t>
-        </is>
-      </c>
-      <c r="AZ2" t="inlineStr">
-        <is>
-          <t>8.94</t>
-        </is>
-      </c>
-      <c r="BA2" t="inlineStr">
-        <is>
-          <t>1.47</t>
-        </is>
-      </c>
-      <c r="BB2" t="inlineStr">
-        <is>
-          <t>2.27</t>
-        </is>
-      </c>
-      <c r="BC2" t="inlineStr">
-        <is>
-          <t>4.62</t>
-        </is>
-      </c>
-      <c r="BD2" t="inlineStr">
-        <is>
-          <t>15.15</t>
-        </is>
-      </c>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr"/>
+      <c r="BA2" t="inlineStr"/>
+      <c r="BB2" t="inlineStr"/>
+      <c r="BC2" t="inlineStr"/>
+      <c r="BD2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ascoli</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sampdoria</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1044,255 +880,91 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Serie B</t>
+          <t>İtalya Serie A</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3243898</t>
+          <t>3243801</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>1.93</t>
+          <t>3.95</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2.95</t>
+          <t>3.42</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>3.01</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>1.11</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>1.45</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>1.28</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>2.48</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>1.99</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>3.55</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>9.28</t>
-        </is>
-      </c>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>3.29</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>1.14</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>1.67</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>1.69</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>1.19</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>2.87</t>
-        </is>
-      </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>5.76</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>4.04</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>1.07</t>
-        </is>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>3.57</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>3.63</t>
-        </is>
-      </c>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>4.53</t>
-        </is>
-      </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>6.58</t>
-        </is>
-      </c>
-      <c r="AJ3" t="inlineStr">
-        <is>
-          <t>2.67</t>
-        </is>
-      </c>
-      <c r="AK3" t="inlineStr">
-        <is>
-          <t>1.23</t>
-        </is>
-      </c>
-      <c r="AL3" t="inlineStr">
-        <is>
-          <t>1.28</t>
-        </is>
-      </c>
-      <c r="AM3" t="inlineStr">
-        <is>
-          <t>2.47</t>
-        </is>
-      </c>
-      <c r="AN3" t="inlineStr">
-        <is>
-          <t>3.01</t>
-        </is>
-      </c>
-      <c r="AO3" t="inlineStr">
-        <is>
-          <t>12.35</t>
-        </is>
-      </c>
-      <c r="AP3" t="inlineStr">
-        <is>
-          <t>34.50</t>
-        </is>
-      </c>
-      <c r="AQ3" t="inlineStr">
-        <is>
-          <t>5.09</t>
-        </is>
-      </c>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>4.50</t>
-        </is>
-      </c>
-      <c r="AS3" t="inlineStr">
-        <is>
-          <t>7.10</t>
-        </is>
-      </c>
-      <c r="AT3" t="inlineStr">
-        <is>
-          <t>26.00</t>
-        </is>
-      </c>
-      <c r="AU3" t="inlineStr">
-        <is>
-          <t>13.00</t>
-        </is>
-      </c>
-      <c r="AV3" t="inlineStr">
-        <is>
-          <t>5.07</t>
-        </is>
-      </c>
-      <c r="AW3" t="inlineStr">
-        <is>
-          <t>3.23</t>
-        </is>
-      </c>
-      <c r="AX3" t="inlineStr">
-        <is>
-          <t>1.77</t>
-        </is>
-      </c>
-      <c r="AY3" t="inlineStr">
-        <is>
-          <t>3.49</t>
-        </is>
-      </c>
-      <c r="AZ3" t="inlineStr">
-        <is>
-          <t>13.75</t>
-        </is>
-      </c>
-      <c r="BA3" t="inlineStr">
-        <is>
-          <t>1.88</t>
-        </is>
-      </c>
-      <c r="BB3" t="inlineStr">
-        <is>
-          <t>4.15</t>
-        </is>
-      </c>
-      <c r="BC3" t="inlineStr">
-        <is>
-          <t>2.55</t>
-        </is>
-      </c>
-      <c r="BD3" t="inlineStr">
-        <is>
-          <t>6.77</t>
-        </is>
-      </c>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="inlineStr"/>
+      <c r="BA3" t="inlineStr"/>
+      <c r="BB3" t="inlineStr"/>
+      <c r="BC3" t="inlineStr"/>
+      <c r="BD3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Roma</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1302,7 +974,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1312,24 +984,24 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3243683</t>
+          <t>3243656</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2.85</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>3.17</t>
+          <t>4.94</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.93</t>
+          <t>8.07</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -1381,12 +1053,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cesena</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Empoli</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1396,245 +1068,81 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Serie B</t>
+          <t>İtalya Serie A</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3243866</t>
+          <t>3243683</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>2.96</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2.99</t>
+          <t>3.21</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2.82</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>1.13</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>1.45</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>1.26</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>2.56</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>2.00</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>3.38</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>9.59</t>
-        </is>
-      </c>
+          <t>1.87</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>3.36</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>1.13</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>1.71</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>1.67</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>1.21</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>2.80</t>
-        </is>
-      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>5.58</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>3.96</t>
-        </is>
-      </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t>1.07</t>
-        </is>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>3.74</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>3.68</t>
-        </is>
-      </c>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>4.37</t>
-        </is>
-      </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>6.01</t>
-        </is>
-      </c>
-      <c r="AJ5" t="inlineStr">
-        <is>
-          <t>2.70</t>
-        </is>
-      </c>
-      <c r="AK5" t="inlineStr">
-        <is>
-          <t>1.22</t>
-        </is>
-      </c>
-      <c r="AL5" t="inlineStr">
-        <is>
-          <t>1.28</t>
-        </is>
-      </c>
-      <c r="AM5" t="inlineStr">
-        <is>
-          <t>2.44</t>
-        </is>
-      </c>
-      <c r="AN5" t="inlineStr">
-        <is>
-          <t>3.14</t>
-        </is>
-      </c>
-      <c r="AO5" t="inlineStr">
-        <is>
-          <t>12.55</t>
-        </is>
-      </c>
-      <c r="AP5" t="inlineStr">
-        <is>
-          <t>32.00</t>
-        </is>
-      </c>
-      <c r="AQ5" t="inlineStr">
-        <is>
-          <t>5.21</t>
-        </is>
-      </c>
-      <c r="AR5" t="inlineStr">
-        <is>
-          <t>4.62</t>
-        </is>
-      </c>
-      <c r="AS5" t="inlineStr">
-        <is>
-          <t>6.74</t>
-        </is>
-      </c>
-      <c r="AT5" t="inlineStr">
-        <is>
-          <t>26.00</t>
-        </is>
-      </c>
-      <c r="AU5" t="inlineStr">
-        <is>
-          <t>13.00</t>
-        </is>
-      </c>
-      <c r="AV5" t="inlineStr">
-        <is>
-          <t>4.71</t>
-        </is>
-      </c>
-      <c r="AW5" t="inlineStr">
-        <is>
-          <t>3.31</t>
-        </is>
-      </c>
-      <c r="AX5" t="inlineStr">
-        <is>
-          <t>1.78</t>
-        </is>
-      </c>
-      <c r="AY5" t="inlineStr">
-        <is>
-          <t>3.43</t>
-        </is>
-      </c>
-      <c r="AZ5" t="inlineStr">
-        <is>
-          <t>13.15</t>
-        </is>
-      </c>
-      <c r="BA5" t="inlineStr">
-        <is>
-          <t>1.91</t>
-        </is>
-      </c>
-      <c r="BB5" t="inlineStr">
-        <is>
-          <t>4.25</t>
-        </is>
-      </c>
-      <c r="BC5" t="inlineStr">
-        <is>
-          <t>2.41</t>
-        </is>
-      </c>
-      <c r="BD5" t="inlineStr">
-        <is>
-          <t>6.21</t>
-        </is>
-      </c>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="inlineStr"/>
+      <c r="BA5" t="inlineStr"/>
+      <c r="BB5" t="inlineStr"/>
+      <c r="BC5" t="inlineStr"/>
+      <c r="BD5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1733,12 +1241,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mantova</t>
+          <t>Padova</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cremonese</t>
+          <t>Südtirol</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1753,250 +1261,86 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Serie B</t>
+          <t>İtalya Serie B</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3243727</t>
+          <t>3243718</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1.93</t>
+          <t>2.14</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>2.85</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.98</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>1.11</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>1.47</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>1.26</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>2.52</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>1.95</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>3.58</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>8.85</t>
-        </is>
-      </c>
+          <t>2.71</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>3.10</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>1.15</t>
-        </is>
-      </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>1.62</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>1.75</t>
-        </is>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>1.16</t>
-        </is>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>3.06</t>
-        </is>
-      </c>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr">
-        <is>
-          <t>6.23</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>4.22</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>1.80</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>3.63</t>
-        </is>
-      </c>
-      <c r="AE7" t="inlineStr">
-        <is>
-          <t>3.56</t>
-        </is>
-      </c>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>4.42</t>
-        </is>
-      </c>
-      <c r="AI7" t="inlineStr">
-        <is>
-          <t>6.62</t>
-        </is>
-      </c>
-      <c r="AJ7" t="inlineStr">
-        <is>
-          <t>2.58</t>
-        </is>
-      </c>
-      <c r="AK7" t="inlineStr">
-        <is>
-          <t>1.25</t>
-        </is>
-      </c>
-      <c r="AL7" t="inlineStr">
-        <is>
-          <t>1.25</t>
-        </is>
-      </c>
-      <c r="AM7" t="inlineStr">
-        <is>
-          <t>2.58</t>
-        </is>
-      </c>
-      <c r="AN7" t="inlineStr">
-        <is>
-          <t>3.04</t>
-        </is>
-      </c>
-      <c r="AO7" t="inlineStr">
-        <is>
-          <t>12.95</t>
-        </is>
-      </c>
-      <c r="AP7" t="inlineStr">
-        <is>
-          <t>34.50</t>
-        </is>
-      </c>
-      <c r="AQ7" t="inlineStr">
-        <is>
-          <t>4.96</t>
-        </is>
-      </c>
-      <c r="AR7" t="inlineStr">
-        <is>
-          <t>4.48</t>
-        </is>
-      </c>
-      <c r="AS7" t="inlineStr">
-        <is>
-          <t>6.88</t>
-        </is>
-      </c>
-      <c r="AT7" t="inlineStr">
-        <is>
-          <t>26.50</t>
-        </is>
-      </c>
-      <c r="AU7" t="inlineStr">
-        <is>
-          <t>13.60</t>
-        </is>
-      </c>
-      <c r="AV7" t="inlineStr">
-        <is>
-          <t>5.05</t>
-        </is>
-      </c>
-      <c r="AW7" t="inlineStr">
-        <is>
-          <t>3.04</t>
-        </is>
-      </c>
-      <c r="AX7" t="inlineStr">
-        <is>
-          <t>1.76</t>
-        </is>
-      </c>
-      <c r="AY7" t="inlineStr">
-        <is>
-          <t>3.68</t>
-        </is>
-      </c>
-      <c r="AZ7" t="inlineStr">
-        <is>
-          <t>15.55</t>
-        </is>
-      </c>
-      <c r="BA7" t="inlineStr">
-        <is>
-          <t>1.95</t>
-        </is>
-      </c>
-      <c r="BB7" t="inlineStr">
-        <is>
-          <t>4.38</t>
-        </is>
-      </c>
-      <c r="BC7" t="inlineStr">
-        <is>
-          <t>2.64</t>
-        </is>
-      </c>
-      <c r="BD7" t="inlineStr">
-        <is>
-          <t>7.12</t>
-        </is>
-      </c>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr"/>
+      <c r="AZ7" t="inlineStr"/>
+      <c r="BA7" t="inlineStr"/>
+      <c r="BB7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr"/>
+      <c r="BD7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Vicenza</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Modena</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2006,34 +1350,34 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>İtalya Serie A</t>
+          <t>İtalya Serie B</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>3243801</t>
+          <t>3243709</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>4.14</t>
+          <t>3.15</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>3.47</t>
+          <t>3.10</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>1.83</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -2085,12 +1429,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Padova</t>
+          <t>Cesena</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Südtirol</t>
+          <t>Empoli</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2110,24 +1454,24 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>3243718</t>
+          <t>3243866</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2.14</t>
+          <t>1.87</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2.85</t>
+          <t>2.95</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2.71</t>
+          <t>3.18</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -2179,12 +1523,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Coritiba</t>
+          <t>Mantova</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Gremio P.</t>
+          <t>Cremonese</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2194,34 +1538,34 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>01:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Brezilya Serie A</t>
+          <t>İtalya Serie B</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>3239148</t>
+          <t>3243727</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>1.98</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>3.02</t>
+          <t>2.95</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2.81</t>
+          <t>2.91</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -2367,12 +1711,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Leicester City</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Modena</t>
+          <t>Wigan Ath</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2382,34 +1726,34 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>İtalya Serie B</t>
+          <t>İngiltere 1. Lig</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>3243709</t>
+          <t>3248006</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>3.05</t>
+          <t>1.21</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>3.16</t>
+          <t>4.29</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>1.84</t>
+          <t>5.89</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
@@ -2493,17 +1837,17 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2.66</t>
+          <t>2.96</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>3.22</t>
+          <t>3.32</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2.00</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -2555,12 +1899,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Flamengo</t>
+          <t>Luton Town</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Atl. Mineiro</t>
+          <t>Doncaster</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2570,34 +1914,34 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Brezilya Serie A</t>
+          <t>İngiltere 1. Lig</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3239128</t>
+          <t>3297737</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.33</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>5.24</t>
+          <t>3.86</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>9.72</t>
+          <t>4.57</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -2649,12 +1993,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Leicester City</t>
+          <t>Oxford Utd</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Wigan Ath</t>
+          <t>Stockport</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2674,24 +2018,24 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3248006</t>
+          <t>3243887</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>2.86</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>4.37</t>
+          <t>3.13</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>5.94</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
@@ -2743,12 +2087,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Luton Town</t>
+          <t>MK Dons</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Doncaster</t>
+          <t>Bromley</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2768,24 +2112,24 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>3297737</t>
+          <t>3328891</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1.33</t>
+          <t>1.40</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3.86</t>
+          <t>3.62</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>4.57</t>
+          <t>4.14</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
@@ -2837,12 +2181,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MK Dons</t>
+          <t>S. Wednesday</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bromley</t>
+          <t>Cambridge</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2862,24 +2206,24 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>3328891</t>
+          <t>3270647</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>1.40</t>
+          <t>1.77</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>3.62</t>
+          <t>3.10</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>4.14</t>
+          <t>2.90</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
@@ -2931,12 +2275,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Oxford Utd</t>
+          <t>Landskrona</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Stockport</t>
+          <t>Varbergs</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2946,34 +2290,34 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>İngiltere 1. Lig</t>
+          <t>İsveç Superettan</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>3243887</t>
+          <t>3243769</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2.85</t>
+          <t>1.72</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>3.16</t>
+          <t>3.18</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.77</t>
+          <t>2.98</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
@@ -3025,12 +2369,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>S. Wednesday</t>
+          <t>D. Zagreb</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cambridge</t>
+          <t>Rijeka</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3040,34 +2384,34 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>İngiltere 1. Lig</t>
+          <t>Hırvatistan 1. HNL</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3270647</t>
+          <t>3236281</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.74</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>3.14</t>
+          <t>3.36</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.97</t>
+          <t>4.29</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
@@ -3119,12 +2463,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Landskrona</t>
+          <t>Barnet</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Varbergs</t>
+          <t>York City</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3134,34 +2478,34 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>İsveç Superettan</t>
+          <t>İngiltere 2. Lig</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>3243769</t>
+          <t>3270642</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1.75</t>
+          <t>1.78</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>3.15</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2.89</t>
+          <t>2.74</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
@@ -3213,12 +2557,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Barnet</t>
+          <t>Ross County</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Hamilton</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3233,29 +2577,29 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>İngiltere 2. Lig</t>
+          <t>İskoçya 1. Lig</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>3270642</t>
+          <t>3335588</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1.78</t>
+          <t>1.31</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>3.24</t>
+          <t>3.78</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>2.76</t>
+          <t>4.89</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
@@ -3307,12 +2651,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>D. Zagreb</t>
+          <t>Stenhousemuir</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Rijeka</t>
+          <t>Dunfermline</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3322,34 +2666,34 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Hırvatistan 1. HNL</t>
+          <t>İskoçya Championship</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>3236281</t>
+          <t>3245963</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1.47</t>
+          <t>3.20</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>3.27</t>
+          <t>2.92</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>4.04</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>
@@ -3398,194 +2742,6 @@
       <c r="BC22" t="inlineStr"/>
       <c r="BD22" t="inlineStr"/>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Stenhousemuir</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Dunfermline</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>22:45</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>İskoçya Championship</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>3245963</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>3.29</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>2.87</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>1.72</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
-      <c r="AA23" t="inlineStr"/>
-      <c r="AB23" t="inlineStr"/>
-      <c r="AC23" t="inlineStr"/>
-      <c r="AD23" t="inlineStr"/>
-      <c r="AE23" t="inlineStr"/>
-      <c r="AF23" t="inlineStr"/>
-      <c r="AG23" t="inlineStr"/>
-      <c r="AH23" t="inlineStr"/>
-      <c r="AI23" t="inlineStr"/>
-      <c r="AJ23" t="inlineStr"/>
-      <c r="AK23" t="inlineStr"/>
-      <c r="AL23" t="inlineStr"/>
-      <c r="AM23" t="inlineStr"/>
-      <c r="AN23" t="inlineStr"/>
-      <c r="AO23" t="inlineStr"/>
-      <c r="AP23" t="inlineStr"/>
-      <c r="AQ23" t="inlineStr"/>
-      <c r="AR23" t="inlineStr"/>
-      <c r="AS23" t="inlineStr"/>
-      <c r="AT23" t="inlineStr"/>
-      <c r="AU23" t="inlineStr"/>
-      <c r="AV23" t="inlineStr"/>
-      <c r="AW23" t="inlineStr"/>
-      <c r="AX23" t="inlineStr"/>
-      <c r="AY23" t="inlineStr"/>
-      <c r="AZ23" t="inlineStr"/>
-      <c r="BA23" t="inlineStr"/>
-      <c r="BB23" t="inlineStr"/>
-      <c r="BC23" t="inlineStr"/>
-      <c r="BD23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Ross County</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Hamilton</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>22:45</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>İskoçya 1. Lig</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>3335588</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>1.38</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>3.59</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>4.35</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="inlineStr"/>
-      <c r="AA24" t="inlineStr"/>
-      <c r="AB24" t="inlineStr"/>
-      <c r="AC24" t="inlineStr"/>
-      <c r="AD24" t="inlineStr"/>
-      <c r="AE24" t="inlineStr"/>
-      <c r="AF24" t="inlineStr"/>
-      <c r="AG24" t="inlineStr"/>
-      <c r="AH24" t="inlineStr"/>
-      <c r="AI24" t="inlineStr"/>
-      <c r="AJ24" t="inlineStr"/>
-      <c r="AK24" t="inlineStr"/>
-      <c r="AL24" t="inlineStr"/>
-      <c r="AM24" t="inlineStr"/>
-      <c r="AN24" t="inlineStr"/>
-      <c r="AO24" t="inlineStr"/>
-      <c r="AP24" t="inlineStr"/>
-      <c r="AQ24" t="inlineStr"/>
-      <c r="AR24" t="inlineStr"/>
-      <c r="AS24" t="inlineStr"/>
-      <c r="AT24" t="inlineStr"/>
-      <c r="AU24" t="inlineStr"/>
-      <c r="AV24" t="inlineStr"/>
-      <c r="AW24" t="inlineStr"/>
-      <c r="AX24" t="inlineStr"/>
-      <c r="AY24" t="inlineStr"/>
-      <c r="AZ24" t="inlineStr"/>
-      <c r="BA24" t="inlineStr"/>
-      <c r="BB24" t="inlineStr"/>
-      <c r="BC24" t="inlineStr"/>
-      <c r="BD24" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
veri: iddaa guncellendi (28.10.2026 12:30)
</commit_message>
<xml_diff>
--- a/iddaa/gunluk/gunlukmaclar.xlsx
+++ b/iddaa/gunluk/gunlukmaclar.xlsx
@@ -429,10 +429,10 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
@@ -442,9 +442,9 @@
     <col width="7" customWidth="1" min="12" max="12"/>
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
-    <col width="5" customWidth="1" min="15" max="15"/>
-    <col width="5" customWidth="1" min="16" max="16"/>
-    <col width="5" customWidth="1" min="17" max="17"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
+    <col width="6" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
@@ -771,111 +771,271 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ascoli</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sampdoria</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>İtalya Serie B</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3243898</t>
+          <t>3246154</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1.93</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2.96</t>
+          <t>3.45</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>3.02</t>
+          <t>4.68</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>1.41</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>2.07</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>1.98</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>5.02</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>8.31</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>2.86</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>1.20</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>1.86</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>1.33</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>3.55</t>
+        </is>
+      </c>
       <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>6.97</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>5.05</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>1.78</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>2.81</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>3.38</t>
+        </is>
+      </c>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>5.72</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>12.00</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>2.72</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>1.47</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>2.89</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>2.47</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>15.05</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>34.70</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>4.33</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>4.82</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>9.66</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>26.20</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>16.75</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>8.24</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>1.95</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>4.17</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>18.70</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>3.55</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>4.10</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>12.30</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -885,91 +1045,255 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>İtalya Serie A</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3243801</t>
+          <t>3246308</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>3.95</t>
+          <t>4.12</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>3.42</t>
+          <t>3.67</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1.56</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+          <t>1.75</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1.63</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1.57</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>4.28</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2.17</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2.03</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>11.65</t>
+        </is>
+      </c>
       <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
-      <c r="Y3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>3.94</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>1.93</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>1.49</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>2.59</t>
+        </is>
+      </c>
       <c r="Z3" t="inlineStr"/>
-      <c r="AA3" t="inlineStr"/>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>4.47</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>3.72</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>1.08</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>8.94</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>5.40</t>
+        </is>
+      </c>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
-      <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
-      <c r="AX3" t="inlineStr"/>
-      <c r="AY3" t="inlineStr"/>
-      <c r="AZ3" t="inlineStr"/>
-      <c r="BA3" t="inlineStr"/>
-      <c r="BB3" t="inlineStr"/>
-      <c r="BC3" t="inlineStr"/>
-      <c r="BD3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>3.64</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>2.73</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>3.24</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>1.36</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>1.57</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>2.39</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>6.74</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>14.80</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>21.70</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>9.07</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>5.47</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>4.49</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>34.50</t>
+        </is>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>13.55</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>2.28</t>
+        </is>
+      </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>4.11</t>
+        </is>
+      </c>
+      <c r="AX3" t="inlineStr">
+        <is>
+          <t>2.03</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>3.24</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>9.92</t>
+        </is>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>2.97</t>
+        </is>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>7.65</t>
+        </is>
+      </c>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>3.07</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Roma</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -984,24 +1308,24 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3243656</t>
+          <t>3246374</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>4.64</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>4.94</t>
+          <t>3.05</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>8.07</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -1053,17 +1377,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Inter</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1078,24 +1402,24 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3243683</t>
+          <t>3246456</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2.96</t>
+          <t>6.51</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>3.21</t>
+          <t>5.12</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.87</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -1147,49 +1471,49 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Benevento</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Catanzaro</t>
+          <t>Udinese</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>İtalya Serie B</t>
+          <t>İtalya Serie A</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3243912</t>
+          <t>3246220</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>2.43</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>3.50</t>
+          <t>2.81</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>4.00</t>
+          <t>2.39</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -1241,22 +1565,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Padova</t>
+          <t>Pisa</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Südtirol</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1266,24 +1590,24 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3243718</t>
+          <t>3246336</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2.14</t>
+          <t>2.18</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2.85</t>
+          <t>3.01</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.71</t>
+          <t>2.53</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
@@ -1335,17 +1659,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Vicenza</t>
+          <t>Carrarese</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Modena</t>
+          <t>Arezzo</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1360,24 +1684,24 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>3243709</t>
+          <t>3246468</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>3.15</t>
+          <t>2.02</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>3.10</t>
+          <t>2.86</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>1.83</t>
+          <t>2.91</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -1429,49 +1753,49 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cesena</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Empoli</t>
+          <t>Falkirk</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>İtalya Serie B</t>
+          <t>İskoçya Premiership</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>3243866</t>
+          <t>3246149</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1.87</t>
+          <t>1.79</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2.95</t>
+          <t>3.12</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>3.18</t>
+          <t>3.26</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -1523,17 +1847,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mantova</t>
+          <t>Juve Stabia</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cremonese</t>
+          <t>Hellas Verona</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1548,14 +1872,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>3243727</t>
+          <t>3246285</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>1.98</t>
+          <t>2.65</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1565,7 +1889,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2.91</t>
+          <t>2.12</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -1617,49 +1941,49 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Virtus Entella</t>
+          <t>Celtic</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Avellino</t>
+          <t>Dundee Utd.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>İtalya Serie B</t>
+          <t>İskoçya Premiership</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>3243640</t>
+          <t>3246337</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1.87</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2.87</t>
+          <t>6.29</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>3.30</t>
+          <t>9.41</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -1711,17 +2035,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Leicester City</t>
+          <t>Dundee FC</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Wigan Ath</t>
+          <t>Kilmarnock</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1731,29 +2055,29 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>İngiltere 1. Lig</t>
+          <t>İskoçya Premiership</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>3248006</t>
+          <t>3246191</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1.21</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>4.29</t>
+          <t>3.36</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>5.89</t>
+          <t>3.22</t>
         </is>
       </c>
       <c r="L12" t="inlineStr"/>
@@ -1805,49 +2129,49 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AIK Solna</t>
+          <t>St. Johnstone</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IF Elfsborg</t>
+          <t>Motherwell</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>İsveç Allsvenskan</t>
+          <t>İskoçya Premiership</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3243623</t>
+          <t>3246440</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2.96</t>
+          <t>2.24</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>3.32</t>
+          <t>3.10</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>1.82</t>
+          <t>2.39</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -1899,17 +2223,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Luton Town</t>
+          <t>St. Mirren</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Doncaster</t>
+          <t>Hibernian</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1919,29 +2243,29 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>İngiltere 1. Lig</t>
+          <t>İskoçya Premiership</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3297737</t>
+          <t>3246378</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1.33</t>
+          <t>2.77</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>3.86</t>
+          <t>3.22</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>4.57</t>
+          <t>1.94</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -1993,49 +2317,49 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Oxford Utd</t>
+          <t>Hearts</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Stockport</t>
+          <t>Rangers</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>İngiltere 1. Lig</t>
+          <t>İskoçya Premiership</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3243887</t>
+          <t>3246416</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2.86</t>
+          <t>3.31</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>3.40</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>1.77</t>
+          <t>1.69</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
@@ -2087,49 +2411,49 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MK Dons</t>
+          <t>Brommapojkarna</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Bromley</t>
+          <t>Hacken</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>İngiltere 1. Lig</t>
+          <t>İsveç Allsvenskan</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>3328891</t>
+          <t>3246290</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1.40</t>
+          <t>4.74</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>3.62</t>
+          <t>4.16</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>4.14</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
@@ -2181,49 +2505,49 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>S. Wednesday</t>
+          <t>Degerfors IF</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cambridge</t>
+          <t>Vasteras SK</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>İngiltere 1. Lig</t>
+          <t>İsveç Allsvenskan</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>3270647</t>
+          <t>3246444</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>1.77</t>
+          <t>2.41</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>3.10</t>
+          <t>3.00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>2.90</t>
+          <t>2.27</t>
         </is>
       </c>
       <c r="L17" t="inlineStr"/>
@@ -2275,17 +2599,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Landskrona</t>
+          <t>Göteborg</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Varbergs</t>
+          <t>Djurgarden</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2295,29 +2619,29 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>İsveç Superettan</t>
+          <t>İsveç Allsvenskan</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>3243769</t>
+          <t>3246250</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>2.93</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>3.18</t>
+          <t>3.37</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>2.98</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="L18" t="inlineStr"/>
@@ -2369,49 +2693,49 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>D. Zagreb</t>
+          <t>Radnicki K.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Rijeka</t>
+          <t>Zeleznicar</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Hırvatistan 1. HNL</t>
+          <t>Sırbistan Süper Lig</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3236281</t>
+          <t>3330524</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>2.02</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>3.36</t>
+          <t>2.86</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>4.29</t>
+          <t>2.57</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
@@ -2463,49 +2787,49 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Barnet</t>
+          <t>Halmstads BK</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>York City</t>
+          <t>Malmö</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>İngiltere 2. Lig</t>
+          <t>İsveç Allsvenskan</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>3270642</t>
+          <t>3246234</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1.78</t>
+          <t>4.08</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>3.25</t>
+          <t>3.62</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>2.74</t>
+          <t>1.50</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>
@@ -2557,49 +2881,49 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ross County</t>
+          <t>Oulu</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Hamilton</t>
+          <t>Vaasan PS</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>İskoçya 1. Lig</t>
+          <t>Finlandiya Veikkausliiga</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>3335588</t>
+          <t>3246281</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>2.19</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>3.78</t>
+          <t>3.06</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>4.89</t>
+          <t>2.48</t>
         </is>
       </c>
       <c r="L21" t="inlineStr"/>
@@ -2651,49 +2975,49 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Stenhousemuir</t>
+          <t>Radnicki Nis</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dunfermline</t>
+          <t>Partizan</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>27.10.2026</t>
+          <t>28.10.2026</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>İskoçya Championship</t>
+          <t>Sırbistan Süper Lig</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>3245963</t>
+          <t>3335647</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>3.20</t>
+          <t>3.40</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2.92</t>
+          <t>3.24</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>1.59</t>
         </is>
       </c>
       <c r="L22" t="inlineStr"/>

</xml_diff>

<commit_message>
veri: ikisi guncellendi (28.10.2026 13:48)
</commit_message>
<xml_diff>
--- a/iddaa/gunluk/gunlukmaclar.xlsx
+++ b/iddaa/gunluk/gunlukmaclar.xlsx
@@ -457,7 +457,7 @@
     <col width="12" customWidth="1" min="27" max="27"/>
     <col width="8" customWidth="1" min="28" max="28"/>
     <col width="8" customWidth="1" min="29" max="29"/>
-    <col width="6" customWidth="1" min="30" max="30"/>
+    <col width="7" customWidth="1" min="30" max="30"/>
     <col width="6" customWidth="1" min="31" max="31"/>
     <col width="6" customWidth="1" min="32" max="32"/>
     <col width="8" customWidth="1" min="33" max="33"/>
@@ -771,12 +771,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Milan</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bologna</t>
+          <t>Inter</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -796,241 +796,237 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3246154</t>
+          <t>3246456</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>6.54</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>3.45</t>
+          <t>5.26</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>4.68</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
+          <t>1.41</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1.46</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>1.41</t>
-        </is>
-      </c>
+          <t>1.42</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2.07</t>
+          <t>5.77</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>1.98</t>
+          <t>2.67</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>5.02</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>8.31</t>
-        </is>
-      </c>
+          <t>1.56</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2.86</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>1.20</t>
-        </is>
-      </c>
+          <t>6.12</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>1.54</t>
+          <t>2.75</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>1.86</t>
+          <t>1.21</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>1.33</t>
+          <t>1.65</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>3.55</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr"/>
+          <t>1.72</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
+      </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>6.97</t>
+          <t>2.77</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>5.05</t>
+          <t>3.43</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t>1.78</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>2.81</t>
+          <t>14.55</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>3.38</t>
+          <t>7.73</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>5.72</t>
+          <t>3.90</t>
         </is>
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>12.00</t>
+          <t>1.86</t>
         </is>
       </c>
       <c r="AJ2" t="inlineStr">
         <is>
-          <t>2.72</t>
+          <t>4.15</t>
         </is>
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>1.47</t>
+          <t>1.06</t>
         </is>
       </c>
       <c r="AL2" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.84</t>
         </is>
       </c>
       <c r="AM2" t="inlineStr">
         <is>
-          <t>2.89</t>
+          <t>1.94</t>
         </is>
       </c>
       <c r="AN2" t="inlineStr">
         <is>
-          <t>2.47</t>
+          <t>11.05</t>
         </is>
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>15.05</t>
+          <t>19.75</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
         <is>
+          <t>18.50</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>15.10</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>8.68</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>4.37</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
           <t>34.70</t>
         </is>
       </c>
-      <c r="AQ2" t="inlineStr">
-        <is>
-          <t>4.33</t>
-        </is>
-      </c>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>4.82</t>
-        </is>
-      </c>
-      <c r="AS2" t="inlineStr">
-        <is>
-          <t>9.66</t>
-        </is>
-      </c>
-      <c r="AT2" t="inlineStr">
-        <is>
-          <t>26.20</t>
-        </is>
-      </c>
       <c r="AU2" t="inlineStr">
         <is>
-          <t>16.75</t>
+          <t>17.70</t>
         </is>
       </c>
       <c r="AV2" t="inlineStr">
         <is>
-          <t>8.24</t>
+          <t>1.82</t>
         </is>
       </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>3.00</t>
+          <t>6.34</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>1.95</t>
+          <t>2.13</t>
         </is>
       </c>
       <c r="AY2" t="inlineStr">
         <is>
-          <t>4.17</t>
+          <t>2.46</t>
         </is>
       </c>
       <c r="AZ2" t="inlineStr">
         <is>
-          <t>18.70</t>
+          <t>5.02</t>
         </is>
       </c>
       <c r="BA2" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>3.18</t>
         </is>
       </c>
       <c r="BB2" t="inlineStr">
         <is>
-          <t>3.55</t>
+          <t>8.63</t>
         </is>
       </c>
       <c r="BC2" t="inlineStr">
         <is>
-          <t>4.10</t>
+          <t>1.36</t>
         </is>
       </c>
       <c r="BD2" t="inlineStr">
         <is>
-          <t>12.30</t>
+          <t>1.96</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Napoli</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1040,7 +1036,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1050,245 +1046,241 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3246308</t>
+          <t>3246154</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>4.12</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>3.67</t>
+          <t>3.45</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1.75</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>1.63</t>
-        </is>
-      </c>
+          <t>4.68</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.66</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>1.26</t>
+          <t>1.61</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>4.28</t>
+          <t>2.07</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2.17</t>
+          <t>1.98</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>5.02</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>11.65</t>
+          <t>8.31</t>
         </is>
       </c>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr">
         <is>
-          <t>3.94</t>
+          <t>3.06</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>1.40</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>1.93</t>
+          <t>1.54</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>1.49</t>
+          <t>1.86</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>1.33</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>2.59</t>
+          <t>3.55</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr"/>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>4.47</t>
+          <t>6.97</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>3.72</t>
+          <t>5.05</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
         <is>
-          <t>1.08</t>
+          <t>1.58</t>
         </is>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>8.94</t>
+          <t>2.81</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>5.40</t>
+          <t>3.38</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>3.64</t>
+          <t>5.72</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>2.73</t>
+          <t>12.00</t>
         </is>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>3.24</t>
+          <t>2.72</t>
         </is>
       </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.47</t>
         </is>
       </c>
       <c r="AL3" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="AM3" t="inlineStr">
         <is>
-          <t>2.39</t>
+          <t>2.89</t>
         </is>
       </c>
       <c r="AN3" t="inlineStr">
         <is>
-          <t>6.74</t>
+          <t>2.47</t>
         </is>
       </c>
       <c r="AO3" t="inlineStr">
         <is>
-          <t>14.80</t>
+          <t>15.05</t>
         </is>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
-          <t>21.70</t>
+          <t>34.70</t>
         </is>
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>9.07</t>
+          <t>4.33</t>
         </is>
       </c>
       <c r="AR3" t="inlineStr">
         <is>
-          <t>5.47</t>
+          <t>4.82</t>
         </is>
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>4.49</t>
+          <t>9.66</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr">
         <is>
-          <t>34.50</t>
+          <t>26.20</t>
         </is>
       </c>
       <c r="AU3" t="inlineStr">
         <is>
-          <t>13.55</t>
+          <t>16.75</t>
         </is>
       </c>
       <c r="AV3" t="inlineStr">
         <is>
-          <t>2.28</t>
+          <t>8.24</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>4.11</t>
+          <t>2.80</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>1.75</t>
         </is>
       </c>
       <c r="AY3" t="inlineStr">
         <is>
-          <t>3.24</t>
+          <t>3.97</t>
         </is>
       </c>
       <c r="AZ3" t="inlineStr">
         <is>
-          <t>9.92</t>
+          <t>18.50</t>
         </is>
       </c>
       <c r="BA3" t="inlineStr">
         <is>
-          <t>2.97</t>
+          <t>1.72</t>
         </is>
       </c>
       <c r="BB3" t="inlineStr">
         <is>
-          <t>7.65</t>
+          <t>3.55</t>
         </is>
       </c>
       <c r="BC3" t="inlineStr">
         <is>
-          <t>1.72</t>
+          <t>4.10</t>
         </is>
       </c>
       <c r="BD3" t="inlineStr">
         <is>
-          <t>3.07</t>
+          <t>12.30</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Udinese</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1298,7 +1290,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1308,24 +1300,24 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3246374</t>
+          <t>3246220</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>4.64</t>
+          <t>2.43</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>3.05</t>
+          <t>2.81</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.55</t>
+          <t>2.39</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -1377,12 +1369,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Inter</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1392,7 +1384,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1402,24 +1394,24 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3246456</t>
+          <t>3246308</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>6.51</t>
+          <t>3.92</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>5.12</t>
+          <t>3.47</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>1.55</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -1471,12 +1463,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Udinese</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1486,7 +1478,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1496,24 +1488,24 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3246220</t>
+          <t>3246374</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2.43</t>
+          <t>4.55</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2.81</t>
+          <t>3.04</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>2.39</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -1691,17 +1683,17 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2.02</t>
+          <t>1.93</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2.86</t>
+          <t>2.91</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>2.91</t>
+          <t>3.07</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -1847,12 +1839,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Juve Stabia</t>
+          <t>Celtic</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Hellas Verona</t>
+          <t>Dundee Utd.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1862,34 +1854,34 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>İtalya Serie B</t>
+          <t>İskoçya Premiership</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>3246285</t>
+          <t>3246337</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2.65</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2.95</t>
+          <t>6.29</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2.12</t>
+          <t>9.41</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -1941,12 +1933,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Celtic</t>
+          <t>Juve Stabia</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dundee Utd.</t>
+          <t>Hellas Verona</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1956,34 +1948,34 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>İskoçya Premiership</t>
+          <t>İtalya Serie B</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>3246337</t>
+          <t>3246285</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1.08</t>
+          <t>2.65</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>6.29</t>
+          <t>2.95</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>9.41</t>
+          <t>2.12</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -2035,12 +2027,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Dundee FC</t>
+          <t>Brommapojkarna</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Kilmarnock</t>
+          <t>Hacken</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2050,91 +2042,247 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>İskoçya Premiership</t>
+          <t>Allsvenskan</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>3246191</t>
+          <t>3246290</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1.73</t>
+          <t>5.06</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>3.36</t>
+          <t>4.29</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>3.22</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>1.62</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
+      </c>
       <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>5.02</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>2.44</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1.74</t>
+        </is>
+      </c>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>5.07</t>
+        </is>
+      </c>
       <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="inlineStr"/>
-      <c r="AA12" t="inlineStr"/>
-      <c r="AB12" t="inlineStr"/>
-      <c r="AC12" t="inlineStr"/>
-      <c r="AD12" t="inlineStr"/>
-      <c r="AE12" t="inlineStr"/>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>2.35</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>1.31</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>1.95</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>3.34</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>3.38</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>11.60</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>6.48</t>
+        </is>
+      </c>
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr"/>
-      <c r="AH12" t="inlineStr"/>
-      <c r="AI12" t="inlineStr"/>
-      <c r="AJ12" t="inlineStr"/>
-      <c r="AK12" t="inlineStr"/>
-      <c r="AL12" t="inlineStr"/>
-      <c r="AM12" t="inlineStr"/>
-      <c r="AN12" t="inlineStr"/>
-      <c r="AO12" t="inlineStr"/>
-      <c r="AP12" t="inlineStr"/>
-      <c r="AQ12" t="inlineStr"/>
-      <c r="AR12" t="inlineStr"/>
-      <c r="AS12" t="inlineStr"/>
-      <c r="AT12" t="inlineStr"/>
-      <c r="AU12" t="inlineStr"/>
-      <c r="AV12" t="inlineStr"/>
-      <c r="AW12" t="inlineStr"/>
-      <c r="AX12" t="inlineStr"/>
-      <c r="AY12" t="inlineStr"/>
-      <c r="AZ12" t="inlineStr"/>
-      <c r="BA12" t="inlineStr"/>
-      <c r="BB12" t="inlineStr"/>
-      <c r="BC12" t="inlineStr"/>
-      <c r="BD12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>3.52</t>
+        </is>
+      </c>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>1.94</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>3.63</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>1.52</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>1.90</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>8.68</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>17.20</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>19.25</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>11.85</t>
+        </is>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>7.04</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>4.24</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>34.50</t>
+        </is>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>15.45</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>1.85</t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>5.14</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>1.97</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>2.65</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>6.51</t>
+        </is>
+      </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>2.85</t>
+        </is>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>7.98</t>
+        </is>
+      </c>
+      <c r="BC12" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
+      </c>
+      <c r="BD12" t="inlineStr">
+        <is>
+          <t>2.11</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>St. Johnstone</t>
+          <t>Dundee FC</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Motherwell</t>
+          <t>Kilmarnock</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2154,24 +2302,24 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>3246440</t>
+          <t>3246191</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2.24</t>
+          <t>1.73</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>3.10</t>
+          <t>3.36</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>2.39</t>
+          <t>3.22</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
@@ -2223,12 +2371,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>St. Mirren</t>
+          <t>St. Johnstone</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Hibernian</t>
+          <t>Motherwell</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2248,24 +2396,24 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3246378</t>
+          <t>3246440</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2.77</t>
+          <t>2.24</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>3.22</t>
+          <t>3.10</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1.94</t>
+          <t>2.39</t>
         </is>
       </c>
       <c r="L14" t="inlineStr"/>
@@ -2317,12 +2465,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Hearts</t>
+          <t>St. Mirren</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Rangers</t>
+          <t>Hibernian</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2332,7 +2480,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>23:00</t>
+          <t>22:45</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -2342,24 +2490,24 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>3246416</t>
+          <t>3246378</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>3.31</t>
+          <t>2.77</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>3.40</t>
+          <t>3.22</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>1.69</t>
+          <t>1.94</t>
         </is>
       </c>
       <c r="L15" t="inlineStr"/>
@@ -2411,12 +2559,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Brommapojkarna</t>
+          <t>Hearts</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Hacken</t>
+          <t>Rangers</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2426,34 +2574,34 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>İsveç Allsvenskan</t>
+          <t>İskoçya Premiership</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>3246290</t>
+          <t>3246416</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>4.74</t>
+          <t>3.31</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>4.16</t>
+          <t>3.40</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1.36</t>
+          <t>1.69</t>
         </is>
       </c>
       <c r="L16" t="inlineStr"/>
@@ -2693,12 +2841,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Radnicki K.</t>
+          <t>Halmstads BK</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Zeleznicar</t>
+          <t>Malmö</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2708,34 +2856,34 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sırbistan Süper Lig</t>
+          <t>İsveç Allsvenskan</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3330524</t>
+          <t>3246234</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2.02</t>
+          <t>4.08</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2.86</t>
+          <t>3.62</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>2.57</t>
+          <t>1.50</t>
         </is>
       </c>
       <c r="L19" t="inlineStr"/>
@@ -2787,12 +2935,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Halmstads BK</t>
+          <t>Radnicki K.</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Malmö</t>
+          <t>Zeleznicar</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2802,34 +2950,34 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>İsveç Allsvenskan</t>
+          <t>Sırbistan Süper Lig</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>3246234</t>
+          <t>3330524</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>4.08</t>
+          <t>2.02</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>3.62</t>
+          <t>2.86</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>2.57</t>
         </is>
       </c>
       <c r="L20" t="inlineStr"/>

</xml_diff>

<commit_message>
veri: ikisi guncellendi (30.10.2026 01:09)
</commit_message>
<xml_diff>
--- a/iddaa/gunluk/gunlukmaclar.xlsx
+++ b/iddaa/gunluk/gunlukmaclar.xlsx
@@ -425,14 +425,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD8"/>
+  <dimension ref="A1:BD47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
@@ -442,9 +442,9 @@
     <col width="7" customWidth="1" min="12" max="12"/>
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
-    <col width="5" customWidth="1" min="15" max="15"/>
-    <col width="5" customWidth="1" min="16" max="16"/>
-    <col width="5" customWidth="1" min="17" max="17"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
+    <col width="6" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
@@ -457,7 +457,7 @@
     <col width="12" customWidth="1" min="27" max="27"/>
     <col width="8" customWidth="1" min="28" max="28"/>
     <col width="8" customWidth="1" min="29" max="29"/>
-    <col width="6" customWidth="1" min="30" max="30"/>
+    <col width="7" customWidth="1" min="30" max="30"/>
     <col width="6" customWidth="1" min="31" max="31"/>
     <col width="6" customWidth="1" min="32" max="32"/>
     <col width="8" customWidth="1" min="33" max="33"/>
@@ -771,143 +771,303 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kalmar</t>
+          <t>Konyaspor</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GAIS</t>
+          <t>Galatasaray</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>29.10.2026</t>
+          <t>30.10.2026</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>İsveç Allsvenskan</t>
+          <t>Trendyol Süper Lig</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>3248009</t>
+          <t>3258190</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2.13</t>
+          <t>4.98</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2.99</t>
+          <t>4.13</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>2.60</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+          <t>1.58</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1.74</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>5.18</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>2.46</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>2.04</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>12.50</t>
+        </is>
+      </c>
       <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>4.28</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>1.46</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>2.32</t>
+        </is>
+      </c>
       <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>4.46</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>4.03</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>11.50</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>6.06</t>
+        </is>
+      </c>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="inlineStr"/>
-      <c r="BA2" t="inlineStr"/>
-      <c r="BB2" t="inlineStr"/>
-      <c r="BC2" t="inlineStr"/>
-      <c r="BD2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>3.56</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>2.33</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>3.36</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>1.35</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>1.60</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>2.33</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>8.55</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>17.20</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>21.15</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>10.95</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>6.32</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>4.36</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>34.70</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>15.45</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>2.18</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>4.26</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>2.05</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>9.35</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>3.17</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>9.24</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>1.61</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>2.50</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Örgryte</t>
+          <t>Esenler Erokspor</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Mjallby</t>
+          <t>Keçiörengücü</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>29.10.2026</t>
+          <t>30.10.2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>İsveç Allsvenskan</t>
+          <t>Türkiye Trendyol 1. Lig</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>3247724</t>
+          <t>3258192</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2.64</t>
+          <t>1.62</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>3.13</t>
+          <t>3.17</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>2.05</t>
+          <t>3.31</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -959,49 +1119,49 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hammarby</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IK Sirius</t>
+          <t>Espanyol</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>29.10.2026</t>
+          <t>30.10.2026</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>23:00</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>İsveç Allsvenskan</t>
+          <t>İspanya LaLiga</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>3248004</t>
+          <t>3258486</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>1.25</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>4.21</t>
+          <t>4.58</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>5.01</t>
+          <t>5.92</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -1053,49 +1213,49 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Le Havre</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Atalanta</t>
+          <t>PSG</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>29.10.2026</t>
+          <t>30.10.2026</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>İtalya Serie A</t>
+          <t>Fransa Ligue 1</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3247862</t>
+          <t>3252325</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2.04</t>
+          <t>8.49</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>3.20</t>
+          <t>5.92</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2.60</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -1147,49 +1307,49 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Lens</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>29.10.2026</t>
+          <t>30.10.2026</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>23:05</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>İtalya Serie A</t>
+          <t>Fransa Ligue 1</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>3247795</t>
+          <t>3253790</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1.48</t>
+          <t>2.23</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>3.81</t>
+          <t>3.11</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>4.02</t>
+          <t>2.39</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -1241,143 +1401,295 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Inter Turku</t>
+          <t>Casa Pia</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>HJK Helsinki</t>
+          <t>Sporting CP</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>29.10.2026</t>
+          <t>30.10.2026</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Finlandiya Veikkausliiga</t>
+          <t>Premier Lig</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>3247870</t>
+          <t>3259957</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2.13</t>
+          <t>8.30</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>3.04</t>
+          <t>5.10</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>2.56</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+          <t>1.15</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1.84</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>7.48</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>2.50</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1.53</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>13.65</t>
+        </is>
+      </c>
       <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>4.30</t>
+        </is>
+      </c>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="inlineStr"/>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="inlineStr"/>
-      <c r="AC7" t="inlineStr"/>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>2.08</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>1.41</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>1.35</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>2.22</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>3.99</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>4.38</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>1.59</t>
+        </is>
+      </c>
       <c r="AD7" t="inlineStr"/>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
-      <c r="AL7" t="inlineStr"/>
-      <c r="AM7" t="inlineStr"/>
-      <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr"/>
-      <c r="AP7" t="inlineStr"/>
-      <c r="AQ7" t="inlineStr"/>
-      <c r="AR7" t="inlineStr"/>
-      <c r="AS7" t="inlineStr"/>
-      <c r="AT7" t="inlineStr"/>
-      <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="inlineStr"/>
-      <c r="AW7" t="inlineStr"/>
-      <c r="AX7" t="inlineStr"/>
-      <c r="AY7" t="inlineStr"/>
-      <c r="AZ7" t="inlineStr"/>
-      <c r="BA7" t="inlineStr"/>
-      <c r="BB7" t="inlineStr"/>
-      <c r="BC7" t="inlineStr"/>
-      <c r="BD7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>3.42</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>1.60</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>3.38</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>2.04</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>15.05</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>23.85</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>22.10</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>17.45</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>7.49</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>3.78</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>34.50</t>
+        </is>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>20.45</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>1.55</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
+        <is>
+          <t>4.29</t>
+        </is>
+      </c>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>1.87</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>2.88</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>8.40</t>
+        </is>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>4.76</t>
+        </is>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>15.55</t>
+        </is>
+      </c>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>1.24</t>
+        </is>
+      </c>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>1.99</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kuopion</t>
+          <t>Elversberg</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Gnistan</t>
+          <t>Mainz</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>29.10.2026</t>
+          <t>30.10.2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Finlandiya Veikkausliiga</t>
+          <t>Almanya Bundesliga</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>3247911</t>
+          <t>3253900</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>2.66</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>4.13</t>
+          <t>3.38</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>5.57</t>
+          <t>1.94</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -1426,6 +1738,3836 @@
       <c r="BC8" t="inlineStr"/>
       <c r="BD8" t="inlineStr"/>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Zulte Waregem</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Club Brugge</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Belçika Pro Lig</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>3254887</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>5.09</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>4.31</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr"/>
+      <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr"/>
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr"/>
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr"/>
+      <c r="AS9" t="inlineStr"/>
+      <c r="AT9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr"/>
+      <c r="AW9" t="inlineStr"/>
+      <c r="AX9" t="inlineStr"/>
+      <c r="AY9" t="inlineStr"/>
+      <c r="AZ9" t="inlineStr"/>
+      <c r="BA9" t="inlineStr"/>
+      <c r="BB9" t="inlineStr"/>
+      <c r="BC9" t="inlineStr"/>
+      <c r="BD9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sheffield Utd</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Wrexham</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>İngiltere Championship</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>3255481</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2.19</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>3.03</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr"/>
+      <c r="AZ10" t="inlineStr"/>
+      <c r="BA10" t="inlineStr"/>
+      <c r="BB10" t="inlineStr"/>
+      <c r="BC10" t="inlineStr"/>
+      <c r="BD10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Grenoble</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Dijon</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Fransa Ligue 2</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>3252374</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2.77</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2.91</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2.06</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
+      <c r="Z11" t="inlineStr"/>
+      <c r="AA11" t="inlineStr"/>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr"/>
+      <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr"/>
+      <c r="AQ11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr"/>
+      <c r="AS11" t="inlineStr"/>
+      <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr"/>
+      <c r="AY11" t="inlineStr"/>
+      <c r="AZ11" t="inlineStr"/>
+      <c r="BA11" t="inlineStr"/>
+      <c r="BB11" t="inlineStr"/>
+      <c r="BC11" t="inlineStr"/>
+      <c r="BD11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Metz</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pau</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Fransa Ligue 2</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>3252715</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>1.87</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>3.14</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2.98</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr"/>
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr"/>
+      <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr"/>
+      <c r="AR12" t="inlineStr"/>
+      <c r="AS12" t="inlineStr"/>
+      <c r="AT12" t="inlineStr"/>
+      <c r="AU12" t="inlineStr"/>
+      <c r="AV12" t="inlineStr"/>
+      <c r="AW12" t="inlineStr"/>
+      <c r="AX12" t="inlineStr"/>
+      <c r="AY12" t="inlineStr"/>
+      <c r="AZ12" t="inlineStr"/>
+      <c r="BA12" t="inlineStr"/>
+      <c r="BB12" t="inlineStr"/>
+      <c r="BC12" t="inlineStr"/>
+      <c r="BD12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Lavallois</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Boulogne</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Fransa Ligue 2</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>3252391</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2.12</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2.91</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2.70</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
+      <c r="AG13" t="inlineStr"/>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr"/>
+      <c r="AK13" t="inlineStr"/>
+      <c r="AL13" t="inlineStr"/>
+      <c r="AM13" t="inlineStr"/>
+      <c r="AN13" t="inlineStr"/>
+      <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="inlineStr"/>
+      <c r="AQ13" t="inlineStr"/>
+      <c r="AR13" t="inlineStr"/>
+      <c r="AS13" t="inlineStr"/>
+      <c r="AT13" t="inlineStr"/>
+      <c r="AU13" t="inlineStr"/>
+      <c r="AV13" t="inlineStr"/>
+      <c r="AW13" t="inlineStr"/>
+      <c r="AX13" t="inlineStr"/>
+      <c r="AY13" t="inlineStr"/>
+      <c r="AZ13" t="inlineStr"/>
+      <c r="BA13" t="inlineStr"/>
+      <c r="BB13" t="inlineStr"/>
+      <c r="BC13" t="inlineStr"/>
+      <c r="BD13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Nantes</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Clermont</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Fransa Ligue 2</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>3252321</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>1.31</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>3.92</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>5.92</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr"/>
+      <c r="AM14" t="inlineStr"/>
+      <c r="AN14" t="inlineStr"/>
+      <c r="AO14" t="inlineStr"/>
+      <c r="AP14" t="inlineStr"/>
+      <c r="AQ14" t="inlineStr"/>
+      <c r="AR14" t="inlineStr"/>
+      <c r="AS14" t="inlineStr"/>
+      <c r="AT14" t="inlineStr"/>
+      <c r="AU14" t="inlineStr"/>
+      <c r="AV14" t="inlineStr"/>
+      <c r="AW14" t="inlineStr"/>
+      <c r="AX14" t="inlineStr"/>
+      <c r="AY14" t="inlineStr"/>
+      <c r="AZ14" t="inlineStr"/>
+      <c r="BA14" t="inlineStr"/>
+      <c r="BB14" t="inlineStr"/>
+      <c r="BC14" t="inlineStr"/>
+      <c r="BD14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Rodez</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Dunkerque</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Fransa Ligue 2</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>3252655</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>1.87</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>3.30</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2.85</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
+      <c r="AJ15" t="inlineStr"/>
+      <c r="AK15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr"/>
+      <c r="AM15" t="inlineStr"/>
+      <c r="AN15" t="inlineStr"/>
+      <c r="AO15" t="inlineStr"/>
+      <c r="AP15" t="inlineStr"/>
+      <c r="AQ15" t="inlineStr"/>
+      <c r="AR15" t="inlineStr"/>
+      <c r="AS15" t="inlineStr"/>
+      <c r="AT15" t="inlineStr"/>
+      <c r="AU15" t="inlineStr"/>
+      <c r="AV15" t="inlineStr"/>
+      <c r="AW15" t="inlineStr"/>
+      <c r="AX15" t="inlineStr"/>
+      <c r="AY15" t="inlineStr"/>
+      <c r="AZ15" t="inlineStr"/>
+      <c r="BA15" t="inlineStr"/>
+      <c r="BB15" t="inlineStr"/>
+      <c r="BC15" t="inlineStr"/>
+      <c r="BD15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>A. Bielefeld</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Braunschweig</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Almanya 2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>3252618</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>1.64</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>3.42</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>3.53</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
+      <c r="AJ16" t="inlineStr"/>
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr"/>
+      <c r="AM16" t="inlineStr"/>
+      <c r="AN16" t="inlineStr"/>
+      <c r="AO16" t="inlineStr"/>
+      <c r="AP16" t="inlineStr"/>
+      <c r="AQ16" t="inlineStr"/>
+      <c r="AR16" t="inlineStr"/>
+      <c r="AS16" t="inlineStr"/>
+      <c r="AT16" t="inlineStr"/>
+      <c r="AU16" t="inlineStr"/>
+      <c r="AV16" t="inlineStr"/>
+      <c r="AW16" t="inlineStr"/>
+      <c r="AX16" t="inlineStr"/>
+      <c r="AY16" t="inlineStr"/>
+      <c r="AZ16" t="inlineStr"/>
+      <c r="BA16" t="inlineStr"/>
+      <c r="BB16" t="inlineStr"/>
+      <c r="BC16" t="inlineStr"/>
+      <c r="BD16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Helmond</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>FC Eindhoven</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Hollanda Eerste Divisie</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>3252360</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>1.82</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>3.30</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2.62</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr"/>
+      <c r="AM17" t="inlineStr"/>
+      <c r="AN17" t="inlineStr"/>
+      <c r="AO17" t="inlineStr"/>
+      <c r="AP17" t="inlineStr"/>
+      <c r="AQ17" t="inlineStr"/>
+      <c r="AR17" t="inlineStr"/>
+      <c r="AS17" t="inlineStr"/>
+      <c r="AT17" t="inlineStr"/>
+      <c r="AU17" t="inlineStr"/>
+      <c r="AV17" t="inlineStr"/>
+      <c r="AW17" t="inlineStr"/>
+      <c r="AX17" t="inlineStr"/>
+      <c r="AY17" t="inlineStr"/>
+      <c r="AZ17" t="inlineStr"/>
+      <c r="BA17" t="inlineStr"/>
+      <c r="BB17" t="inlineStr"/>
+      <c r="BC17" t="inlineStr"/>
+      <c r="BD17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>E. Cottbus</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Bochum</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Almanya 2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>3252309</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2.46</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>3.35</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>2.07</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr"/>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
+      <c r="AL18" t="inlineStr"/>
+      <c r="AM18" t="inlineStr"/>
+      <c r="AN18" t="inlineStr"/>
+      <c r="AO18" t="inlineStr"/>
+      <c r="AP18" t="inlineStr"/>
+      <c r="AQ18" t="inlineStr"/>
+      <c r="AR18" t="inlineStr"/>
+      <c r="AS18" t="inlineStr"/>
+      <c r="AT18" t="inlineStr"/>
+      <c r="AU18" t="inlineStr"/>
+      <c r="AV18" t="inlineStr"/>
+      <c r="AW18" t="inlineStr"/>
+      <c r="AX18" t="inlineStr"/>
+      <c r="AY18" t="inlineStr"/>
+      <c r="AZ18" t="inlineStr"/>
+      <c r="BA18" t="inlineStr"/>
+      <c r="BB18" t="inlineStr"/>
+      <c r="BC18" t="inlineStr"/>
+      <c r="BD18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Roda</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Jong AZ</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Hollanda Eerste Divisie</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>3252153</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>1.47</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>3.59</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>3.59</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr"/>
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
+      <c r="Z19" t="inlineStr"/>
+      <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr"/>
+      <c r="AD19" t="inlineStr"/>
+      <c r="AE19" t="inlineStr"/>
+      <c r="AF19" t="inlineStr"/>
+      <c r="AG19" t="inlineStr"/>
+      <c r="AH19" t="inlineStr"/>
+      <c r="AI19" t="inlineStr"/>
+      <c r="AJ19" t="inlineStr"/>
+      <c r="AK19" t="inlineStr"/>
+      <c r="AL19" t="inlineStr"/>
+      <c r="AM19" t="inlineStr"/>
+      <c r="AN19" t="inlineStr"/>
+      <c r="AO19" t="inlineStr"/>
+      <c r="AP19" t="inlineStr"/>
+      <c r="AQ19" t="inlineStr"/>
+      <c r="AR19" t="inlineStr"/>
+      <c r="AS19" t="inlineStr"/>
+      <c r="AT19" t="inlineStr"/>
+      <c r="AU19" t="inlineStr"/>
+      <c r="AV19" t="inlineStr"/>
+      <c r="AW19" t="inlineStr"/>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr"/>
+      <c r="AZ19" t="inlineStr"/>
+      <c r="BA19" t="inlineStr"/>
+      <c r="BB19" t="inlineStr"/>
+      <c r="BC19" t="inlineStr"/>
+      <c r="BD19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Volendam</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>De Graafschap</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Hollanda Eerste Divisie</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>3252395</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>1.73</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>3.53</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2.71</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
+      <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr"/>
+      <c r="Z20" t="inlineStr"/>
+      <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
+      <c r="AC20" t="inlineStr"/>
+      <c r="AD20" t="inlineStr"/>
+      <c r="AE20" t="inlineStr"/>
+      <c r="AF20" t="inlineStr"/>
+      <c r="AG20" t="inlineStr"/>
+      <c r="AH20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr"/>
+      <c r="AJ20" t="inlineStr"/>
+      <c r="AK20" t="inlineStr"/>
+      <c r="AL20" t="inlineStr"/>
+      <c r="AM20" t="inlineStr"/>
+      <c r="AN20" t="inlineStr"/>
+      <c r="AO20" t="inlineStr"/>
+      <c r="AP20" t="inlineStr"/>
+      <c r="AQ20" t="inlineStr"/>
+      <c r="AR20" t="inlineStr"/>
+      <c r="AS20" t="inlineStr"/>
+      <c r="AT20" t="inlineStr"/>
+      <c r="AU20" t="inlineStr"/>
+      <c r="AV20" t="inlineStr"/>
+      <c r="AW20" t="inlineStr"/>
+      <c r="AX20" t="inlineStr"/>
+      <c r="AY20" t="inlineStr"/>
+      <c r="AZ20" t="inlineStr"/>
+      <c r="BA20" t="inlineStr"/>
+      <c r="BB20" t="inlineStr"/>
+      <c r="BC20" t="inlineStr"/>
+      <c r="BD20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Waalwijk</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Almere City</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Hollanda Eerste Divisie</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>3252359</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>1.86</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2.50</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr"/>
+      <c r="AF21" t="inlineStr"/>
+      <c r="AG21" t="inlineStr"/>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
+      <c r="AJ21" t="inlineStr"/>
+      <c r="AK21" t="inlineStr"/>
+      <c r="AL21" t="inlineStr"/>
+      <c r="AM21" t="inlineStr"/>
+      <c r="AN21" t="inlineStr"/>
+      <c r="AO21" t="inlineStr"/>
+      <c r="AP21" t="inlineStr"/>
+      <c r="AQ21" t="inlineStr"/>
+      <c r="AR21" t="inlineStr"/>
+      <c r="AS21" t="inlineStr"/>
+      <c r="AT21" t="inlineStr"/>
+      <c r="AU21" t="inlineStr"/>
+      <c r="AV21" t="inlineStr"/>
+      <c r="AW21" t="inlineStr"/>
+      <c r="AX21" t="inlineStr"/>
+      <c r="AY21" t="inlineStr"/>
+      <c r="AZ21" t="inlineStr"/>
+      <c r="BA21" t="inlineStr"/>
+      <c r="BB21" t="inlineStr"/>
+      <c r="BC21" t="inlineStr"/>
+      <c r="BD21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Grazer AK</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Hartberg</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Avusturya Bundesliga</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>3252455</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>1.97</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>3.03</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>2.86</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr"/>
+      <c r="AB22" t="inlineStr"/>
+      <c r="AC22" t="inlineStr"/>
+      <c r="AD22" t="inlineStr"/>
+      <c r="AE22" t="inlineStr"/>
+      <c r="AF22" t="inlineStr"/>
+      <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
+      <c r="AJ22" t="inlineStr"/>
+      <c r="AK22" t="inlineStr"/>
+      <c r="AL22" t="inlineStr"/>
+      <c r="AM22" t="inlineStr"/>
+      <c r="AN22" t="inlineStr"/>
+      <c r="AO22" t="inlineStr"/>
+      <c r="AP22" t="inlineStr"/>
+      <c r="AQ22" t="inlineStr"/>
+      <c r="AR22" t="inlineStr"/>
+      <c r="AS22" t="inlineStr"/>
+      <c r="AT22" t="inlineStr"/>
+      <c r="AU22" t="inlineStr"/>
+      <c r="AV22" t="inlineStr"/>
+      <c r="AW22" t="inlineStr"/>
+      <c r="AX22" t="inlineStr"/>
+      <c r="AY22" t="inlineStr"/>
+      <c r="AZ22" t="inlineStr"/>
+      <c r="BA22" t="inlineStr"/>
+      <c r="BB22" t="inlineStr"/>
+      <c r="BC22" t="inlineStr"/>
+      <c r="BD22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Bodo/Glimt</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Viking</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Norveç Eliteserien</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>3258297</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>4.16</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>4.02</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
+      <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="inlineStr"/>
+      <c r="AB23" t="inlineStr"/>
+      <c r="AC23" t="inlineStr"/>
+      <c r="AD23" t="inlineStr"/>
+      <c r="AE23" t="inlineStr"/>
+      <c r="AF23" t="inlineStr"/>
+      <c r="AG23" t="inlineStr"/>
+      <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr"/>
+      <c r="AJ23" t="inlineStr"/>
+      <c r="AK23" t="inlineStr"/>
+      <c r="AL23" t="inlineStr"/>
+      <c r="AM23" t="inlineStr"/>
+      <c r="AN23" t="inlineStr"/>
+      <c r="AO23" t="inlineStr"/>
+      <c r="AP23" t="inlineStr"/>
+      <c r="AQ23" t="inlineStr"/>
+      <c r="AR23" t="inlineStr"/>
+      <c r="AS23" t="inlineStr"/>
+      <c r="AT23" t="inlineStr"/>
+      <c r="AU23" t="inlineStr"/>
+      <c r="AV23" t="inlineStr"/>
+      <c r="AW23" t="inlineStr"/>
+      <c r="AX23" t="inlineStr"/>
+      <c r="AY23" t="inlineStr"/>
+      <c r="AZ23" t="inlineStr"/>
+      <c r="BA23" t="inlineStr"/>
+      <c r="BB23" t="inlineStr"/>
+      <c r="BC23" t="inlineStr"/>
+      <c r="BD23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Cracovia</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Motor Lublin</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Polonya Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>3255197</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>1.96</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>3.01</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>2.56</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
+      <c r="AC24" t="inlineStr"/>
+      <c r="AD24" t="inlineStr"/>
+      <c r="AE24" t="inlineStr"/>
+      <c r="AF24" t="inlineStr"/>
+      <c r="AG24" t="inlineStr"/>
+      <c r="AH24" t="inlineStr"/>
+      <c r="AI24" t="inlineStr"/>
+      <c r="AJ24" t="inlineStr"/>
+      <c r="AK24" t="inlineStr"/>
+      <c r="AL24" t="inlineStr"/>
+      <c r="AM24" t="inlineStr"/>
+      <c r="AN24" t="inlineStr"/>
+      <c r="AO24" t="inlineStr"/>
+      <c r="AP24" t="inlineStr"/>
+      <c r="AQ24" t="inlineStr"/>
+      <c r="AR24" t="inlineStr"/>
+      <c r="AS24" t="inlineStr"/>
+      <c r="AT24" t="inlineStr"/>
+      <c r="AU24" t="inlineStr"/>
+      <c r="AV24" t="inlineStr"/>
+      <c r="AW24" t="inlineStr"/>
+      <c r="AX24" t="inlineStr"/>
+      <c r="AY24" t="inlineStr"/>
+      <c r="AZ24" t="inlineStr"/>
+      <c r="BA24" t="inlineStr"/>
+      <c r="BB24" t="inlineStr"/>
+      <c r="BC24" t="inlineStr"/>
+      <c r="BD24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Gornik Zabrze</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Legia Varşova</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Polonya Ekstraklasa</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>3253859</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>1.84</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2.93</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>2.88</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr"/>
+      <c r="AC25" t="inlineStr"/>
+      <c r="AD25" t="inlineStr"/>
+      <c r="AE25" t="inlineStr"/>
+      <c r="AF25" t="inlineStr"/>
+      <c r="AG25" t="inlineStr"/>
+      <c r="AH25" t="inlineStr"/>
+      <c r="AI25" t="inlineStr"/>
+      <c r="AJ25" t="inlineStr"/>
+      <c r="AK25" t="inlineStr"/>
+      <c r="AL25" t="inlineStr"/>
+      <c r="AM25" t="inlineStr"/>
+      <c r="AN25" t="inlineStr"/>
+      <c r="AO25" t="inlineStr"/>
+      <c r="AP25" t="inlineStr"/>
+      <c r="AQ25" t="inlineStr"/>
+      <c r="AR25" t="inlineStr"/>
+      <c r="AS25" t="inlineStr"/>
+      <c r="AT25" t="inlineStr"/>
+      <c r="AU25" t="inlineStr"/>
+      <c r="AV25" t="inlineStr"/>
+      <c r="AW25" t="inlineStr"/>
+      <c r="AX25" t="inlineStr"/>
+      <c r="AY25" t="inlineStr"/>
+      <c r="AZ25" t="inlineStr"/>
+      <c r="BA25" t="inlineStr"/>
+      <c r="BB25" t="inlineStr"/>
+      <c r="BC25" t="inlineStr"/>
+      <c r="BD25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Brisbane</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Auckland</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Avustralya A Lig</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>3252151</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2.47</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>3.02</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>2.21</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr"/>
+      <c r="AC26" t="inlineStr"/>
+      <c r="AD26" t="inlineStr"/>
+      <c r="AE26" t="inlineStr"/>
+      <c r="AF26" t="inlineStr"/>
+      <c r="AG26" t="inlineStr"/>
+      <c r="AH26" t="inlineStr"/>
+      <c r="AI26" t="inlineStr"/>
+      <c r="AJ26" t="inlineStr"/>
+      <c r="AK26" t="inlineStr"/>
+      <c r="AL26" t="inlineStr"/>
+      <c r="AM26" t="inlineStr"/>
+      <c r="AN26" t="inlineStr"/>
+      <c r="AO26" t="inlineStr"/>
+      <c r="AP26" t="inlineStr"/>
+      <c r="AQ26" t="inlineStr"/>
+      <c r="AR26" t="inlineStr"/>
+      <c r="AS26" t="inlineStr"/>
+      <c r="AT26" t="inlineStr"/>
+      <c r="AU26" t="inlineStr"/>
+      <c r="AV26" t="inlineStr"/>
+      <c r="AW26" t="inlineStr"/>
+      <c r="AX26" t="inlineStr"/>
+      <c r="AY26" t="inlineStr"/>
+      <c r="AZ26" t="inlineStr"/>
+      <c r="BA26" t="inlineStr"/>
+      <c r="BB26" t="inlineStr"/>
+      <c r="BC26" t="inlineStr"/>
+      <c r="BD26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Vasco Da Gama</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>02:00</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Serie A</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>3246353</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>3.80</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>3.22</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>1.63</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>1.38</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>1.41</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>4.56</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>2.30</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>9.98</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>3.44</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>1.94</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>1.83</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>1.41</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>2.93</t>
+        </is>
+      </c>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>5.56</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>4.29</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>1.26</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>8.89</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>5.20</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr"/>
+      <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>3.41</t>
+        </is>
+      </c>
+      <c r="AI27" t="inlineStr">
+        <is>
+          <t>2.77</t>
+        </is>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>2.98</t>
+        </is>
+      </c>
+      <c r="AK27" t="inlineStr">
+        <is>
+          <t>1.41</t>
+        </is>
+      </c>
+      <c r="AL27" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="AM27" t="inlineStr">
+        <is>
+          <t>2.59</t>
+        </is>
+      </c>
+      <c r="AN27" t="inlineStr">
+        <is>
+          <t>7.03</t>
+        </is>
+      </c>
+      <c r="AO27" t="inlineStr">
+        <is>
+          <t>15.10</t>
+        </is>
+      </c>
+      <c r="AP27" t="inlineStr">
+        <is>
+          <t>23.60</t>
+        </is>
+      </c>
+      <c r="AQ27" t="inlineStr">
+        <is>
+          <t>9.01</t>
+        </is>
+      </c>
+      <c r="AR27" t="inlineStr">
+        <is>
+          <t>5.20</t>
+        </is>
+      </c>
+      <c r="AS27" t="inlineStr">
+        <is>
+          <t>4.64</t>
+        </is>
+      </c>
+      <c r="AT27" t="inlineStr">
+        <is>
+          <t>34.70</t>
+        </is>
+      </c>
+      <c r="AU27" t="inlineStr">
+        <is>
+          <t>13.80</t>
+        </is>
+      </c>
+      <c r="AV27" t="inlineStr">
+        <is>
+          <t>2.57</t>
+        </is>
+      </c>
+      <c r="AW27" t="inlineStr">
+        <is>
+          <t>3.40</t>
+        </is>
+      </c>
+      <c r="AX27" t="inlineStr">
+        <is>
+          <t>1.79</t>
+        </is>
+      </c>
+      <c r="AY27" t="inlineStr">
+        <is>
+          <t>3.35</t>
+        </is>
+      </c>
+      <c r="AZ27" t="inlineStr">
+        <is>
+          <t>12.45</t>
+        </is>
+      </c>
+      <c r="BA27" t="inlineStr">
+        <is>
+          <t>3.23</t>
+        </is>
+      </c>
+      <c r="BB27" t="inlineStr">
+        <is>
+          <t>8.96</t>
+        </is>
+      </c>
+      <c r="BC27" t="inlineStr">
+        <is>
+          <t>1.65</t>
+        </is>
+      </c>
+      <c r="BD27" t="inlineStr">
+        <is>
+          <t>3.44</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Atl. Mineiro</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Cruzeiro MG</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>01:30</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Brezilya Serie A</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>3246495</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2.48</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>3.21</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>2.12</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr"/>
+      <c r="AC28" t="inlineStr"/>
+      <c r="AD28" t="inlineStr"/>
+      <c r="AE28" t="inlineStr"/>
+      <c r="AF28" t="inlineStr"/>
+      <c r="AG28" t="inlineStr"/>
+      <c r="AH28" t="inlineStr"/>
+      <c r="AI28" t="inlineStr"/>
+      <c r="AJ28" t="inlineStr"/>
+      <c r="AK28" t="inlineStr"/>
+      <c r="AL28" t="inlineStr"/>
+      <c r="AM28" t="inlineStr"/>
+      <c r="AN28" t="inlineStr"/>
+      <c r="AO28" t="inlineStr"/>
+      <c r="AP28" t="inlineStr"/>
+      <c r="AQ28" t="inlineStr"/>
+      <c r="AR28" t="inlineStr"/>
+      <c r="AS28" t="inlineStr"/>
+      <c r="AT28" t="inlineStr"/>
+      <c r="AU28" t="inlineStr"/>
+      <c r="AV28" t="inlineStr"/>
+      <c r="AW28" t="inlineStr"/>
+      <c r="AX28" t="inlineStr"/>
+      <c r="AY28" t="inlineStr"/>
+      <c r="AZ28" t="inlineStr"/>
+      <c r="BA28" t="inlineStr"/>
+      <c r="BB28" t="inlineStr"/>
+      <c r="BC28" t="inlineStr"/>
+      <c r="BD28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Gremio P.</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Paranaense</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>03:30</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Brezilya Serie A</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>3246211</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2.09</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>2.66</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr"/>
+      <c r="AC29" t="inlineStr"/>
+      <c r="AD29" t="inlineStr"/>
+      <c r="AE29" t="inlineStr"/>
+      <c r="AF29" t="inlineStr"/>
+      <c r="AG29" t="inlineStr"/>
+      <c r="AH29" t="inlineStr"/>
+      <c r="AI29" t="inlineStr"/>
+      <c r="AJ29" t="inlineStr"/>
+      <c r="AK29" t="inlineStr"/>
+      <c r="AL29" t="inlineStr"/>
+      <c r="AM29" t="inlineStr"/>
+      <c r="AN29" t="inlineStr"/>
+      <c r="AO29" t="inlineStr"/>
+      <c r="AP29" t="inlineStr"/>
+      <c r="AQ29" t="inlineStr"/>
+      <c r="AR29" t="inlineStr"/>
+      <c r="AS29" t="inlineStr"/>
+      <c r="AT29" t="inlineStr"/>
+      <c r="AU29" t="inlineStr"/>
+      <c r="AV29" t="inlineStr"/>
+      <c r="AW29" t="inlineStr"/>
+      <c r="AX29" t="inlineStr"/>
+      <c r="AY29" t="inlineStr"/>
+      <c r="AZ29" t="inlineStr"/>
+      <c r="BA29" t="inlineStr"/>
+      <c r="BB29" t="inlineStr"/>
+      <c r="BC29" t="inlineStr"/>
+      <c r="BD29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Aalborg</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Hobro</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Danimarka 1. Lig</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>3252505</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>1.48</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>3.32</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>3.85</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr"/>
+      <c r="AD30" t="inlineStr"/>
+      <c r="AE30" t="inlineStr"/>
+      <c r="AF30" t="inlineStr"/>
+      <c r="AG30" t="inlineStr"/>
+      <c r="AH30" t="inlineStr"/>
+      <c r="AI30" t="inlineStr"/>
+      <c r="AJ30" t="inlineStr"/>
+      <c r="AK30" t="inlineStr"/>
+      <c r="AL30" t="inlineStr"/>
+      <c r="AM30" t="inlineStr"/>
+      <c r="AN30" t="inlineStr"/>
+      <c r="AO30" t="inlineStr"/>
+      <c r="AP30" t="inlineStr"/>
+      <c r="AQ30" t="inlineStr"/>
+      <c r="AR30" t="inlineStr"/>
+      <c r="AS30" t="inlineStr"/>
+      <c r="AT30" t="inlineStr"/>
+      <c r="AU30" t="inlineStr"/>
+      <c r="AV30" t="inlineStr"/>
+      <c r="AW30" t="inlineStr"/>
+      <c r="AX30" t="inlineStr"/>
+      <c r="AY30" t="inlineStr"/>
+      <c r="AZ30" t="inlineStr"/>
+      <c r="BA30" t="inlineStr"/>
+      <c r="BB30" t="inlineStr"/>
+      <c r="BC30" t="inlineStr"/>
+      <c r="BD30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>IK Oddevold</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>IK Brage</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>İsveç Superettan</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>3252673</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>1.51</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>3.49</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>3.52</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr"/>
+      <c r="AC31" t="inlineStr"/>
+      <c r="AD31" t="inlineStr"/>
+      <c r="AE31" t="inlineStr"/>
+      <c r="AF31" t="inlineStr"/>
+      <c r="AG31" t="inlineStr"/>
+      <c r="AH31" t="inlineStr"/>
+      <c r="AI31" t="inlineStr"/>
+      <c r="AJ31" t="inlineStr"/>
+      <c r="AK31" t="inlineStr"/>
+      <c r="AL31" t="inlineStr"/>
+      <c r="AM31" t="inlineStr"/>
+      <c r="AN31" t="inlineStr"/>
+      <c r="AO31" t="inlineStr"/>
+      <c r="AP31" t="inlineStr"/>
+      <c r="AQ31" t="inlineStr"/>
+      <c r="AR31" t="inlineStr"/>
+      <c r="AS31" t="inlineStr"/>
+      <c r="AT31" t="inlineStr"/>
+      <c r="AU31" t="inlineStr"/>
+      <c r="AV31" t="inlineStr"/>
+      <c r="AW31" t="inlineStr"/>
+      <c r="AX31" t="inlineStr"/>
+      <c r="AY31" t="inlineStr"/>
+      <c r="AZ31" t="inlineStr"/>
+      <c r="BA31" t="inlineStr"/>
+      <c r="BB31" t="inlineStr"/>
+      <c r="BC31" t="inlineStr"/>
+      <c r="BD31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Rapperswil</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Nyon</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>İsviçre Challenge Lig</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>3252161</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>1.28</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>4.16</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>4.76</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr"/>
+      <c r="AC32" t="inlineStr"/>
+      <c r="AD32" t="inlineStr"/>
+      <c r="AE32" t="inlineStr"/>
+      <c r="AF32" t="inlineStr"/>
+      <c r="AG32" t="inlineStr"/>
+      <c r="AH32" t="inlineStr"/>
+      <c r="AI32" t="inlineStr"/>
+      <c r="AJ32" t="inlineStr"/>
+      <c r="AK32" t="inlineStr"/>
+      <c r="AL32" t="inlineStr"/>
+      <c r="AM32" t="inlineStr"/>
+      <c r="AN32" t="inlineStr"/>
+      <c r="AO32" t="inlineStr"/>
+      <c r="AP32" t="inlineStr"/>
+      <c r="AQ32" t="inlineStr"/>
+      <c r="AR32" t="inlineStr"/>
+      <c r="AS32" t="inlineStr"/>
+      <c r="AT32" t="inlineStr"/>
+      <c r="AU32" t="inlineStr"/>
+      <c r="AV32" t="inlineStr"/>
+      <c r="AW32" t="inlineStr"/>
+      <c r="AX32" t="inlineStr"/>
+      <c r="AY32" t="inlineStr"/>
+      <c r="AZ32" t="inlineStr"/>
+      <c r="BA32" t="inlineStr"/>
+      <c r="BB32" t="inlineStr"/>
+      <c r="BC32" t="inlineStr"/>
+      <c r="BD32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Stade Ouchy</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Yverdon</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>İsviçre Challenge Lig</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>3252570</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>2.13</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>3.00</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>2.32</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr"/>
+      <c r="AD33" t="inlineStr"/>
+      <c r="AE33" t="inlineStr"/>
+      <c r="AF33" t="inlineStr"/>
+      <c r="AG33" t="inlineStr"/>
+      <c r="AH33" t="inlineStr"/>
+      <c r="AI33" t="inlineStr"/>
+      <c r="AJ33" t="inlineStr"/>
+      <c r="AK33" t="inlineStr"/>
+      <c r="AL33" t="inlineStr"/>
+      <c r="AM33" t="inlineStr"/>
+      <c r="AN33" t="inlineStr"/>
+      <c r="AO33" t="inlineStr"/>
+      <c r="AP33" t="inlineStr"/>
+      <c r="AQ33" t="inlineStr"/>
+      <c r="AR33" t="inlineStr"/>
+      <c r="AS33" t="inlineStr"/>
+      <c r="AT33" t="inlineStr"/>
+      <c r="AU33" t="inlineStr"/>
+      <c r="AV33" t="inlineStr"/>
+      <c r="AW33" t="inlineStr"/>
+      <c r="AX33" t="inlineStr"/>
+      <c r="AY33" t="inlineStr"/>
+      <c r="AZ33" t="inlineStr"/>
+      <c r="BA33" t="inlineStr"/>
+      <c r="BB33" t="inlineStr"/>
+      <c r="BC33" t="inlineStr"/>
+      <c r="BD33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Etoile Carouge</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Kriens</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>İsviçre Challenge Lig</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>3254319</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>1.87</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>3.18</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>2.62</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr"/>
+      <c r="W34" t="inlineStr"/>
+      <c r="X34" t="inlineStr"/>
+      <c r="Y34" t="inlineStr"/>
+      <c r="Z34" t="inlineStr"/>
+      <c r="AA34" t="inlineStr"/>
+      <c r="AB34" t="inlineStr"/>
+      <c r="AC34" t="inlineStr"/>
+      <c r="AD34" t="inlineStr"/>
+      <c r="AE34" t="inlineStr"/>
+      <c r="AF34" t="inlineStr"/>
+      <c r="AG34" t="inlineStr"/>
+      <c r="AH34" t="inlineStr"/>
+      <c r="AI34" t="inlineStr"/>
+      <c r="AJ34" t="inlineStr"/>
+      <c r="AK34" t="inlineStr"/>
+      <c r="AL34" t="inlineStr"/>
+      <c r="AM34" t="inlineStr"/>
+      <c r="AN34" t="inlineStr"/>
+      <c r="AO34" t="inlineStr"/>
+      <c r="AP34" t="inlineStr"/>
+      <c r="AQ34" t="inlineStr"/>
+      <c r="AR34" t="inlineStr"/>
+      <c r="AS34" t="inlineStr"/>
+      <c r="AT34" t="inlineStr"/>
+      <c r="AU34" t="inlineStr"/>
+      <c r="AV34" t="inlineStr"/>
+      <c r="AW34" t="inlineStr"/>
+      <c r="AX34" t="inlineStr"/>
+      <c r="AY34" t="inlineStr"/>
+      <c r="AZ34" t="inlineStr"/>
+      <c r="BA34" t="inlineStr"/>
+      <c r="BB34" t="inlineStr"/>
+      <c r="BC34" t="inlineStr"/>
+      <c r="BD34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>N. Xamax</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Aarau</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>İsviçre Challenge Lig</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>3255047</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2.26</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>3.26</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>2.06</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr"/>
+      <c r="W35" t="inlineStr"/>
+      <c r="X35" t="inlineStr"/>
+      <c r="Y35" t="inlineStr"/>
+      <c r="Z35" t="inlineStr"/>
+      <c r="AA35" t="inlineStr"/>
+      <c r="AB35" t="inlineStr"/>
+      <c r="AC35" t="inlineStr"/>
+      <c r="AD35" t="inlineStr"/>
+      <c r="AE35" t="inlineStr"/>
+      <c r="AF35" t="inlineStr"/>
+      <c r="AG35" t="inlineStr"/>
+      <c r="AH35" t="inlineStr"/>
+      <c r="AI35" t="inlineStr"/>
+      <c r="AJ35" t="inlineStr"/>
+      <c r="AK35" t="inlineStr"/>
+      <c r="AL35" t="inlineStr"/>
+      <c r="AM35" t="inlineStr"/>
+      <c r="AN35" t="inlineStr"/>
+      <c r="AO35" t="inlineStr"/>
+      <c r="AP35" t="inlineStr"/>
+      <c r="AQ35" t="inlineStr"/>
+      <c r="AR35" t="inlineStr"/>
+      <c r="AS35" t="inlineStr"/>
+      <c r="AT35" t="inlineStr"/>
+      <c r="AU35" t="inlineStr"/>
+      <c r="AV35" t="inlineStr"/>
+      <c r="AW35" t="inlineStr"/>
+      <c r="AX35" t="inlineStr"/>
+      <c r="AY35" t="inlineStr"/>
+      <c r="AZ35" t="inlineStr"/>
+      <c r="BA35" t="inlineStr"/>
+      <c r="BB35" t="inlineStr"/>
+      <c r="BC35" t="inlineStr"/>
+      <c r="BD35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Jong Gent</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Lierse K.</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Belçika Challenger Pro Lig</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>3252207</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2.13</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>3.06</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>2.28</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr"/>
+      <c r="W36" t="inlineStr"/>
+      <c r="X36" t="inlineStr"/>
+      <c r="Y36" t="inlineStr"/>
+      <c r="Z36" t="inlineStr"/>
+      <c r="AA36" t="inlineStr"/>
+      <c r="AB36" t="inlineStr"/>
+      <c r="AC36" t="inlineStr"/>
+      <c r="AD36" t="inlineStr"/>
+      <c r="AE36" t="inlineStr"/>
+      <c r="AF36" t="inlineStr"/>
+      <c r="AG36" t="inlineStr"/>
+      <c r="AH36" t="inlineStr"/>
+      <c r="AI36" t="inlineStr"/>
+      <c r="AJ36" t="inlineStr"/>
+      <c r="AK36" t="inlineStr"/>
+      <c r="AL36" t="inlineStr"/>
+      <c r="AM36" t="inlineStr"/>
+      <c r="AN36" t="inlineStr"/>
+      <c r="AO36" t="inlineStr"/>
+      <c r="AP36" t="inlineStr"/>
+      <c r="AQ36" t="inlineStr"/>
+      <c r="AR36" t="inlineStr"/>
+      <c r="AS36" t="inlineStr"/>
+      <c r="AT36" t="inlineStr"/>
+      <c r="AU36" t="inlineStr"/>
+      <c r="AV36" t="inlineStr"/>
+      <c r="AW36" t="inlineStr"/>
+      <c r="AX36" t="inlineStr"/>
+      <c r="AY36" t="inlineStr"/>
+      <c r="AZ36" t="inlineStr"/>
+      <c r="BA36" t="inlineStr"/>
+      <c r="BB36" t="inlineStr"/>
+      <c r="BC36" t="inlineStr"/>
+      <c r="BD36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>RFC Seraing</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Liege</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Belçika Challenger Pro Lig</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>3252169</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2.00</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>3.04</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>2.46</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr"/>
+      <c r="W37" t="inlineStr"/>
+      <c r="X37" t="inlineStr"/>
+      <c r="Y37" t="inlineStr"/>
+      <c r="Z37" t="inlineStr"/>
+      <c r="AA37" t="inlineStr"/>
+      <c r="AB37" t="inlineStr"/>
+      <c r="AC37" t="inlineStr"/>
+      <c r="AD37" t="inlineStr"/>
+      <c r="AE37" t="inlineStr"/>
+      <c r="AF37" t="inlineStr"/>
+      <c r="AG37" t="inlineStr"/>
+      <c r="AH37" t="inlineStr"/>
+      <c r="AI37" t="inlineStr"/>
+      <c r="AJ37" t="inlineStr"/>
+      <c r="AK37" t="inlineStr"/>
+      <c r="AL37" t="inlineStr"/>
+      <c r="AM37" t="inlineStr"/>
+      <c r="AN37" t="inlineStr"/>
+      <c r="AO37" t="inlineStr"/>
+      <c r="AP37" t="inlineStr"/>
+      <c r="AQ37" t="inlineStr"/>
+      <c r="AR37" t="inlineStr"/>
+      <c r="AS37" t="inlineStr"/>
+      <c r="AT37" t="inlineStr"/>
+      <c r="AU37" t="inlineStr"/>
+      <c r="AV37" t="inlineStr"/>
+      <c r="AW37" t="inlineStr"/>
+      <c r="AX37" t="inlineStr"/>
+      <c r="AY37" t="inlineStr"/>
+      <c r="AZ37" t="inlineStr"/>
+      <c r="BA37" t="inlineStr"/>
+      <c r="BB37" t="inlineStr"/>
+      <c r="BC37" t="inlineStr"/>
+      <c r="BD37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Slaven</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Istra</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Hırvatistan 1. HNL</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>3253915</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>1.88</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>3.15</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>2.59</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="inlineStr"/>
+      <c r="V38" t="inlineStr"/>
+      <c r="W38" t="inlineStr"/>
+      <c r="X38" t="inlineStr"/>
+      <c r="Y38" t="inlineStr"/>
+      <c r="Z38" t="inlineStr"/>
+      <c r="AA38" t="inlineStr"/>
+      <c r="AB38" t="inlineStr"/>
+      <c r="AC38" t="inlineStr"/>
+      <c r="AD38" t="inlineStr"/>
+      <c r="AE38" t="inlineStr"/>
+      <c r="AF38" t="inlineStr"/>
+      <c r="AG38" t="inlineStr"/>
+      <c r="AH38" t="inlineStr"/>
+      <c r="AI38" t="inlineStr"/>
+      <c r="AJ38" t="inlineStr"/>
+      <c r="AK38" t="inlineStr"/>
+      <c r="AL38" t="inlineStr"/>
+      <c r="AM38" t="inlineStr"/>
+      <c r="AN38" t="inlineStr"/>
+      <c r="AO38" t="inlineStr"/>
+      <c r="AP38" t="inlineStr"/>
+      <c r="AQ38" t="inlineStr"/>
+      <c r="AR38" t="inlineStr"/>
+      <c r="AS38" t="inlineStr"/>
+      <c r="AT38" t="inlineStr"/>
+      <c r="AU38" t="inlineStr"/>
+      <c r="AV38" t="inlineStr"/>
+      <c r="AW38" t="inlineStr"/>
+      <c r="AX38" t="inlineStr"/>
+      <c r="AY38" t="inlineStr"/>
+      <c r="AZ38" t="inlineStr"/>
+      <c r="BA38" t="inlineStr"/>
+      <c r="BB38" t="inlineStr"/>
+      <c r="BC38" t="inlineStr"/>
+      <c r="BD38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Newport</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Chesterfield</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>İngiltere 2. Lig</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>3253950</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>3.07</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>3.01</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>1.74</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="inlineStr"/>
+      <c r="V39" t="inlineStr"/>
+      <c r="W39" t="inlineStr"/>
+      <c r="X39" t="inlineStr"/>
+      <c r="Y39" t="inlineStr"/>
+      <c r="Z39" t="inlineStr"/>
+      <c r="AA39" t="inlineStr"/>
+      <c r="AB39" t="inlineStr"/>
+      <c r="AC39" t="inlineStr"/>
+      <c r="AD39" t="inlineStr"/>
+      <c r="AE39" t="inlineStr"/>
+      <c r="AF39" t="inlineStr"/>
+      <c r="AG39" t="inlineStr"/>
+      <c r="AH39" t="inlineStr"/>
+      <c r="AI39" t="inlineStr"/>
+      <c r="AJ39" t="inlineStr"/>
+      <c r="AK39" t="inlineStr"/>
+      <c r="AL39" t="inlineStr"/>
+      <c r="AM39" t="inlineStr"/>
+      <c r="AN39" t="inlineStr"/>
+      <c r="AO39" t="inlineStr"/>
+      <c r="AP39" t="inlineStr"/>
+      <c r="AQ39" t="inlineStr"/>
+      <c r="AR39" t="inlineStr"/>
+      <c r="AS39" t="inlineStr"/>
+      <c r="AT39" t="inlineStr"/>
+      <c r="AU39" t="inlineStr"/>
+      <c r="AV39" t="inlineStr"/>
+      <c r="AW39" t="inlineStr"/>
+      <c r="AX39" t="inlineStr"/>
+      <c r="AY39" t="inlineStr"/>
+      <c r="AZ39" t="inlineStr"/>
+      <c r="BA39" t="inlineStr"/>
+      <c r="BB39" t="inlineStr"/>
+      <c r="BC39" t="inlineStr"/>
+      <c r="BD39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Stenhousemuir</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Livingston</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>İskoçya Championship</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>3255271</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>3.51</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>3.27</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>1.55</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr"/>
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr"/>
+      <c r="W40" t="inlineStr"/>
+      <c r="X40" t="inlineStr"/>
+      <c r="Y40" t="inlineStr"/>
+      <c r="Z40" t="inlineStr"/>
+      <c r="AA40" t="inlineStr"/>
+      <c r="AB40" t="inlineStr"/>
+      <c r="AC40" t="inlineStr"/>
+      <c r="AD40" t="inlineStr"/>
+      <c r="AE40" t="inlineStr"/>
+      <c r="AF40" t="inlineStr"/>
+      <c r="AG40" t="inlineStr"/>
+      <c r="AH40" t="inlineStr"/>
+      <c r="AI40" t="inlineStr"/>
+      <c r="AJ40" t="inlineStr"/>
+      <c r="AK40" t="inlineStr"/>
+      <c r="AL40" t="inlineStr"/>
+      <c r="AM40" t="inlineStr"/>
+      <c r="AN40" t="inlineStr"/>
+      <c r="AO40" t="inlineStr"/>
+      <c r="AP40" t="inlineStr"/>
+      <c r="AQ40" t="inlineStr"/>
+      <c r="AR40" t="inlineStr"/>
+      <c r="AS40" t="inlineStr"/>
+      <c r="AT40" t="inlineStr"/>
+      <c r="AU40" t="inlineStr"/>
+      <c r="AV40" t="inlineStr"/>
+      <c r="AW40" t="inlineStr"/>
+      <c r="AX40" t="inlineStr"/>
+      <c r="AY40" t="inlineStr"/>
+      <c r="AZ40" t="inlineStr"/>
+      <c r="BA40" t="inlineStr"/>
+      <c r="BB40" t="inlineStr"/>
+      <c r="BC40" t="inlineStr"/>
+      <c r="BD40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Marsilya (K)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Nantes (K)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>23:00</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Fransa 1. Lig Kadınlar</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>3253964</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>1.45</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>3.46</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>3.95</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
+      <c r="T41" t="inlineStr"/>
+      <c r="U41" t="inlineStr"/>
+      <c r="V41" t="inlineStr"/>
+      <c r="W41" t="inlineStr"/>
+      <c r="X41" t="inlineStr"/>
+      <c r="Y41" t="inlineStr"/>
+      <c r="Z41" t="inlineStr"/>
+      <c r="AA41" t="inlineStr"/>
+      <c r="AB41" t="inlineStr"/>
+      <c r="AC41" t="inlineStr"/>
+      <c r="AD41" t="inlineStr"/>
+      <c r="AE41" t="inlineStr"/>
+      <c r="AF41" t="inlineStr"/>
+      <c r="AG41" t="inlineStr"/>
+      <c r="AH41" t="inlineStr"/>
+      <c r="AI41" t="inlineStr"/>
+      <c r="AJ41" t="inlineStr"/>
+      <c r="AK41" t="inlineStr"/>
+      <c r="AL41" t="inlineStr"/>
+      <c r="AM41" t="inlineStr"/>
+      <c r="AN41" t="inlineStr"/>
+      <c r="AO41" t="inlineStr"/>
+      <c r="AP41" t="inlineStr"/>
+      <c r="AQ41" t="inlineStr"/>
+      <c r="AR41" t="inlineStr"/>
+      <c r="AS41" t="inlineStr"/>
+      <c r="AT41" t="inlineStr"/>
+      <c r="AU41" t="inlineStr"/>
+      <c r="AV41" t="inlineStr"/>
+      <c r="AW41" t="inlineStr"/>
+      <c r="AX41" t="inlineStr"/>
+      <c r="AY41" t="inlineStr"/>
+      <c r="AZ41" t="inlineStr"/>
+      <c r="BA41" t="inlineStr"/>
+      <c r="BB41" t="inlineStr"/>
+      <c r="BC41" t="inlineStr"/>
+      <c r="BD41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Veles Moskova</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Spartak Ks</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Rusya FNL</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>3252523</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2.82</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>2.08</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
+      <c r="T42" t="inlineStr"/>
+      <c r="U42" t="inlineStr"/>
+      <c r="V42" t="inlineStr"/>
+      <c r="W42" t="inlineStr"/>
+      <c r="X42" t="inlineStr"/>
+      <c r="Y42" t="inlineStr"/>
+      <c r="Z42" t="inlineStr"/>
+      <c r="AA42" t="inlineStr"/>
+      <c r="AB42" t="inlineStr"/>
+      <c r="AC42" t="inlineStr"/>
+      <c r="AD42" t="inlineStr"/>
+      <c r="AE42" t="inlineStr"/>
+      <c r="AF42" t="inlineStr"/>
+      <c r="AG42" t="inlineStr"/>
+      <c r="AH42" t="inlineStr"/>
+      <c r="AI42" t="inlineStr"/>
+      <c r="AJ42" t="inlineStr"/>
+      <c r="AK42" t="inlineStr"/>
+      <c r="AL42" t="inlineStr"/>
+      <c r="AM42" t="inlineStr"/>
+      <c r="AN42" t="inlineStr"/>
+      <c r="AO42" t="inlineStr"/>
+      <c r="AP42" t="inlineStr"/>
+      <c r="AQ42" t="inlineStr"/>
+      <c r="AR42" t="inlineStr"/>
+      <c r="AS42" t="inlineStr"/>
+      <c r="AT42" t="inlineStr"/>
+      <c r="AU42" t="inlineStr"/>
+      <c r="AV42" t="inlineStr"/>
+      <c r="AW42" t="inlineStr"/>
+      <c r="AX42" t="inlineStr"/>
+      <c r="AY42" t="inlineStr"/>
+      <c r="AZ42" t="inlineStr"/>
+      <c r="BA42" t="inlineStr"/>
+      <c r="BB42" t="inlineStr"/>
+      <c r="BC42" t="inlineStr"/>
+      <c r="BD42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Nizhny Nov.</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Arsenal Tula</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Rusya FNL</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>3252368</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>1.27</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>3.89</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>5.41</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
+      <c r="T43" t="inlineStr"/>
+      <c r="U43" t="inlineStr"/>
+      <c r="V43" t="inlineStr"/>
+      <c r="W43" t="inlineStr"/>
+      <c r="X43" t="inlineStr"/>
+      <c r="Y43" t="inlineStr"/>
+      <c r="Z43" t="inlineStr"/>
+      <c r="AA43" t="inlineStr"/>
+      <c r="AB43" t="inlineStr"/>
+      <c r="AC43" t="inlineStr"/>
+      <c r="AD43" t="inlineStr"/>
+      <c r="AE43" t="inlineStr"/>
+      <c r="AF43" t="inlineStr"/>
+      <c r="AG43" t="inlineStr"/>
+      <c r="AH43" t="inlineStr"/>
+      <c r="AI43" t="inlineStr"/>
+      <c r="AJ43" t="inlineStr"/>
+      <c r="AK43" t="inlineStr"/>
+      <c r="AL43" t="inlineStr"/>
+      <c r="AM43" t="inlineStr"/>
+      <c r="AN43" t="inlineStr"/>
+      <c r="AO43" t="inlineStr"/>
+      <c r="AP43" t="inlineStr"/>
+      <c r="AQ43" t="inlineStr"/>
+      <c r="AR43" t="inlineStr"/>
+      <c r="AS43" t="inlineStr"/>
+      <c r="AT43" t="inlineStr"/>
+      <c r="AU43" t="inlineStr"/>
+      <c r="AV43" t="inlineStr"/>
+      <c r="AW43" t="inlineStr"/>
+      <c r="AX43" t="inlineStr"/>
+      <c r="AY43" t="inlineStr"/>
+      <c r="AZ43" t="inlineStr"/>
+      <c r="BA43" t="inlineStr"/>
+      <c r="BB43" t="inlineStr"/>
+      <c r="BC43" t="inlineStr"/>
+      <c r="BD43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Pogon GM</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Stal Mielec</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Polonya 1. Lig</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>3253368</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>1.82</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>3.16</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>2.71</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr"/>
+      <c r="T44" t="inlineStr"/>
+      <c r="U44" t="inlineStr"/>
+      <c r="V44" t="inlineStr"/>
+      <c r="W44" t="inlineStr"/>
+      <c r="X44" t="inlineStr"/>
+      <c r="Y44" t="inlineStr"/>
+      <c r="Z44" t="inlineStr"/>
+      <c r="AA44" t="inlineStr"/>
+      <c r="AB44" t="inlineStr"/>
+      <c r="AC44" t="inlineStr"/>
+      <c r="AD44" t="inlineStr"/>
+      <c r="AE44" t="inlineStr"/>
+      <c r="AF44" t="inlineStr"/>
+      <c r="AG44" t="inlineStr"/>
+      <c r="AH44" t="inlineStr"/>
+      <c r="AI44" t="inlineStr"/>
+      <c r="AJ44" t="inlineStr"/>
+      <c r="AK44" t="inlineStr"/>
+      <c r="AL44" t="inlineStr"/>
+      <c r="AM44" t="inlineStr"/>
+      <c r="AN44" t="inlineStr"/>
+      <c r="AO44" t="inlineStr"/>
+      <c r="AP44" t="inlineStr"/>
+      <c r="AQ44" t="inlineStr"/>
+      <c r="AR44" t="inlineStr"/>
+      <c r="AS44" t="inlineStr"/>
+      <c r="AT44" t="inlineStr"/>
+      <c r="AU44" t="inlineStr"/>
+      <c r="AV44" t="inlineStr"/>
+      <c r="AW44" t="inlineStr"/>
+      <c r="AX44" t="inlineStr"/>
+      <c r="AY44" t="inlineStr"/>
+      <c r="AZ44" t="inlineStr"/>
+      <c r="BA44" t="inlineStr"/>
+      <c r="BB44" t="inlineStr"/>
+      <c r="BC44" t="inlineStr"/>
+      <c r="BD44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Sandecja</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Olim. Grudziadz</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Polonya 2. Lig</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>3255503</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>1.76</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>3.16</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>2.87</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
+      <c r="T45" t="inlineStr"/>
+      <c r="U45" t="inlineStr"/>
+      <c r="V45" t="inlineStr"/>
+      <c r="W45" t="inlineStr"/>
+      <c r="X45" t="inlineStr"/>
+      <c r="Y45" t="inlineStr"/>
+      <c r="Z45" t="inlineStr"/>
+      <c r="AA45" t="inlineStr"/>
+      <c r="AB45" t="inlineStr"/>
+      <c r="AC45" t="inlineStr"/>
+      <c r="AD45" t="inlineStr"/>
+      <c r="AE45" t="inlineStr"/>
+      <c r="AF45" t="inlineStr"/>
+      <c r="AG45" t="inlineStr"/>
+      <c r="AH45" t="inlineStr"/>
+      <c r="AI45" t="inlineStr"/>
+      <c r="AJ45" t="inlineStr"/>
+      <c r="AK45" t="inlineStr"/>
+      <c r="AL45" t="inlineStr"/>
+      <c r="AM45" t="inlineStr"/>
+      <c r="AN45" t="inlineStr"/>
+      <c r="AO45" t="inlineStr"/>
+      <c r="AP45" t="inlineStr"/>
+      <c r="AQ45" t="inlineStr"/>
+      <c r="AR45" t="inlineStr"/>
+      <c r="AS45" t="inlineStr"/>
+      <c r="AT45" t="inlineStr"/>
+      <c r="AU45" t="inlineStr"/>
+      <c r="AV45" t="inlineStr"/>
+      <c r="AW45" t="inlineStr"/>
+      <c r="AX45" t="inlineStr"/>
+      <c r="AY45" t="inlineStr"/>
+      <c r="AZ45" t="inlineStr"/>
+      <c r="BA45" t="inlineStr"/>
+      <c r="BB45" t="inlineStr"/>
+      <c r="BC45" t="inlineStr"/>
+      <c r="BD45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Hellerup IK</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Nykobing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Danimarka 2. Lig</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>3252171</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>4.52</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>3.93</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="inlineStr"/>
+      <c r="U46" t="inlineStr"/>
+      <c r="V46" t="inlineStr"/>
+      <c r="W46" t="inlineStr"/>
+      <c r="X46" t="inlineStr"/>
+      <c r="Y46" t="inlineStr"/>
+      <c r="Z46" t="inlineStr"/>
+      <c r="AA46" t="inlineStr"/>
+      <c r="AB46" t="inlineStr"/>
+      <c r="AC46" t="inlineStr"/>
+      <c r="AD46" t="inlineStr"/>
+      <c r="AE46" t="inlineStr"/>
+      <c r="AF46" t="inlineStr"/>
+      <c r="AG46" t="inlineStr"/>
+      <c r="AH46" t="inlineStr"/>
+      <c r="AI46" t="inlineStr"/>
+      <c r="AJ46" t="inlineStr"/>
+      <c r="AK46" t="inlineStr"/>
+      <c r="AL46" t="inlineStr"/>
+      <c r="AM46" t="inlineStr"/>
+      <c r="AN46" t="inlineStr"/>
+      <c r="AO46" t="inlineStr"/>
+      <c r="AP46" t="inlineStr"/>
+      <c r="AQ46" t="inlineStr"/>
+      <c r="AR46" t="inlineStr"/>
+      <c r="AS46" t="inlineStr"/>
+      <c r="AT46" t="inlineStr"/>
+      <c r="AU46" t="inlineStr"/>
+      <c r="AV46" t="inlineStr"/>
+      <c r="AW46" t="inlineStr"/>
+      <c r="AX46" t="inlineStr"/>
+      <c r="AY46" t="inlineStr"/>
+      <c r="AZ46" t="inlineStr"/>
+      <c r="BA46" t="inlineStr"/>
+      <c r="BB46" t="inlineStr"/>
+      <c r="BC46" t="inlineStr"/>
+      <c r="BD46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Skive</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>VSK Aarhus</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>30.10.2026</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Danimarka 2. Lig</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>3252510</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>2.09</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>3.04</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>2.35</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
+      <c r="T47" t="inlineStr"/>
+      <c r="U47" t="inlineStr"/>
+      <c r="V47" t="inlineStr"/>
+      <c r="W47" t="inlineStr"/>
+      <c r="X47" t="inlineStr"/>
+      <c r="Y47" t="inlineStr"/>
+      <c r="Z47" t="inlineStr"/>
+      <c r="AA47" t="inlineStr"/>
+      <c r="AB47" t="inlineStr"/>
+      <c r="AC47" t="inlineStr"/>
+      <c r="AD47" t="inlineStr"/>
+      <c r="AE47" t="inlineStr"/>
+      <c r="AF47" t="inlineStr"/>
+      <c r="AG47" t="inlineStr"/>
+      <c r="AH47" t="inlineStr"/>
+      <c r="AI47" t="inlineStr"/>
+      <c r="AJ47" t="inlineStr"/>
+      <c r="AK47" t="inlineStr"/>
+      <c r="AL47" t="inlineStr"/>
+      <c r="AM47" t="inlineStr"/>
+      <c r="AN47" t="inlineStr"/>
+      <c r="AO47" t="inlineStr"/>
+      <c r="AP47" t="inlineStr"/>
+      <c r="AQ47" t="inlineStr"/>
+      <c r="AR47" t="inlineStr"/>
+      <c r="AS47" t="inlineStr"/>
+      <c r="AT47" t="inlineStr"/>
+      <c r="AU47" t="inlineStr"/>
+      <c r="AV47" t="inlineStr"/>
+      <c r="AW47" t="inlineStr"/>
+      <c r="AX47" t="inlineStr"/>
+      <c r="AY47" t="inlineStr"/>
+      <c r="AZ47" t="inlineStr"/>
+      <c r="BA47" t="inlineStr"/>
+      <c r="BB47" t="inlineStr"/>
+      <c r="BC47" t="inlineStr"/>
+      <c r="BD47" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>